<commit_message>
feat(thd): apply BA answers — critical complaints per PPL, CC = Tech Executive L1
- Critical complaints match on PPL + Complaint Code only (BA: mapped per PPL as
  in the CRM complaint master). A row without a PPL never raises a case and is
  listed as pending; the BA's E32 row has no PPL yet.
- Rule 8: 'Tech Executive/CC' — CC is the Command Centre, handled as Tech
  Executive L1.
- THD Rule Tester counts the unmapped critical complaints as pending and
  explains why a code does not fire for the chosen PPL.
- docs/THD_MASTERS.md records each BA answer and what is still open.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DwiSAaMRyjNA589tWt8iz
</commit_message>
<xml_diff>
--- a/docs/templates/TML_Existing_Masters_Catalogue.xlsx
+++ b/docs/templates/TML_Existing_Masters_Catalogue.xlsx
@@ -3098,7 +3098,7 @@
         <v>THD Rules</v>
       </c>
       <c r="G43" t="str">
-        <v>Complaint codes that automatically raise a THD case when added to a Job Card. Blank PPL = every PPL.</v>
+        <v>Complaint codes that automatically raise a THD case when added to a Job Card, mapped per PPL as in the CRM complaint master. A row without a PPL does not raise a case until its PPL is filled.</v>
       </c>
     </row>
     <row r="44">
@@ -19368,7 +19368,7 @@
         <v/>
       </c>
       <c r="Q259" t="str">
-        <v>Leave blank to apply to all PPLs.</v>
+        <v>One row per PPL + Complaint Code, as in the CRM complaint master. Needed to raise a case; a row without a PPL is listed as pending.</v>
       </c>
     </row>
     <row r="260">
@@ -24481,7 +24481,7 @@
         <v>THD_UNATTENDED</v>
       </c>
       <c r="D9" t="str">
-        <v>A THD case stays unattended by DET for more than 24 hours from creation; an auto request goes to Tech Executive L1.</v>
+        <v>A THD case stays unattended by DET for more than 24 hours from creation; an auto request goes to Tech Executive L1 (Excel "Tech Executive/CC"; CC = Command Centre, handled as Tech Executive L1).</v>
       </c>
       <c r="E9" t="str">
         <v>THD Age</v>

</xml_diff>

<commit_message>
feat(claims): apply BA answers — SHQ Lead 1 approves above Rs 20,000
- Approval matrix: Claim Manager approves up to and including Rs 20,000;
  above that the request goes via CCM/ACCM to SHQ Lead 1, who approves with no
  upper limit. New 'Can Approve' column; limits are inclusive; a blank limit
  on an approver means no upper limit.
- Reminders after 24 h are a notification and an email only (no
  auto-escalation), recorded per level.
- Special Goodwill Claim (IUPR, Thrive) is an identification tag only.
- New checks: a non-approver has no limit and must forward; an approver with a
  limit must name who handles larger amounts; levels after an unlimited
  approver are flagged as unreachable.
- docs/CLAIM_MASTERS.md records each BA answer and what is still open.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DwiSAaMRyjNA589tWt8iz
</commit_message>
<xml_diff>
--- a/docs/templates/TML_Existing_Masters_Catalogue.xlsx
+++ b/docs/templates/TML_Existing_Masters_Catalogue.xlsx
@@ -2822,7 +2822,7 @@
         <v>Claim Dropdown Lists</v>
       </c>
       <c r="G31" t="str">
-        <v>Selected by the Claim Manager for special claim approvals (BA sheet "Special claim"). Only Active values are shown, in Order.</v>
+        <v>Identification tag on a Goodwill Authorization Request (does not change the approval path) (BA sheet "Special claim"). Only Active values are shown, in Order.</v>
       </c>
     </row>
     <row r="32">
@@ -2899,7 +2899,7 @@
         <v>claim_warranty_approval_matrix</v>
       </c>
       <c r="B35" t="str">
-        <v>Warranty Authorization Approval Matrix</v>
+        <v>AMC / Warranty Authorization Approval Matrix</v>
       </c>
       <c r="C35" t="str">
         <v>claim</v>
@@ -2914,7 +2914,7 @@
         <v>Claim Rules</v>
       </c>
       <c r="G35" t="str">
-        <v>Who can approve a Warranty Authorization Request, by Level (BA sheet "Warranty Approval Matrix"). A level approves amounts below its "Approves Below (₹)"; blank = cannot approve and must forward. A reminder goes out after the Reminder hours.</v>
+        <v>Who approves an Authorization Request, level by level (BA sheet "Warranty Approval Matrix" and BA answers). A level with Can Approve = Y approves amounts up to and including its limit; a blank limit means no upper limit. Otherwise the request moves to the next level. After the Reminder hours the pending approver gets a notification and an email only; nothing is escalated automatically.</v>
       </c>
     </row>
     <row r="36">
@@ -5642,7 +5642,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q326"/>
+  <dimension ref="A1:Q328"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -16885,25 +16885,25 @@
         <v>claim_warranty_approval_matrix</v>
       </c>
       <c r="B213" t="str">
-        <v>approvesBelow</v>
+        <v>canApprove</v>
       </c>
       <c r="C213" t="str">
-        <v>Approves Below (₹)</v>
+        <v>Can Approve</v>
       </c>
       <c r="D213" t="str">
-        <v>number</v>
+        <v>select</v>
       </c>
       <c r="E213" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F213" t="str">
-        <v/>
-      </c>
-      <c r="G213">
-        <v>1</v>
-      </c>
-      <c r="H213">
-        <v>100000000</v>
+        <v>Y, N</v>
+      </c>
+      <c r="G213" t="str">
+        <v/>
+      </c>
+      <c r="H213" t="str">
+        <v/>
       </c>
       <c r="I213" t="str">
         <v/>
@@ -16930,7 +16930,7 @@
         <v/>
       </c>
       <c r="Q213" t="str">
-        <v>Blank = this persona cannot approve.</v>
+        <v/>
       </c>
     </row>
     <row r="214">
@@ -16938,25 +16938,25 @@
         <v>claim_warranty_approval_matrix</v>
       </c>
       <c r="B214" t="str">
-        <v>actions</v>
+        <v>approvesUpTo</v>
       </c>
       <c r="C214" t="str">
-        <v>Action / Authority</v>
+        <v>Approves Up To (₹)</v>
       </c>
       <c r="D214" t="str">
-        <v>text</v>
+        <v>number</v>
       </c>
       <c r="E214" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F214" t="str">
         <v/>
       </c>
-      <c r="G214" t="str">
-        <v/>
-      </c>
-      <c r="H214" t="str">
-        <v/>
+      <c r="G214">
+        <v>1</v>
+      </c>
+      <c r="H214">
+        <v>100000000</v>
       </c>
       <c r="I214" t="str">
         <v/>
@@ -16983,7 +16983,7 @@
         <v/>
       </c>
       <c r="Q214" t="str">
-        <v>Comma-separated actions available to this persona.</v>
+        <v>Inclusive. Blank with Can Approve = Y means no upper limit.</v>
       </c>
     </row>
     <row r="215">
@@ -16991,16 +16991,16 @@
         <v>claim_warranty_approval_matrix</v>
       </c>
       <c r="B215" t="str">
-        <v>forwardTo</v>
+        <v>actions</v>
       </c>
       <c r="C215" t="str">
-        <v>Forwards To</v>
+        <v>Action / Authority</v>
       </c>
       <c r="D215" t="str">
         <v>text</v>
       </c>
       <c r="E215" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F215" t="str">
         <v/>
@@ -17036,7 +17036,7 @@
         <v/>
       </c>
       <c r="Q215" t="str">
-        <v>Persona of the next level, when the amount is above this level.</v>
+        <v>Comma-separated actions available to this persona.</v>
       </c>
     </row>
     <row r="216">
@@ -17044,25 +17044,25 @@
         <v>claim_warranty_approval_matrix</v>
       </c>
       <c r="B216" t="str">
-        <v>reminderHours</v>
+        <v>forwardTo</v>
       </c>
       <c r="C216" t="str">
-        <v>Reminder (Hrs)</v>
+        <v>Forwards To</v>
       </c>
       <c r="D216" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E216" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F216" t="str">
         <v/>
       </c>
-      <c r="G216">
-        <v>1</v>
-      </c>
-      <c r="H216">
-        <v>720</v>
+      <c r="G216" t="str">
+        <v/>
+      </c>
+      <c r="H216" t="str">
+        <v/>
       </c>
       <c r="I216" t="str">
         <v/>
@@ -17089,7 +17089,7 @@
         <v/>
       </c>
       <c r="Q216" t="str">
-        <v/>
+        <v>Persona of the next level, for amounts this level cannot approve.</v>
       </c>
     </row>
     <row r="217">
@@ -17097,25 +17097,25 @@
         <v>claim_warranty_approval_matrix</v>
       </c>
       <c r="B217" t="str">
-        <v>status</v>
+        <v>reminderHours</v>
       </c>
       <c r="C217" t="str">
-        <v>Status</v>
+        <v>Reminder (Hrs)</v>
       </c>
       <c r="D217" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E217" t="str">
         <v>Y</v>
       </c>
       <c r="F217" t="str">
-        <v>Active, Inactive</v>
-      </c>
-      <c r="G217" t="str">
-        <v/>
-      </c>
-      <c r="H217" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G217">
+        <v>1</v>
+      </c>
+      <c r="H217">
+        <v>720</v>
       </c>
       <c r="I217" t="str">
         <v/>
@@ -17147,13 +17147,13 @@
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>claim_service_guideline</v>
+        <v>claim_warranty_approval_matrix</v>
       </c>
       <c r="B218" t="str">
-        <v>requestType</v>
+        <v>reminderVia</v>
       </c>
       <c r="C218" t="str">
-        <v>Request Type</v>
+        <v>Reminder Via</v>
       </c>
       <c r="D218" t="str">
         <v>select</v>
@@ -17162,7 +17162,7 @@
         <v>Y</v>
       </c>
       <c r="F218" t="str">
-        <v>AMC, Extended Warranty</v>
+        <v>Notification + Email</v>
       </c>
       <c r="G218" t="str">
         <v/>
@@ -17200,13 +17200,13 @@
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>claim_service_guideline</v>
+        <v>claim_warranty_approval_matrix</v>
       </c>
       <c r="B219" t="str">
-        <v>bu</v>
+        <v>status</v>
       </c>
       <c r="C219" t="str">
-        <v>BU</v>
+        <v>Status</v>
       </c>
       <c r="D219" t="str">
         <v>select</v>
@@ -17215,7 +17215,7 @@
         <v>Y</v>
       </c>
       <c r="F219" t="str">
-        <v>PV, EV</v>
+        <v>Active, Inactive</v>
       </c>
       <c r="G219" t="str">
         <v/>
@@ -17256,19 +17256,19 @@
         <v>claim_service_guideline</v>
       </c>
       <c r="B220" t="str">
-        <v>fileName</v>
+        <v>requestType</v>
       </c>
       <c r="C220" t="str">
-        <v>Guideline File</v>
+        <v>Request Type</v>
       </c>
       <c r="D220" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E220" t="str">
         <v>Y</v>
       </c>
       <c r="F220" t="str">
-        <v/>
+        <v>AMC, Extended Warranty</v>
       </c>
       <c r="G220" t="str">
         <v/>
@@ -17301,7 +17301,7 @@
         <v/>
       </c>
       <c r="Q220" t="str">
-        <v>File name or link of the PDF.</v>
+        <v/>
       </c>
     </row>
     <row r="221">
@@ -17309,19 +17309,19 @@
         <v>claim_service_guideline</v>
       </c>
       <c r="B221" t="str">
-        <v>version</v>
+        <v>bu</v>
       </c>
       <c r="C221" t="str">
-        <v>Version</v>
+        <v>BU</v>
       </c>
       <c r="D221" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E221" t="str">
         <v>Y</v>
       </c>
       <c r="F221" t="str">
-        <v/>
+        <v>PV, EV</v>
       </c>
       <c r="G221" t="str">
         <v/>
@@ -17362,13 +17362,13 @@
         <v>claim_service_guideline</v>
       </c>
       <c r="B222" t="str">
-        <v>effectiveFrom</v>
+        <v>fileName</v>
       </c>
       <c r="C222" t="str">
-        <v>Effective From</v>
+        <v>Guideline File</v>
       </c>
       <c r="D222" t="str">
-        <v>date</v>
+        <v>text</v>
       </c>
       <c r="E222" t="str">
         <v>Y</v>
@@ -17407,7 +17407,7 @@
         <v/>
       </c>
       <c r="Q222" t="str">
-        <v/>
+        <v>File name or link of the PDF.</v>
       </c>
     </row>
     <row r="223">
@@ -17415,19 +17415,19 @@
         <v>claim_service_guideline</v>
       </c>
       <c r="B223" t="str">
-        <v>status</v>
+        <v>version</v>
       </c>
       <c r="C223" t="str">
-        <v>Status</v>
+        <v>Version</v>
       </c>
       <c r="D223" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E223" t="str">
         <v>Y</v>
       </c>
       <c r="F223" t="str">
-        <v>Active, Inactive</v>
+        <v/>
       </c>
       <c r="G223" t="str">
         <v/>
@@ -17465,22 +17465,22 @@
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>claim_shq_users</v>
+        <v>claim_service_guideline</v>
       </c>
       <c r="B224" t="str">
-        <v>bu</v>
+        <v>effectiveFrom</v>
       </c>
       <c r="C224" t="str">
-        <v>BU</v>
+        <v>Effective From</v>
       </c>
       <c r="D224" t="str">
-        <v>select</v>
+        <v>date</v>
       </c>
       <c r="E224" t="str">
         <v>Y</v>
       </c>
       <c r="F224" t="str">
-        <v>PV, EV</v>
+        <v/>
       </c>
       <c r="G224" t="str">
         <v/>
@@ -17518,22 +17518,22 @@
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v>claim_shq_users</v>
+        <v>claim_service_guideline</v>
       </c>
       <c r="B225" t="str">
-        <v>userName</v>
+        <v>status</v>
       </c>
       <c r="C225" t="str">
-        <v>User Name</v>
+        <v>Status</v>
       </c>
       <c r="D225" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E225" t="str">
         <v>Y</v>
       </c>
       <c r="F225" t="str">
-        <v/>
+        <v>Active, Inactive</v>
       </c>
       <c r="G225" t="str">
         <v/>
@@ -17574,19 +17574,19 @@
         <v>claim_shq_users</v>
       </c>
       <c r="B226" t="str">
-        <v>crmUserId</v>
+        <v>bu</v>
       </c>
       <c r="C226" t="str">
-        <v>CRM User ID</v>
+        <v>BU</v>
       </c>
       <c r="D226" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E226" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F226" t="str">
-        <v/>
+        <v>PV, EV</v>
       </c>
       <c r="G226" t="str">
         <v/>
@@ -17627,19 +17627,19 @@
         <v>claim_shq_users</v>
       </c>
       <c r="B227" t="str">
-        <v>status</v>
+        <v>userName</v>
       </c>
       <c r="C227" t="str">
-        <v>Status</v>
+        <v>User Name</v>
       </c>
       <c r="D227" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E227" t="str">
         <v>Y</v>
       </c>
       <c r="F227" t="str">
-        <v>Active, Inactive</v>
+        <v/>
       </c>
       <c r="G227" t="str">
         <v/>
@@ -17677,19 +17677,19 @@
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>spd_issuance_priority</v>
+        <v>claim_shq_users</v>
       </c>
       <c r="B228" t="str">
-        <v>priorityCode</v>
+        <v>crmUserId</v>
       </c>
       <c r="C228" t="str">
-        <v>Priority Code</v>
+        <v>CRM User ID</v>
       </c>
       <c r="D228" t="str">
         <v>text</v>
       </c>
       <c r="E228" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F228" t="str">
         <v/>
@@ -17730,22 +17730,22 @@
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v>spd_issuance_priority</v>
+        <v>claim_shq_users</v>
       </c>
       <c r="B229" t="str">
-        <v>priorityLevel</v>
+        <v>status</v>
       </c>
       <c r="C229" t="str">
-        <v>Priority Tag</v>
+        <v>Status</v>
       </c>
       <c r="D229" t="str">
         <v>select</v>
       </c>
       <c r="E229" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F229" t="str">
-        <v>Emergency VOR, Running Repair Express, Scheduled Periodic Maintenance, Recall Campaign</v>
+        <v>Active, Inactive</v>
       </c>
       <c r="G229" t="str">
         <v/>
@@ -17786,13 +17786,13 @@
         <v>spd_issuance_priority</v>
       </c>
       <c r="B230" t="str">
-        <v>slaMins</v>
+        <v>priorityCode</v>
       </c>
       <c r="C230" t="str">
-        <v>Picking SLA (Minutes)</v>
+        <v>Priority Code</v>
       </c>
       <c r="D230" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E230" t="str">
         <v>Y</v>
@@ -17839,10 +17839,10 @@
         <v>spd_issuance_priority</v>
       </c>
       <c r="B231" t="str">
-        <v>requireOtp</v>
+        <v>priorityLevel</v>
       </c>
       <c r="C231" t="str">
-        <v>Mechanic Fingerprint / OTP Verification</v>
+        <v>Priority Tag</v>
       </c>
       <c r="D231" t="str">
         <v>select</v>
@@ -17851,7 +17851,7 @@
         <v>N</v>
       </c>
       <c r="F231" t="str">
-        <v>Y, N</v>
+        <v>Emergency VOR, Running Repair Express, Scheduled Periodic Maintenance, Recall Campaign</v>
       </c>
       <c r="G231" t="str">
         <v/>
@@ -17892,19 +17892,19 @@
         <v>spd_issuance_priority</v>
       </c>
       <c r="B232" t="str">
-        <v>active</v>
+        <v>slaMins</v>
       </c>
       <c r="C232" t="str">
-        <v>Active</v>
+        <v>Picking SLA (Minutes)</v>
       </c>
       <c r="D232" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E232" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F232" t="str">
-        <v>Y, N</v>
+        <v/>
       </c>
       <c r="G232" t="str">
         <v/>
@@ -17942,22 +17942,22 @@
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>parts_delay_reasons</v>
+        <v>spd_issuance_priority</v>
       </c>
       <c r="B233" t="str">
-        <v>delayCode</v>
+        <v>requireOtp</v>
       </c>
       <c r="C233" t="str">
-        <v>Delay Code</v>
+        <v>Mechanic Fingerprint / OTP Verification</v>
       </c>
       <c r="D233" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E233" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F233" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G233" t="str">
         <v/>
@@ -17995,22 +17995,22 @@
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>parts_delay_reasons</v>
+        <v>spd_issuance_priority</v>
       </c>
       <c r="B234" t="str">
-        <v>reasonName</v>
+        <v>active</v>
       </c>
       <c r="C234" t="str">
-        <v>Non-Availability Root Cause</v>
+        <v>Active</v>
       </c>
       <c r="D234" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E234" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F234" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G234" t="str">
         <v/>
@@ -18051,19 +18051,19 @@
         <v>parts_delay_reasons</v>
       </c>
       <c r="B235" t="str">
-        <v>autoOrderSap</v>
+        <v>delayCode</v>
       </c>
       <c r="C235" t="str">
-        <v>Auto Trigger SAP Emergency Order</v>
+        <v>Delay Code</v>
       </c>
       <c r="D235" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E235" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F235" t="str">
-        <v>Y, N</v>
+        <v/>
       </c>
       <c r="G235" t="str">
         <v/>
@@ -18104,19 +18104,19 @@
         <v>parts_delay_reasons</v>
       </c>
       <c r="B236" t="str">
-        <v>smsCustomer</v>
+        <v>reasonName</v>
       </c>
       <c r="C236" t="str">
-        <v>Trigger Customer ETA SMS</v>
+        <v>Non-Availability Root Cause</v>
       </c>
       <c r="D236" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E236" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F236" t="str">
-        <v>Y, N</v>
+        <v/>
       </c>
       <c r="G236" t="str">
         <v/>
@@ -18157,10 +18157,10 @@
         <v>parts_delay_reasons</v>
       </c>
       <c r="B237" t="str">
-        <v>active</v>
+        <v>autoOrderSap</v>
       </c>
       <c r="C237" t="str">
-        <v>Active</v>
+        <v>Auto Trigger SAP Emergency Order</v>
       </c>
       <c r="D237" t="str">
         <v>select</v>
@@ -18207,22 +18207,22 @@
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>thd_escalation_categories</v>
+        <v>parts_delay_reasons</v>
       </c>
       <c r="B238" t="str">
-        <v>categoryCode</v>
+        <v>smsCustomer</v>
       </c>
       <c r="C238" t="str">
-        <v>Escalation Category</v>
+        <v>Trigger Customer ETA SMS</v>
       </c>
       <c r="D238" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E238" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F238" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G238" t="str">
         <v/>
@@ -18260,13 +18260,13 @@
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>thd_escalation_categories</v>
+        <v>parts_delay_reasons</v>
       </c>
       <c r="B239" t="str">
-        <v>systemDomain</v>
+        <v>active</v>
       </c>
       <c r="C239" t="str">
-        <v>Engineering System</v>
+        <v>Active</v>
       </c>
       <c r="D239" t="str">
         <v>select</v>
@@ -18275,7 +18275,7 @@
         <v>N</v>
       </c>
       <c r="F239" t="str">
-        <v>EV High Voltage Traction, DCA Dual Clutch Transmission, ADAS &amp; Radar Calibration, Braking &amp; ESP Hydraulics, CAN Bus Network Communication</v>
+        <v>Y, N</v>
       </c>
       <c r="G239" t="str">
         <v/>
@@ -18316,19 +18316,19 @@
         <v>thd_escalation_categories</v>
       </c>
       <c r="B240" t="str">
-        <v>severityTier</v>
+        <v>categoryCode</v>
       </c>
       <c r="C240" t="str">
-        <v>Plant Response SLA</v>
+        <v>Escalation Category</v>
       </c>
       <c r="D240" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E240" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F240" t="str">
-        <v>Tier 1 Critical (&lt; 4 Hours), Tier 2 High (&lt; 12 Hours), Tier 3 Standard (&lt; 24 Hours)</v>
+        <v/>
       </c>
       <c r="G240" t="str">
         <v/>
@@ -18369,10 +18369,10 @@
         <v>thd_escalation_categories</v>
       </c>
       <c r="B241" t="str">
-        <v>requiresPlantVisit</v>
+        <v>systemDomain</v>
       </c>
       <c r="C241" t="str">
-        <v>Plant Field Engineer Dispatch</v>
+        <v>Engineering System</v>
       </c>
       <c r="D241" t="str">
         <v>select</v>
@@ -18381,7 +18381,7 @@
         <v>N</v>
       </c>
       <c r="F241" t="str">
-        <v>Y, N</v>
+        <v>EV High Voltage Traction, DCA Dual Clutch Transmission, ADAS &amp; Radar Calibration, Braking &amp; ESP Hydraulics, CAN Bus Network Communication</v>
       </c>
       <c r="G241" t="str">
         <v/>
@@ -18422,10 +18422,10 @@
         <v>thd_escalation_categories</v>
       </c>
       <c r="B242" t="str">
-        <v>active</v>
+        <v>severityTier</v>
       </c>
       <c r="C242" t="str">
-        <v>Active</v>
+        <v>Plant Response SLA</v>
       </c>
       <c r="D242" t="str">
         <v>select</v>
@@ -18434,7 +18434,7 @@
         <v>N</v>
       </c>
       <c r="F242" t="str">
-        <v>Y, N</v>
+        <v>Tier 1 Critical (&lt; 4 Hours), Tier 2 High (&lt; 12 Hours), Tier 3 Standard (&lt; 24 Hours)</v>
       </c>
       <c r="G242" t="str">
         <v/>
@@ -18472,22 +18472,22 @@
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>tib_bulletin_codes</v>
+        <v>thd_escalation_categories</v>
       </c>
       <c r="B243" t="str">
-        <v>tibNumber</v>
+        <v>requiresPlantVisit</v>
       </c>
       <c r="C243" t="str">
-        <v>TIB Bulletin Reference</v>
+        <v>Plant Field Engineer Dispatch</v>
       </c>
       <c r="D243" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E243" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F243" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G243" t="str">
         <v/>
@@ -18525,22 +18525,22 @@
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>tib_bulletin_codes</v>
+        <v>thd_escalation_categories</v>
       </c>
       <c r="B244" t="str">
-        <v>title</v>
+        <v>active</v>
       </c>
       <c r="C244" t="str">
-        <v>Subject / Advisory Scope</v>
+        <v>Active</v>
       </c>
       <c r="D244" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E244" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F244" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G244" t="str">
         <v/>
@@ -18581,19 +18581,19 @@
         <v>tib_bulletin_codes</v>
       </c>
       <c r="B245" t="str">
-        <v>affectedPpl</v>
+        <v>tibNumber</v>
       </c>
       <c r="C245" t="str">
-        <v>Applicable Vehicle PPL</v>
+        <v>TIB Bulletin Reference</v>
       </c>
       <c r="D245" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E245" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F245" t="str">
-        <v>Nexon EV, Nexon ICE, Harrier / Safari, Curvv EV, Altroz</v>
+        <v/>
       </c>
       <c r="G245" t="str">
         <v/>
@@ -18634,19 +18634,19 @@
         <v>tib_bulletin_codes</v>
       </c>
       <c r="B246" t="str">
-        <v>reworkType</v>
+        <v>title</v>
       </c>
       <c r="C246" t="str">
-        <v>Rework Classification</v>
+        <v>Subject / Advisory Scope</v>
       </c>
       <c r="D246" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E246" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F246" t="str">
-        <v>ECU Firmware Update, Harness Rerouting, Hardware Bush Replacement, Torque Audit</v>
+        <v/>
       </c>
       <c r="G246" t="str">
         <v/>
@@ -18687,10 +18687,10 @@
         <v>tib_bulletin_codes</v>
       </c>
       <c r="B247" t="str">
-        <v>active</v>
+        <v>affectedPpl</v>
       </c>
       <c r="C247" t="str">
-        <v>Active</v>
+        <v>Applicable Vehicle PPL</v>
       </c>
       <c r="D247" t="str">
         <v>select</v>
@@ -18699,7 +18699,7 @@
         <v>N</v>
       </c>
       <c r="F247" t="str">
-        <v>Y, N</v>
+        <v>Nexon EV, Nexon ICE, Harrier / Safari, Curvv EV, Altroz</v>
       </c>
       <c r="G247" t="str">
         <v/>
@@ -18737,28 +18737,28 @@
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>thd_auto_trigger_rules</v>
+        <v>tib_bulletin_codes</v>
       </c>
       <c r="B248" t="str">
-        <v>ruleNo</v>
+        <v>reworkType</v>
       </c>
       <c r="C248" t="str">
-        <v>Rule No.</v>
+        <v>Rework Classification</v>
       </c>
       <c r="D248" t="str">
-        <v>number</v>
+        <v>select</v>
       </c>
       <c r="E248" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F248" t="str">
-        <v/>
-      </c>
-      <c r="G248">
-        <v>1</v>
-      </c>
-      <c r="H248">
-        <v>99</v>
+        <v>ECU Firmware Update, Harness Rerouting, Hardware Bush Replacement, Torque Audit</v>
+      </c>
+      <c r="G248" t="str">
+        <v/>
+      </c>
+      <c r="H248" t="str">
+        <v/>
       </c>
       <c r="I248" t="str">
         <v/>
@@ -18790,22 +18790,22 @@
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>thd_auto_trigger_rules</v>
+        <v>tib_bulletin_codes</v>
       </c>
       <c r="B249" t="str">
-        <v>scenarioCode</v>
+        <v>active</v>
       </c>
       <c r="C249" t="str">
-        <v>Scenario</v>
+        <v>Active</v>
       </c>
       <c r="D249" t="str">
         <v>select</v>
       </c>
       <c r="E249" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F249" t="str">
-        <v>REPEAT_COMPLAINT, CRITICAL_AT_JC_CREATION, CRITICAL_AFTER_JC_CREATION, DELAY_REASON, QI_THD_REQUIRED, OPEN_ESCALATION, CRITICAL_DTC, THD_UNATTENDED</v>
+        <v>Y, N</v>
       </c>
       <c r="G249" t="str">
         <v/>
@@ -18838,7 +18838,7 @@
         <v/>
       </c>
       <c r="Q249" t="str">
-        <v>What the system checks. Fixed list — each one is coded in the rules engine.</v>
+        <v/>
       </c>
     </row>
     <row r="250">
@@ -18846,13 +18846,13 @@
         <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B250" t="str">
-        <v>businessCondition</v>
+        <v>ruleNo</v>
       </c>
       <c r="C250" t="str">
-        <v>Business Condition</v>
+        <v>Rule No.</v>
       </c>
       <c r="D250" t="str">
-        <v>text</v>
+        <v>number</v>
       </c>
       <c r="E250" t="str">
         <v>Y</v>
@@ -18860,11 +18860,11 @@
       <c r="F250" t="str">
         <v/>
       </c>
-      <c r="G250" t="str">
-        <v/>
-      </c>
-      <c r="H250" t="str">
-        <v/>
+      <c r="G250">
+        <v>1</v>
+      </c>
+      <c r="H250">
+        <v>99</v>
       </c>
       <c r="I250" t="str">
         <v/>
@@ -18899,10 +18899,10 @@
         <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B251" t="str">
-        <v>triggerPoint</v>
+        <v>scenarioCode</v>
       </c>
       <c r="C251" t="str">
-        <v>Trigger Point</v>
+        <v>Scenario</v>
       </c>
       <c r="D251" t="str">
         <v>select</v>
@@ -18911,7 +18911,7 @@
         <v>Y</v>
       </c>
       <c r="F251" t="str">
-        <v>Job Card Creation, Open Job Card, Job Card Closure, THD Age</v>
+        <v>REPEAT_COMPLAINT, CRITICAL_AT_JC_CREATION, CRITICAL_AFTER_JC_CREATION, DELAY_REASON, QI_THD_REQUIRED, OPEN_ESCALATION, CRITICAL_DTC, THD_UNATTENDED</v>
       </c>
       <c r="G251" t="str">
         <v/>
@@ -18944,7 +18944,7 @@
         <v/>
       </c>
       <c r="Q251" t="str">
-        <v/>
+        <v>What the system checks. Fixed list — each one is coded in the rules engine.</v>
       </c>
     </row>
     <row r="252">
@@ -18952,25 +18952,25 @@
         <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B252" t="str">
-        <v>windowValue</v>
+        <v>businessCondition</v>
       </c>
       <c r="C252" t="str">
-        <v>Time Window</v>
+        <v>Business Condition</v>
       </c>
       <c r="D252" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E252" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F252" t="str">
         <v/>
       </c>
-      <c r="G252">
-        <v>1</v>
-      </c>
-      <c r="H252">
-        <v>999</v>
+      <c r="G252" t="str">
+        <v/>
+      </c>
+      <c r="H252" t="str">
+        <v/>
       </c>
       <c r="I252" t="str">
         <v/>
@@ -18997,7 +18997,7 @@
         <v/>
       </c>
       <c r="Q252" t="str">
-        <v>e.g. 30 (days) for repeat visits, 24 (hours) for an unattended THD. Blank = pending from business.</v>
+        <v/>
       </c>
     </row>
     <row r="253">
@@ -19005,19 +19005,19 @@
         <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B253" t="str">
-        <v>windowUnit</v>
+        <v>triggerPoint</v>
       </c>
       <c r="C253" t="str">
-        <v>Window Unit</v>
+        <v>Trigger Point</v>
       </c>
       <c r="D253" t="str">
         <v>select</v>
       </c>
       <c r="E253" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F253" t="str">
-        <v>Hours, Days</v>
+        <v>Job Card Creation, Open Job Card, Job Card Closure, THD Age</v>
       </c>
       <c r="G253" t="str">
         <v/>
@@ -19058,13 +19058,13 @@
         <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B254" t="str">
-        <v>triggerValues</v>
+        <v>windowValue</v>
       </c>
       <c r="C254" t="str">
-        <v>Trigger Values</v>
+        <v>Time Window</v>
       </c>
       <c r="D254" t="str">
-        <v>text</v>
+        <v>number</v>
       </c>
       <c r="E254" t="str">
         <v>N</v>
@@ -19072,11 +19072,11 @@
       <c r="F254" t="str">
         <v/>
       </c>
-      <c r="G254" t="str">
-        <v/>
-      </c>
-      <c r="H254" t="str">
-        <v/>
+      <c r="G254">
+        <v>1</v>
+      </c>
+      <c r="H254">
+        <v>999</v>
       </c>
       <c r="I254" t="str">
         <v/>
@@ -19103,7 +19103,7 @@
         <v/>
       </c>
       <c r="Q254" t="str">
-        <v>Comma-separated values the rule looks for, e.g. the Job Card delay reasons.</v>
+        <v>e.g. 30 (days) for repeat visits, 24 (hours) for an unattended THD. Blank = pending from business.</v>
       </c>
     </row>
     <row r="255">
@@ -19111,19 +19111,19 @@
         <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B255" t="str">
-        <v>escalationComplaint</v>
+        <v>windowUnit</v>
       </c>
       <c r="C255" t="str">
-        <v>Escalation Complaint</v>
+        <v>Window Unit</v>
       </c>
       <c r="D255" t="str">
         <v>select</v>
       </c>
       <c r="E255" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F255" t="str">
-        <v>Yes, No, Yes/No, NA</v>
+        <v>Hours, Days</v>
       </c>
       <c r="G255" t="str">
         <v/>
@@ -19164,16 +19164,16 @@
         <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B256" t="str">
-        <v>thdTag</v>
+        <v>triggerValues</v>
       </c>
       <c r="C256" t="str">
-        <v>THD Tag</v>
+        <v>Trigger Values</v>
       </c>
       <c r="D256" t="str">
         <v>text</v>
       </c>
       <c r="E256" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F256" t="str">
         <v/>
@@ -19209,7 +19209,7 @@
         <v/>
       </c>
       <c r="Q256" t="str">
-        <v/>
+        <v>Comma-separated values the rule looks for, e.g. the Job Card delay reasons.</v>
       </c>
     </row>
     <row r="257">
@@ -19217,10 +19217,10 @@
         <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B257" t="str">
-        <v>assignedTo</v>
+        <v>escalationComplaint</v>
       </c>
       <c r="C257" t="str">
-        <v>Assigned To</v>
+        <v>Escalation Complaint</v>
       </c>
       <c r="D257" t="str">
         <v>select</v>
@@ -19229,7 +19229,7 @@
         <v>Y</v>
       </c>
       <c r="F257" t="str">
-        <v>DET, Tech Executive L1</v>
+        <v>Yes, No, Yes/No, NA</v>
       </c>
       <c r="G257" t="str">
         <v/>
@@ -19270,19 +19270,19 @@
         <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B258" t="str">
-        <v>status</v>
+        <v>thdTag</v>
       </c>
       <c r="C258" t="str">
-        <v>Status</v>
+        <v>THD Tag</v>
       </c>
       <c r="D258" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E258" t="str">
         <v>Y</v>
       </c>
       <c r="F258" t="str">
-        <v>Active, Inactive</v>
+        <v/>
       </c>
       <c r="G258" t="str">
         <v/>
@@ -19320,22 +19320,22 @@
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>thd_critical_complaints</v>
+        <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B259" t="str">
-        <v>ppl</v>
+        <v>assignedTo</v>
       </c>
       <c r="C259" t="str">
-        <v>PPL</v>
+        <v>Assigned To</v>
       </c>
       <c r="D259" t="str">
         <v>select</v>
       </c>
       <c r="E259" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F259" t="str">
-        <v>Nexon, Nexon EV, Altroz, Harrier, Safari, Punch, Punch EV, Tiago, Tiago EV, Tigor, Curvv, Curvv EV</v>
+        <v>DET, Tech Executive L1</v>
       </c>
       <c r="G259" t="str">
         <v/>
@@ -19368,27 +19368,27 @@
         <v/>
       </c>
       <c r="Q259" t="str">
-        <v>One row per PPL + Complaint Code, as in the CRM complaint master. Needed to raise a case; a row without a PPL is listed as pending.</v>
+        <v/>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>thd_critical_complaints</v>
+        <v>thd_auto_trigger_rules</v>
       </c>
       <c r="B260" t="str">
-        <v>complaintCode</v>
+        <v>status</v>
       </c>
       <c r="C260" t="str">
-        <v>Complaint Code</v>
+        <v>Status</v>
       </c>
       <c r="D260" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E260" t="str">
         <v>Y</v>
       </c>
       <c r="F260" t="str">
-        <v/>
+        <v>Active, Inactive</v>
       </c>
       <c r="G260" t="str">
         <v/>
@@ -19429,19 +19429,19 @@
         <v>thd_critical_complaints</v>
       </c>
       <c r="B261" t="str">
-        <v>complaintDescription</v>
+        <v>ppl</v>
       </c>
       <c r="C261" t="str">
-        <v>Complaint Description</v>
+        <v>PPL</v>
       </c>
       <c r="D261" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E261" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F261" t="str">
-        <v/>
+        <v>Nexon, Nexon EV, Altroz, Harrier, Safari, Punch, Punch EV, Tiago, Tiago EV, Tigor, Curvv, Curvv EV</v>
       </c>
       <c r="G261" t="str">
         <v/>
@@ -19474,7 +19474,7 @@
         <v/>
       </c>
       <c r="Q261" t="str">
-        <v/>
+        <v>One row per PPL + Complaint Code, as in the CRM complaint master. Needed to raise a case; a row without a PPL is listed as pending.</v>
       </c>
     </row>
     <row r="262">
@@ -19482,10 +19482,10 @@
         <v>thd_critical_complaints</v>
       </c>
       <c r="B262" t="str">
-        <v>aggregate</v>
+        <v>complaintCode</v>
       </c>
       <c r="C262" t="str">
-        <v>Aggregate</v>
+        <v>Complaint Code</v>
       </c>
       <c r="D262" t="str">
         <v>text</v>
@@ -19535,10 +19535,10 @@
         <v>thd_critical_complaints</v>
       </c>
       <c r="B263" t="str">
-        <v>complaintType</v>
+        <v>complaintDescription</v>
       </c>
       <c r="C263" t="str">
-        <v>Complaint Type</v>
+        <v>Complaint Description</v>
       </c>
       <c r="D263" t="str">
         <v>text</v>
@@ -19588,19 +19588,19 @@
         <v>thd_critical_complaints</v>
       </c>
       <c r="B264" t="str">
-        <v>critical</v>
+        <v>aggregate</v>
       </c>
       <c r="C264" t="str">
-        <v>Critical Complaint</v>
+        <v>Aggregate</v>
       </c>
       <c r="D264" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E264" t="str">
         <v>Y</v>
       </c>
       <c r="F264" t="str">
-        <v>Y, N</v>
+        <v/>
       </c>
       <c r="G264" t="str">
         <v/>
@@ -19641,19 +19641,19 @@
         <v>thd_critical_complaints</v>
       </c>
       <c r="B265" t="str">
-        <v>status</v>
+        <v>complaintType</v>
       </c>
       <c r="C265" t="str">
-        <v>Status</v>
+        <v>Complaint Type</v>
       </c>
       <c r="D265" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E265" t="str">
         <v>Y</v>
       </c>
       <c r="F265" t="str">
-        <v>Active, Inactive</v>
+        <v/>
       </c>
       <c r="G265" t="str">
         <v/>
@@ -19691,22 +19691,22 @@
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>thd_progress</v>
+        <v>thd_critical_complaints</v>
       </c>
       <c r="B266" t="str">
-        <v>value</v>
+        <v>critical</v>
       </c>
       <c r="C266" t="str">
-        <v>Progress</v>
+        <v>Critical Complaint</v>
       </c>
       <c r="D266" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E266" t="str">
         <v>Y</v>
       </c>
       <c r="F266" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G266" t="str">
         <v/>
@@ -19744,7 +19744,7 @@
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>thd_progress</v>
+        <v>thd_critical_complaints</v>
       </c>
       <c r="B267" t="str">
         <v>status</v>
@@ -19800,13 +19800,13 @@
         <v>thd_progress</v>
       </c>
       <c r="B268" t="str">
-        <v>order</v>
+        <v>value</v>
       </c>
       <c r="C268" t="str">
-        <v>Order</v>
+        <v>Progress</v>
       </c>
       <c r="D268" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E268" t="str">
         <v>Y</v>
@@ -19814,11 +19814,11 @@
       <c r="F268" t="str">
         <v/>
       </c>
-      <c r="G268">
-        <v>1</v>
-      </c>
-      <c r="H268">
-        <v>99</v>
+      <c r="G268" t="str">
+        <v/>
+      </c>
+      <c r="H268" t="str">
+        <v/>
       </c>
       <c r="I268" t="str">
         <v/>
@@ -19845,18 +19845,18 @@
         <v/>
       </c>
       <c r="Q268" t="str">
-        <v>Display order in the dropdown.</v>
+        <v/>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>thd_progress_sub_status</v>
+        <v>thd_progress</v>
       </c>
       <c r="B269" t="str">
-        <v>progress</v>
+        <v>status</v>
       </c>
       <c r="C269" t="str">
-        <v>Progress</v>
+        <v>Status</v>
       </c>
       <c r="D269" t="str">
         <v>select</v>
@@ -19865,7 +19865,7 @@
         <v>Y</v>
       </c>
       <c r="F269" t="str">
-        <v>Under Diagnosis, Work in process, Pending for parts, Pending for vendor support, Pending for commercial decision, Pending for Vehicle availability</v>
+        <v>Active, Inactive</v>
       </c>
       <c r="G269" t="str">
         <v/>
@@ -19903,16 +19903,16 @@
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>thd_progress_sub_status</v>
+        <v>thd_progress</v>
       </c>
       <c r="B270" t="str">
-        <v>subStatus</v>
+        <v>order</v>
       </c>
       <c r="C270" t="str">
-        <v>Progress Sub Status</v>
+        <v>Order</v>
       </c>
       <c r="D270" t="str">
-        <v>text</v>
+        <v>number</v>
       </c>
       <c r="E270" t="str">
         <v>Y</v>
@@ -19920,11 +19920,11 @@
       <c r="F270" t="str">
         <v/>
       </c>
-      <c r="G270" t="str">
-        <v/>
-      </c>
-      <c r="H270" t="str">
-        <v/>
+      <c r="G270">
+        <v>1</v>
+      </c>
+      <c r="H270">
+        <v>99</v>
       </c>
       <c r="I270" t="str">
         <v/>
@@ -19951,7 +19951,7 @@
         <v/>
       </c>
       <c r="Q270" t="str">
-        <v/>
+        <v>Display order in the dropdown.</v>
       </c>
     </row>
     <row r="271">
@@ -19959,10 +19959,10 @@
         <v>thd_progress_sub_status</v>
       </c>
       <c r="B271" t="str">
-        <v>status</v>
+        <v>progress</v>
       </c>
       <c r="C271" t="str">
-        <v>Status</v>
+        <v>Progress</v>
       </c>
       <c r="D271" t="str">
         <v>select</v>
@@ -19971,7 +19971,7 @@
         <v>Y</v>
       </c>
       <c r="F271" t="str">
-        <v>Active, Inactive</v>
+        <v>Under Diagnosis, Work in process, Pending for parts, Pending for vendor support, Pending for commercial decision, Pending for Vehicle availability</v>
       </c>
       <c r="G271" t="str">
         <v/>
@@ -20012,13 +20012,13 @@
         <v>thd_progress_sub_status</v>
       </c>
       <c r="B272" t="str">
-        <v>order</v>
+        <v>subStatus</v>
       </c>
       <c r="C272" t="str">
-        <v>Order</v>
+        <v>Progress Sub Status</v>
       </c>
       <c r="D272" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E272" t="str">
         <v>Y</v>
@@ -20026,11 +20026,11 @@
       <c r="F272" t="str">
         <v/>
       </c>
-      <c r="G272">
-        <v>1</v>
-      </c>
-      <c r="H272">
-        <v>99</v>
+      <c r="G272" t="str">
+        <v/>
+      </c>
+      <c r="H272" t="str">
+        <v/>
       </c>
       <c r="I272" t="str">
         <v/>
@@ -20057,27 +20057,27 @@
         <v/>
       </c>
       <c r="Q272" t="str">
-        <v>Display order in the dropdown.</v>
+        <v/>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>thd_complaint_type</v>
+        <v>thd_progress_sub_status</v>
       </c>
       <c r="B273" t="str">
-        <v>value</v>
+        <v>status</v>
       </c>
       <c r="C273" t="str">
-        <v>Type of Complaint</v>
+        <v>Status</v>
       </c>
       <c r="D273" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E273" t="str">
         <v>Y</v>
       </c>
       <c r="F273" t="str">
-        <v/>
+        <v>Active, Inactive</v>
       </c>
       <c r="G273" t="str">
         <v/>
@@ -20115,28 +20115,28 @@
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>thd_complaint_type</v>
+        <v>thd_progress_sub_status</v>
       </c>
       <c r="B274" t="str">
-        <v>status</v>
+        <v>order</v>
       </c>
       <c r="C274" t="str">
-        <v>Status</v>
+        <v>Order</v>
       </c>
       <c r="D274" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E274" t="str">
         <v>Y</v>
       </c>
       <c r="F274" t="str">
-        <v>Active, Inactive</v>
-      </c>
-      <c r="G274" t="str">
-        <v/>
-      </c>
-      <c r="H274" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G274">
+        <v>1</v>
+      </c>
+      <c r="H274">
+        <v>99</v>
       </c>
       <c r="I274" t="str">
         <v/>
@@ -20163,7 +20163,7 @@
         <v/>
       </c>
       <c r="Q274" t="str">
-        <v/>
+        <v>Display order in the dropdown.</v>
       </c>
     </row>
     <row r="275">
@@ -20171,13 +20171,13 @@
         <v>thd_complaint_type</v>
       </c>
       <c r="B275" t="str">
-        <v>order</v>
+        <v>value</v>
       </c>
       <c r="C275" t="str">
-        <v>Order</v>
+        <v>Type of Complaint</v>
       </c>
       <c r="D275" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E275" t="str">
         <v>Y</v>
@@ -20185,11 +20185,11 @@
       <c r="F275" t="str">
         <v/>
       </c>
-      <c r="G275">
-        <v>1</v>
-      </c>
-      <c r="H275">
-        <v>99</v>
+      <c r="G275" t="str">
+        <v/>
+      </c>
+      <c r="H275" t="str">
+        <v/>
       </c>
       <c r="I275" t="str">
         <v/>
@@ -20216,27 +20216,27 @@
         <v/>
       </c>
       <c r="Q275" t="str">
-        <v>Display order in the dropdown.</v>
+        <v/>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>thd_complaint_short_desc</v>
+        <v>thd_complaint_type</v>
       </c>
       <c r="B276" t="str">
-        <v>value</v>
+        <v>status</v>
       </c>
       <c r="C276" t="str">
-        <v>Complaint Short Description</v>
+        <v>Status</v>
       </c>
       <c r="D276" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E276" t="str">
         <v>Y</v>
       </c>
       <c r="F276" t="str">
-        <v/>
+        <v>Active, Inactive</v>
       </c>
       <c r="G276" t="str">
         <v/>
@@ -20274,28 +20274,28 @@
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>thd_complaint_short_desc</v>
+        <v>thd_complaint_type</v>
       </c>
       <c r="B277" t="str">
-        <v>status</v>
+        <v>order</v>
       </c>
       <c r="C277" t="str">
-        <v>Status</v>
+        <v>Order</v>
       </c>
       <c r="D277" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E277" t="str">
         <v>Y</v>
       </c>
       <c r="F277" t="str">
-        <v>Active, Inactive</v>
-      </c>
-      <c r="G277" t="str">
-        <v/>
-      </c>
-      <c r="H277" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G277">
+        <v>1</v>
+      </c>
+      <c r="H277">
+        <v>99</v>
       </c>
       <c r="I277" t="str">
         <v/>
@@ -20322,7 +20322,7 @@
         <v/>
       </c>
       <c r="Q277" t="str">
-        <v/>
+        <v>Display order in the dropdown.</v>
       </c>
     </row>
     <row r="278">
@@ -20330,13 +20330,13 @@
         <v>thd_complaint_short_desc</v>
       </c>
       <c r="B278" t="str">
-        <v>order</v>
+        <v>value</v>
       </c>
       <c r="C278" t="str">
-        <v>Order</v>
+        <v>Complaint Short Description</v>
       </c>
       <c r="D278" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E278" t="str">
         <v>Y</v>
@@ -20344,11 +20344,11 @@
       <c r="F278" t="str">
         <v/>
       </c>
-      <c r="G278">
-        <v>1</v>
-      </c>
-      <c r="H278">
-        <v>99</v>
+      <c r="G278" t="str">
+        <v/>
+      </c>
+      <c r="H278" t="str">
+        <v/>
       </c>
       <c r="I278" t="str">
         <v/>
@@ -20375,27 +20375,27 @@
         <v/>
       </c>
       <c r="Q278" t="str">
-        <v>Display order in the dropdown.</v>
+        <v/>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="str">
-        <v>thd_action_taken</v>
+        <v>thd_complaint_short_desc</v>
       </c>
       <c r="B279" t="str">
-        <v>value</v>
+        <v>status</v>
       </c>
       <c r="C279" t="str">
-        <v>Action Taken</v>
+        <v>Status</v>
       </c>
       <c r="D279" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E279" t="str">
         <v>Y</v>
       </c>
       <c r="F279" t="str">
-        <v/>
+        <v>Active, Inactive</v>
       </c>
       <c r="G279" t="str">
         <v/>
@@ -20433,28 +20433,28 @@
     </row>
     <row r="280">
       <c r="A280" t="str">
-        <v>thd_action_taken</v>
+        <v>thd_complaint_short_desc</v>
       </c>
       <c r="B280" t="str">
-        <v>status</v>
+        <v>order</v>
       </c>
       <c r="C280" t="str">
-        <v>Status</v>
+        <v>Order</v>
       </c>
       <c r="D280" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E280" t="str">
         <v>Y</v>
       </c>
       <c r="F280" t="str">
-        <v>Active, Inactive</v>
-      </c>
-      <c r="G280" t="str">
-        <v/>
-      </c>
-      <c r="H280" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G280">
+        <v>1</v>
+      </c>
+      <c r="H280">
+        <v>99</v>
       </c>
       <c r="I280" t="str">
         <v/>
@@ -20481,7 +20481,7 @@
         <v/>
       </c>
       <c r="Q280" t="str">
-        <v/>
+        <v>Display order in the dropdown.</v>
       </c>
     </row>
     <row r="281">
@@ -20489,13 +20489,13 @@
         <v>thd_action_taken</v>
       </c>
       <c r="B281" t="str">
-        <v>order</v>
+        <v>value</v>
       </c>
       <c r="C281" t="str">
-        <v>Order</v>
+        <v>Action Taken</v>
       </c>
       <c r="D281" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E281" t="str">
         <v>Y</v>
@@ -20503,11 +20503,11 @@
       <c r="F281" t="str">
         <v/>
       </c>
-      <c r="G281">
-        <v>1</v>
-      </c>
-      <c r="H281">
-        <v>99</v>
+      <c r="G281" t="str">
+        <v/>
+      </c>
+      <c r="H281" t="str">
+        <v/>
       </c>
       <c r="I281" t="str">
         <v/>
@@ -20534,27 +20534,27 @@
         <v/>
       </c>
       <c r="Q281" t="str">
-        <v>Display order in the dropdown.</v>
+        <v/>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="str">
-        <v>thd_delay_reason</v>
+        <v>thd_action_taken</v>
       </c>
       <c r="B282" t="str">
-        <v>value</v>
+        <v>status</v>
       </c>
       <c r="C282" t="str">
-        <v>Reason for Delay</v>
+        <v>Status</v>
       </c>
       <c r="D282" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E282" t="str">
         <v>Y</v>
       </c>
       <c r="F282" t="str">
-        <v/>
+        <v>Active, Inactive</v>
       </c>
       <c r="G282" t="str">
         <v/>
@@ -20592,28 +20592,28 @@
     </row>
     <row r="283">
       <c r="A283" t="str">
-        <v>thd_delay_reason</v>
+        <v>thd_action_taken</v>
       </c>
       <c r="B283" t="str">
-        <v>status</v>
+        <v>order</v>
       </c>
       <c r="C283" t="str">
-        <v>Status</v>
+        <v>Order</v>
       </c>
       <c r="D283" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E283" t="str">
         <v>Y</v>
       </c>
       <c r="F283" t="str">
-        <v>Active, Inactive</v>
-      </c>
-      <c r="G283" t="str">
-        <v/>
-      </c>
-      <c r="H283" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G283">
+        <v>1</v>
+      </c>
+      <c r="H283">
+        <v>99</v>
       </c>
       <c r="I283" t="str">
         <v/>
@@ -20640,7 +20640,7 @@
         <v/>
       </c>
       <c r="Q283" t="str">
-        <v/>
+        <v>Display order in the dropdown.</v>
       </c>
     </row>
     <row r="284">
@@ -20648,13 +20648,13 @@
         <v>thd_delay_reason</v>
       </c>
       <c r="B284" t="str">
-        <v>order</v>
+        <v>value</v>
       </c>
       <c r="C284" t="str">
-        <v>Order</v>
+        <v>Reason for Delay</v>
       </c>
       <c r="D284" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E284" t="str">
         <v>Y</v>
@@ -20662,11 +20662,11 @@
       <c r="F284" t="str">
         <v/>
       </c>
-      <c r="G284">
-        <v>1</v>
-      </c>
-      <c r="H284">
-        <v>99</v>
+      <c r="G284" t="str">
+        <v/>
+      </c>
+      <c r="H284" t="str">
+        <v/>
       </c>
       <c r="I284" t="str">
         <v/>
@@ -20693,27 +20693,27 @@
         <v/>
       </c>
       <c r="Q284" t="str">
-        <v>Display order in the dropdown.</v>
+        <v/>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="str">
-        <v>thd_closure_action</v>
+        <v>thd_delay_reason</v>
       </c>
       <c r="B285" t="str">
-        <v>value</v>
+        <v>status</v>
       </c>
       <c r="C285" t="str">
-        <v>Closure Action</v>
+        <v>Status</v>
       </c>
       <c r="D285" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E285" t="str">
         <v>Y</v>
       </c>
       <c r="F285" t="str">
-        <v/>
+        <v>Active, Inactive</v>
       </c>
       <c r="G285" t="str">
         <v/>
@@ -20751,28 +20751,28 @@
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v>thd_closure_action</v>
+        <v>thd_delay_reason</v>
       </c>
       <c r="B286" t="str">
-        <v>status</v>
+        <v>order</v>
       </c>
       <c r="C286" t="str">
-        <v>Status</v>
+        <v>Order</v>
       </c>
       <c r="D286" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E286" t="str">
         <v>Y</v>
       </c>
       <c r="F286" t="str">
-        <v>Active, Inactive</v>
-      </c>
-      <c r="G286" t="str">
-        <v/>
-      </c>
-      <c r="H286" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G286">
+        <v>1</v>
+      </c>
+      <c r="H286">
+        <v>99</v>
       </c>
       <c r="I286" t="str">
         <v/>
@@ -20799,7 +20799,7 @@
         <v/>
       </c>
       <c r="Q286" t="str">
-        <v/>
+        <v>Display order in the dropdown.</v>
       </c>
     </row>
     <row r="287">
@@ -20807,13 +20807,13 @@
         <v>thd_closure_action</v>
       </c>
       <c r="B287" t="str">
-        <v>order</v>
+        <v>value</v>
       </c>
       <c r="C287" t="str">
-        <v>Order</v>
+        <v>Closure Action</v>
       </c>
       <c r="D287" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E287" t="str">
         <v>Y</v>
@@ -20821,11 +20821,11 @@
       <c r="F287" t="str">
         <v/>
       </c>
-      <c r="G287">
-        <v>1</v>
-      </c>
-      <c r="H287">
-        <v>99</v>
+      <c r="G287" t="str">
+        <v/>
+      </c>
+      <c r="H287" t="str">
+        <v/>
       </c>
       <c r="I287" t="str">
         <v/>
@@ -20852,27 +20852,27 @@
         <v/>
       </c>
       <c r="Q287" t="str">
-        <v>Display order in the dropdown.</v>
+        <v/>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>thd_attachment_type</v>
+        <v>thd_closure_action</v>
       </c>
       <c r="B288" t="str">
-        <v>value</v>
+        <v>status</v>
       </c>
       <c r="C288" t="str">
-        <v>Attachment Type</v>
+        <v>Status</v>
       </c>
       <c r="D288" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E288" t="str">
         <v>Y</v>
       </c>
       <c r="F288" t="str">
-        <v/>
+        <v>Active, Inactive</v>
       </c>
       <c r="G288" t="str">
         <v/>
@@ -20910,28 +20910,28 @@
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>thd_attachment_type</v>
+        <v>thd_closure_action</v>
       </c>
       <c r="B289" t="str">
-        <v>status</v>
+        <v>order</v>
       </c>
       <c r="C289" t="str">
-        <v>Status</v>
+        <v>Order</v>
       </c>
       <c r="D289" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E289" t="str">
         <v>Y</v>
       </c>
       <c r="F289" t="str">
-        <v>Active, Inactive</v>
-      </c>
-      <c r="G289" t="str">
-        <v/>
-      </c>
-      <c r="H289" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G289">
+        <v>1</v>
+      </c>
+      <c r="H289">
+        <v>99</v>
       </c>
       <c r="I289" t="str">
         <v/>
@@ -20958,18 +20958,18 @@
         <v/>
       </c>
       <c r="Q289" t="str">
-        <v/>
+        <v>Display order in the dropdown.</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>thd_kms_range</v>
+        <v>thd_attachment_type</v>
       </c>
       <c r="B290" t="str">
-        <v>label</v>
+        <v>value</v>
       </c>
       <c r="C290" t="str">
-        <v>Kms Range</v>
+        <v>Attachment Type</v>
       </c>
       <c r="D290" t="str">
         <v>text</v>
@@ -21016,28 +21016,28 @@
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>thd_kms_range</v>
+        <v>thd_attachment_type</v>
       </c>
       <c r="B291" t="str">
-        <v>fromKm</v>
+        <v>status</v>
       </c>
       <c r="C291" t="str">
-        <v>From Km</v>
+        <v>Status</v>
       </c>
       <c r="D291" t="str">
-        <v>number</v>
+        <v>select</v>
       </c>
       <c r="E291" t="str">
         <v>Y</v>
       </c>
       <c r="F291" t="str">
-        <v/>
-      </c>
-      <c r="G291">
-        <v>0</v>
-      </c>
-      <c r="H291">
-        <v>999999</v>
+        <v>Active, Inactive</v>
+      </c>
+      <c r="G291" t="str">
+        <v/>
+      </c>
+      <c r="H291" t="str">
+        <v/>
       </c>
       <c r="I291" t="str">
         <v/>
@@ -21072,13 +21072,13 @@
         <v>thd_kms_range</v>
       </c>
       <c r="B292" t="str">
-        <v>toKm</v>
+        <v>label</v>
       </c>
       <c r="C292" t="str">
-        <v>To Km</v>
+        <v>Kms Range</v>
       </c>
       <c r="D292" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E292" t="str">
         <v>Y</v>
@@ -21086,11 +21086,11 @@
       <c r="F292" t="str">
         <v/>
       </c>
-      <c r="G292">
-        <v>0</v>
-      </c>
-      <c r="H292">
-        <v>999999</v>
+      <c r="G292" t="str">
+        <v/>
+      </c>
+      <c r="H292" t="str">
+        <v/>
       </c>
       <c r="I292" t="str">
         <v/>
@@ -21125,25 +21125,25 @@
         <v>thd_kms_range</v>
       </c>
       <c r="B293" t="str">
-        <v>status</v>
+        <v>fromKm</v>
       </c>
       <c r="C293" t="str">
-        <v>Status</v>
+        <v>From Km</v>
       </c>
       <c r="D293" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E293" t="str">
         <v>Y</v>
       </c>
       <c r="F293" t="str">
-        <v>Active, Inactive</v>
-      </c>
-      <c r="G293" t="str">
-        <v/>
-      </c>
-      <c r="H293" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G293">
+        <v>0</v>
+      </c>
+      <c r="H293">
+        <v>999999</v>
       </c>
       <c r="I293" t="str">
         <v/>
@@ -21175,16 +21175,16 @@
     </row>
     <row r="294">
       <c r="A294" t="str">
-        <v>thd_vehicle_age</v>
+        <v>thd_kms_range</v>
       </c>
       <c r="B294" t="str">
-        <v>label</v>
+        <v>toKm</v>
       </c>
       <c r="C294" t="str">
-        <v>Age (In Years)</v>
+        <v>To Km</v>
       </c>
       <c r="D294" t="str">
-        <v>text</v>
+        <v>number</v>
       </c>
       <c r="E294" t="str">
         <v>Y</v>
@@ -21192,11 +21192,11 @@
       <c r="F294" t="str">
         <v/>
       </c>
-      <c r="G294" t="str">
-        <v/>
-      </c>
-      <c r="H294" t="str">
-        <v/>
+      <c r="G294">
+        <v>0</v>
+      </c>
+      <c r="H294">
+        <v>999999</v>
       </c>
       <c r="I294" t="str">
         <v/>
@@ -21228,28 +21228,28 @@
     </row>
     <row r="295">
       <c r="A295" t="str">
-        <v>thd_vehicle_age</v>
+        <v>thd_kms_range</v>
       </c>
       <c r="B295" t="str">
-        <v>fromYears</v>
+        <v>status</v>
       </c>
       <c r="C295" t="str">
-        <v>From (Years)</v>
+        <v>Status</v>
       </c>
       <c r="D295" t="str">
-        <v>number</v>
+        <v>select</v>
       </c>
       <c r="E295" t="str">
         <v>Y</v>
       </c>
       <c r="F295" t="str">
-        <v/>
-      </c>
-      <c r="G295">
-        <v>0</v>
-      </c>
-      <c r="H295">
-        <v>50</v>
+        <v>Active, Inactive</v>
+      </c>
+      <c r="G295" t="str">
+        <v/>
+      </c>
+      <c r="H295" t="str">
+        <v/>
       </c>
       <c r="I295" t="str">
         <v/>
@@ -21284,13 +21284,13 @@
         <v>thd_vehicle_age</v>
       </c>
       <c r="B296" t="str">
-        <v>toYears</v>
+        <v>label</v>
       </c>
       <c r="C296" t="str">
-        <v>To (Years)</v>
+        <v>Age (In Years)</v>
       </c>
       <c r="D296" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E296" t="str">
         <v>Y</v>
@@ -21298,11 +21298,11 @@
       <c r="F296" t="str">
         <v/>
       </c>
-      <c r="G296">
-        <v>0</v>
-      </c>
-      <c r="H296">
-        <v>50</v>
+      <c r="G296" t="str">
+        <v/>
+      </c>
+      <c r="H296" t="str">
+        <v/>
       </c>
       <c r="I296" t="str">
         <v/>
@@ -21337,25 +21337,25 @@
         <v>thd_vehicle_age</v>
       </c>
       <c r="B297" t="str">
-        <v>status</v>
+        <v>fromYears</v>
       </c>
       <c r="C297" t="str">
-        <v>Status</v>
+        <v>From (Years)</v>
       </c>
       <c r="D297" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E297" t="str">
         <v>Y</v>
       </c>
       <c r="F297" t="str">
-        <v>Active, Inactive</v>
-      </c>
-      <c r="G297" t="str">
-        <v/>
-      </c>
-      <c r="H297" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G297">
+        <v>0</v>
+      </c>
+      <c r="H297">
+        <v>50</v>
       </c>
       <c r="I297" t="str">
         <v/>
@@ -21387,28 +21387,28 @@
     </row>
     <row r="298">
       <c r="A298" t="str">
-        <v>thd_users</v>
+        <v>thd_vehicle_age</v>
       </c>
       <c r="B298" t="str">
-        <v>role</v>
+        <v>toYears</v>
       </c>
       <c r="C298" t="str">
-        <v>Role</v>
+        <v>To (Years)</v>
       </c>
       <c r="D298" t="str">
-        <v>select</v>
+        <v>number</v>
       </c>
       <c r="E298" t="str">
         <v>Y</v>
       </c>
       <c r="F298" t="str">
-        <v>Tech Executive L1, RTSM, COC L2, Plant, Product Reliability</v>
-      </c>
-      <c r="G298" t="str">
-        <v/>
-      </c>
-      <c r="H298" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="G298">
+        <v>0</v>
+      </c>
+      <c r="H298">
+        <v>50</v>
       </c>
       <c r="I298" t="str">
         <v/>
@@ -21440,13 +21440,13 @@
     </row>
     <row r="299">
       <c r="A299" t="str">
-        <v>thd_users</v>
+        <v>thd_vehicle_age</v>
       </c>
       <c r="B299" t="str">
-        <v>bu</v>
+        <v>status</v>
       </c>
       <c r="C299" t="str">
-        <v>BU</v>
+        <v>Status</v>
       </c>
       <c r="D299" t="str">
         <v>select</v>
@@ -21455,7 +21455,7 @@
         <v>Y</v>
       </c>
       <c r="F299" t="str">
-        <v>PV, EV</v>
+        <v>Active, Inactive</v>
       </c>
       <c r="G299" t="str">
         <v/>
@@ -21496,19 +21496,19 @@
         <v>thd_users</v>
       </c>
       <c r="B300" t="str">
-        <v>userName</v>
+        <v>role</v>
       </c>
       <c r="C300" t="str">
-        <v>User Name</v>
+        <v>Role</v>
       </c>
       <c r="D300" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E300" t="str">
         <v>Y</v>
       </c>
       <c r="F300" t="str">
-        <v/>
+        <v>Tech Executive L1, RTSM, COC L2, Plant, Product Reliability</v>
       </c>
       <c r="G300" t="str">
         <v/>
@@ -21549,19 +21549,19 @@
         <v>thd_users</v>
       </c>
       <c r="B301" t="str">
-        <v>plantName</v>
+        <v>bu</v>
       </c>
       <c r="C301" t="str">
-        <v>Plant Name</v>
+        <v>BU</v>
       </c>
       <c r="D301" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E301" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F301" t="str">
-        <v/>
+        <v>PV, EV</v>
       </c>
       <c r="G301" t="str">
         <v/>
@@ -21594,7 +21594,7 @@
         <v/>
       </c>
       <c r="Q301" t="str">
-        <v>Required for Plant users.</v>
+        <v/>
       </c>
     </row>
     <row r="302">
@@ -21602,16 +21602,16 @@
         <v>thd_users</v>
       </c>
       <c r="B302" t="str">
-        <v>zone</v>
+        <v>userName</v>
       </c>
       <c r="C302" t="str">
-        <v>Zone</v>
+        <v>User Name</v>
       </c>
       <c r="D302" t="str">
         <v>text</v>
       </c>
       <c r="E302" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F302" t="str">
         <v/>
@@ -21655,10 +21655,10 @@
         <v>thd_users</v>
       </c>
       <c r="B303" t="str">
-        <v>region</v>
+        <v>plantName</v>
       </c>
       <c r="C303" t="str">
-        <v>Region</v>
+        <v>Plant Name</v>
       </c>
       <c r="D303" t="str">
         <v>text</v>
@@ -21700,7 +21700,7 @@
         <v/>
       </c>
       <c r="Q303" t="str">
-        <v/>
+        <v>Required for Plant users.</v>
       </c>
     </row>
     <row r="304">
@@ -21708,10 +21708,10 @@
         <v>thd_users</v>
       </c>
       <c r="B304" t="str">
-        <v>crmUserId</v>
+        <v>zone</v>
       </c>
       <c r="C304" t="str">
-        <v>CRM User ID</v>
+        <v>Zone</v>
       </c>
       <c r="D304" t="str">
         <v>text</v>
@@ -21761,10 +21761,10 @@
         <v>thd_users</v>
       </c>
       <c r="B305" t="str">
-        <v>aggregate</v>
+        <v>region</v>
       </c>
       <c r="C305" t="str">
-        <v>Aggregate</v>
+        <v>Region</v>
       </c>
       <c r="D305" t="str">
         <v>text</v>
@@ -21806,7 +21806,7 @@
         <v/>
       </c>
       <c r="Q305" t="str">
-        <v>COC L2 and Plant users can be limited to one aggregate.</v>
+        <v/>
       </c>
     </row>
     <row r="306">
@@ -21814,19 +21814,19 @@
         <v>thd_users</v>
       </c>
       <c r="B306" t="str">
-        <v>status</v>
+        <v>crmUserId</v>
       </c>
       <c r="C306" t="str">
-        <v>Status</v>
+        <v>CRM User ID</v>
       </c>
       <c r="D306" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E306" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F306" t="str">
-        <v>Active, Inactive</v>
+        <v/>
       </c>
       <c r="G306" t="str">
         <v/>
@@ -21864,19 +21864,19 @@
     </row>
     <row r="307">
       <c r="A307" t="str">
-        <v>driver_transit_roster</v>
+        <v>thd_users</v>
       </c>
       <c r="B307" t="str">
-        <v>driverCode</v>
+        <v>aggregate</v>
       </c>
       <c r="C307" t="str">
-        <v>Driver Code</v>
+        <v>Aggregate</v>
       </c>
       <c r="D307" t="str">
         <v>text</v>
       </c>
       <c r="E307" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F307" t="str">
         <v/>
@@ -21912,27 +21912,27 @@
         <v/>
       </c>
       <c r="Q307" t="str">
-        <v/>
+        <v>COC L2 and Plant users can be limited to one aggregate.</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="str">
-        <v>driver_transit_roster</v>
+        <v>thd_users</v>
       </c>
       <c r="B308" t="str">
-        <v>driverName</v>
+        <v>status</v>
       </c>
       <c r="C308" t="str">
-        <v>Driver Full Name</v>
+        <v>Status</v>
       </c>
       <c r="D308" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E308" t="str">
         <v>Y</v>
       </c>
       <c r="F308" t="str">
-        <v/>
+        <v>Active, Inactive</v>
       </c>
       <c r="G308" t="str">
         <v/>
@@ -21973,19 +21973,19 @@
         <v>driver_transit_roster</v>
       </c>
       <c r="B309" t="str">
-        <v>assignedZone</v>
+        <v>driverCode</v>
       </c>
       <c r="C309" t="str">
-        <v>Assigned Territory Zone</v>
+        <v>Driver Code</v>
       </c>
       <c r="D309" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E309" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F309" t="str">
-        <v>Zone A - Hitec City, Zone B - Secunderabad, Zone C - Gachibowli, Zone D - Banjara Hills</v>
+        <v/>
       </c>
       <c r="G309" t="str">
         <v/>
@@ -22026,10 +22026,10 @@
         <v>driver_transit_roster</v>
       </c>
       <c r="B310" t="str">
-        <v>licenseNumber</v>
+        <v>driverName</v>
       </c>
       <c r="C310" t="str">
-        <v>Commercial DL Number</v>
+        <v>Driver Full Name</v>
       </c>
       <c r="D310" t="str">
         <v>text</v>
@@ -22079,10 +22079,10 @@
         <v>driver_transit_roster</v>
       </c>
       <c r="B311" t="str">
-        <v>evCertified</v>
+        <v>assignedZone</v>
       </c>
       <c r="C311" t="str">
-        <v>EV Transit Certified</v>
+        <v>Assigned Territory Zone</v>
       </c>
       <c r="D311" t="str">
         <v>select</v>
@@ -22091,7 +22091,7 @@
         <v>N</v>
       </c>
       <c r="F311" t="str">
-        <v>Y, N</v>
+        <v>Zone A - Hitec City, Zone B - Secunderabad, Zone C - Gachibowli, Zone D - Banjara Hills</v>
       </c>
       <c r="G311" t="str">
         <v/>
@@ -22132,19 +22132,19 @@
         <v>driver_transit_roster</v>
       </c>
       <c r="B312" t="str">
-        <v>active</v>
+        <v>licenseNumber</v>
       </c>
       <c r="C312" t="str">
-        <v>Active</v>
+        <v>Commercial DL Number</v>
       </c>
       <c r="D312" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E312" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F312" t="str">
-        <v>Y, N</v>
+        <v/>
       </c>
       <c r="G312" t="str">
         <v/>
@@ -22182,22 +22182,22 @@
     </row>
     <row r="313">
       <c r="A313" t="str">
-        <v>lounge_reception_checklist</v>
+        <v>driver_transit_roster</v>
       </c>
       <c r="B313" t="str">
-        <v>checkpointCode</v>
+        <v>evCertified</v>
       </c>
       <c r="C313" t="str">
-        <v>Checkpoint Code</v>
+        <v>EV Transit Certified</v>
       </c>
       <c r="D313" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E313" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F313" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G313" t="str">
         <v/>
@@ -22235,22 +22235,22 @@
     </row>
     <row r="314">
       <c r="A314" t="str">
-        <v>lounge_reception_checklist</v>
+        <v>driver_transit_roster</v>
       </c>
       <c r="B314" t="str">
-        <v>checkpointDesc</v>
+        <v>active</v>
       </c>
       <c r="C314" t="str">
-        <v>Reception Standard Requirement</v>
+        <v>Active</v>
       </c>
       <c r="D314" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E314" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F314" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G314" t="str">
         <v/>
@@ -22291,19 +22291,19 @@
         <v>lounge_reception_checklist</v>
       </c>
       <c r="B315" t="str">
-        <v>channel</v>
+        <v>checkpointCode</v>
       </c>
       <c r="C315" t="str">
-        <v>Intake Channel</v>
+        <v>Checkpoint Code</v>
       </c>
       <c r="D315" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E315" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F315" t="str">
-        <v>Walk-in, Pre-Booked Appointment, Express Valet, Breakdown Flatbed</v>
+        <v/>
       </c>
       <c r="G315" t="str">
         <v/>
@@ -22344,19 +22344,19 @@
         <v>lounge_reception_checklist</v>
       </c>
       <c r="B316" t="str">
-        <v>mandatoryProof</v>
+        <v>checkpointDesc</v>
       </c>
       <c r="C316" t="str">
-        <v>Mandatory Photo / Signature</v>
+        <v>Reception Standard Requirement</v>
       </c>
       <c r="D316" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E316" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F316" t="str">
-        <v>Y, N</v>
+        <v/>
       </c>
       <c r="G316" t="str">
         <v/>
@@ -22397,10 +22397,10 @@
         <v>lounge_reception_checklist</v>
       </c>
       <c r="B317" t="str">
-        <v>active</v>
+        <v>channel</v>
       </c>
       <c r="C317" t="str">
-        <v>Active</v>
+        <v>Intake Channel</v>
       </c>
       <c r="D317" t="str">
         <v>select</v>
@@ -22409,7 +22409,7 @@
         <v>N</v>
       </c>
       <c r="F317" t="str">
-        <v>Y, N</v>
+        <v>Walk-in, Pre-Booked Appointment, Express Valet, Breakdown Flatbed</v>
       </c>
       <c r="G317" t="str">
         <v/>
@@ -22447,22 +22447,22 @@
     </row>
     <row r="318">
       <c r="A318" t="str">
-        <v>gate_security_checklist</v>
+        <v>lounge_reception_checklist</v>
       </c>
       <c r="B318" t="str">
-        <v>ruleId</v>
+        <v>mandatoryProof</v>
       </c>
       <c r="C318" t="str">
-        <v>Gate Rule Code</v>
+        <v>Mandatory Photo / Signature</v>
       </c>
       <c r="D318" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E318" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F318" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G318" t="str">
         <v/>
@@ -22500,13 +22500,13 @@
     </row>
     <row r="319">
       <c r="A319" t="str">
-        <v>gate_security_checklist</v>
+        <v>lounge_reception_checklist</v>
       </c>
       <c r="B319" t="str">
-        <v>direction</v>
+        <v>active</v>
       </c>
       <c r="C319" t="str">
-        <v>Movement Direction</v>
+        <v>Active</v>
       </c>
       <c r="D319" t="str">
         <v>select</v>
@@ -22515,7 +22515,7 @@
         <v>N</v>
       </c>
       <c r="F319" t="str">
-        <v>Inward (Check-in), Outward (Check-out), Internal Bay Transit</v>
+        <v>Y, N</v>
       </c>
       <c r="G319" t="str">
         <v/>
@@ -22556,10 +22556,10 @@
         <v>gate_security_checklist</v>
       </c>
       <c r="B320" t="str">
-        <v>verificationItem</v>
+        <v>ruleId</v>
       </c>
       <c r="C320" t="str">
-        <v>Verification Protocol</v>
+        <v>Gate Rule Code</v>
       </c>
       <c r="D320" t="str">
         <v>text</v>
@@ -22609,10 +22609,10 @@
         <v>gate_security_checklist</v>
       </c>
       <c r="B321" t="str">
-        <v>anprSync</v>
+        <v>direction</v>
       </c>
       <c r="C321" t="str">
-        <v>ANPR Camera Auto-Verify</v>
+        <v>Movement Direction</v>
       </c>
       <c r="D321" t="str">
         <v>select</v>
@@ -22621,7 +22621,7 @@
         <v>N</v>
       </c>
       <c r="F321" t="str">
-        <v>Y, N</v>
+        <v>Inward (Check-in), Outward (Check-out), Internal Bay Transit</v>
       </c>
       <c r="G321" t="str">
         <v/>
@@ -22662,19 +22662,19 @@
         <v>gate_security_checklist</v>
       </c>
       <c r="B322" t="str">
-        <v>active</v>
+        <v>verificationItem</v>
       </c>
       <c r="C322" t="str">
-        <v>Active</v>
+        <v>Verification Protocol</v>
       </c>
       <c r="D322" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E322" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F322" t="str">
-        <v>Y, N</v>
+        <v/>
       </c>
       <c r="G322" t="str">
         <v/>
@@ -22712,22 +22712,22 @@
     </row>
     <row r="323">
       <c r="A323" t="str">
-        <v>gate_denial_reasons</v>
+        <v>gate_security_checklist</v>
       </c>
       <c r="B323" t="str">
-        <v>denialCode</v>
+        <v>anprSync</v>
       </c>
       <c r="C323" t="str">
-        <v>Denial Code</v>
+        <v>ANPR Camera Auto-Verify</v>
       </c>
       <c r="D323" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E323" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F323" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G323" t="str">
         <v/>
@@ -22765,22 +22765,22 @@
     </row>
     <row r="324">
       <c r="A324" t="str">
-        <v>gate_denial_reasons</v>
+        <v>gate_security_checklist</v>
       </c>
       <c r="B324" t="str">
-        <v>reason</v>
+        <v>active</v>
       </c>
       <c r="C324" t="str">
-        <v>Security Denial / Hold Reason</v>
+        <v>Active</v>
       </c>
       <c r="D324" t="str">
-        <v>text</v>
+        <v>select</v>
       </c>
       <c r="E324" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F324" t="str">
-        <v/>
+        <v>Y, N</v>
       </c>
       <c r="G324" t="str">
         <v/>
@@ -22821,19 +22821,19 @@
         <v>gate_denial_reasons</v>
       </c>
       <c r="B325" t="str">
-        <v>escalateTo</v>
+        <v>denialCode</v>
       </c>
       <c r="C325" t="str">
-        <v>Immediate Notification Target</v>
+        <v>Denial Code</v>
       </c>
       <c r="D325" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E325" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F325" t="str">
-        <v>Works Manager, Security Officer In-Charge, Service Head, Customer Relation Manager</v>
+        <v/>
       </c>
       <c r="G325" t="str">
         <v/>
@@ -22874,57 +22874,163 @@
         <v>gate_denial_reasons</v>
       </c>
       <c r="B326" t="str">
+        <v>reason</v>
+      </c>
+      <c r="C326" t="str">
+        <v>Security Denial / Hold Reason</v>
+      </c>
+      <c r="D326" t="str">
+        <v>text</v>
+      </c>
+      <c r="E326" t="str">
+        <v>Y</v>
+      </c>
+      <c r="F326" t="str">
+        <v/>
+      </c>
+      <c r="G326" t="str">
+        <v/>
+      </c>
+      <c r="H326" t="str">
+        <v/>
+      </c>
+      <c r="I326" t="str">
+        <v/>
+      </c>
+      <c r="J326" t="str">
+        <v/>
+      </c>
+      <c r="K326" t="str">
+        <v/>
+      </c>
+      <c r="L326" t="str">
+        <v/>
+      </c>
+      <c r="M326" t="str">
+        <v>N</v>
+      </c>
+      <c r="N326" t="str">
+        <v/>
+      </c>
+      <c r="O326" t="str">
+        <v/>
+      </c>
+      <c r="P326" t="str">
+        <v/>
+      </c>
+      <c r="Q326" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>gate_denial_reasons</v>
+      </c>
+      <c r="B327" t="str">
+        <v>escalateTo</v>
+      </c>
+      <c r="C327" t="str">
+        <v>Immediate Notification Target</v>
+      </c>
+      <c r="D327" t="str">
+        <v>select</v>
+      </c>
+      <c r="E327" t="str">
+        <v>N</v>
+      </c>
+      <c r="F327" t="str">
+        <v>Works Manager, Security Officer In-Charge, Service Head, Customer Relation Manager</v>
+      </c>
+      <c r="G327" t="str">
+        <v/>
+      </c>
+      <c r="H327" t="str">
+        <v/>
+      </c>
+      <c r="I327" t="str">
+        <v/>
+      </c>
+      <c r="J327" t="str">
+        <v/>
+      </c>
+      <c r="K327" t="str">
+        <v/>
+      </c>
+      <c r="L327" t="str">
+        <v/>
+      </c>
+      <c r="M327" t="str">
+        <v>N</v>
+      </c>
+      <c r="N327" t="str">
+        <v/>
+      </c>
+      <c r="O327" t="str">
+        <v/>
+      </c>
+      <c r="P327" t="str">
+        <v/>
+      </c>
+      <c r="Q327" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>gate_denial_reasons</v>
+      </c>
+      <c r="B328" t="str">
         <v>active</v>
       </c>
-      <c r="C326" t="str">
+      <c r="C328" t="str">
         <v>Active</v>
       </c>
-      <c r="D326" t="str">
+      <c r="D328" t="str">
         <v>select</v>
       </c>
-      <c r="E326" t="str">
-        <v>N</v>
-      </c>
-      <c r="F326" t="str">
+      <c r="E328" t="str">
+        <v>N</v>
+      </c>
+      <c r="F328" t="str">
         <v>Y, N</v>
       </c>
-      <c r="G326" t="str">
-        <v/>
-      </c>
-      <c r="H326" t="str">
-        <v/>
-      </c>
-      <c r="I326" t="str">
-        <v/>
-      </c>
-      <c r="J326" t="str">
-        <v/>
-      </c>
-      <c r="K326" t="str">
-        <v/>
-      </c>
-      <c r="L326" t="str">
-        <v/>
-      </c>
-      <c r="M326" t="str">
-        <v>N</v>
-      </c>
-      <c r="N326" t="str">
-        <v/>
-      </c>
-      <c r="O326" t="str">
-        <v/>
-      </c>
-      <c r="P326" t="str">
-        <v/>
-      </c>
-      <c r="Q326" t="str">
+      <c r="G328" t="str">
+        <v/>
+      </c>
+      <c r="H328" t="str">
+        <v/>
+      </c>
+      <c r="I328" t="str">
+        <v/>
+      </c>
+      <c r="J328" t="str">
+        <v/>
+      </c>
+      <c r="K328" t="str">
+        <v/>
+      </c>
+      <c r="L328" t="str">
+        <v/>
+      </c>
+      <c r="M328" t="str">
+        <v>N</v>
+      </c>
+      <c r="N328" t="str">
+        <v/>
+      </c>
+      <c r="O328" t="str">
+        <v/>
+      </c>
+      <c r="P328" t="str">
+        <v/>
+      </c>
+      <c r="Q328" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q326"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q328"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -23407,7 +23513,7 @@
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -23420,18 +23526,24 @@
         <v>persona</v>
       </c>
       <c r="D1" t="str">
-        <v>approvesBelow</v>
+        <v>canApprove</v>
       </c>
       <c r="E1" t="str">
+        <v>approvesUpTo</v>
+      </c>
+      <c r="F1" t="str">
         <v>actions</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>forwardTo</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>reminderHours</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
+        <v>reminderVia</v>
+      </c>
+      <c r="J1" t="str">
         <v>status</v>
       </c>
     </row>
@@ -23445,19 +23557,25 @@
       <c r="C2" t="str">
         <v>Claim Manager</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="E2">
         <v>20000</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Approve, Send to CCM/ACCM</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>CCM/ACCM</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>24</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
+        <v>Notification + Email</v>
+      </c>
+      <c r="J2" t="str">
         <v>Active</v>
       </c>
     </row>
@@ -23472,24 +23590,62 @@
         <v>CCM/ACCM</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>N</v>
       </c>
       <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
         <v>Send to SHQ Lead 1, Send Back for Correction</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>SHQ Lead 1</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>24</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
+        <v>Notification + Email</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>WAM-03</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="str">
+        <v>SHQ Lead 1</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v>Approve</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4">
+        <v>24</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Notification + Email</v>
+      </c>
+      <c r="J4" t="str">
         <v>Active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(claims): Reminder Via is a text field (dropdowns need 2+ options)
The regenerated BA catalogue workbook failed its re-import check because a
dropdown must offer at least two options. 'Notification + Email' is now the
default of a text field.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DwiSAaMRyjNA589tWt8iz
</commit_message>
<xml_diff>
--- a/docs/templates/TML_Existing_Masters_Catalogue.xlsx
+++ b/docs/templates/TML_Existing_Masters_Catalogue.xlsx
@@ -17156,13 +17156,13 @@
         <v>Reminder Via</v>
       </c>
       <c r="D218" t="str">
-        <v>select</v>
+        <v>text</v>
       </c>
       <c r="E218" t="str">
         <v>Y</v>
       </c>
       <c r="F218" t="str">
-        <v>Notification + Email</v>
+        <v/>
       </c>
       <c r="G218" t="str">
         <v/>
@@ -17195,7 +17195,7 @@
         <v/>
       </c>
       <c r="Q218" t="str">
-        <v/>
+        <v>BA: a notification and an email only — no automatic escalation.</v>
       </c>
     </row>
     <row r="219">

</xml_diff>

<commit_message>
BU: PV and EV are separate values, no combined "PV + EV"
- Remove COMMON_BU_SCOPE; every BU field uses COMMON_BU (PV, EV, CV)
- Rows that said "PV + EV" are split into a PV row and an EV row (pause reasons, complaint codes);
  sample divisions / bodyshop facilities get a single BU
- Bodyshop facility form drops the "PV + EV (Composite)" option
- Test guards against a combined BU value; docs updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DwiSAaMRyjNA589tWt8iz
</commit_message>
<xml_diff>
--- a/docs/templates/TML_Existing_Masters_Catalogue.xlsx
+++ b/docs/templates/TML_Existing_Masters_Catalogue.xlsx
@@ -768,7 +768,7 @@
         <v>Sample Motors Hyderabad</v>
       </c>
       <c r="D2" t="str">
-        <v>PV + EV</v>
+        <v>PV</v>
       </c>
       <c r="E2">
         <v>10</v>
@@ -806,7 +806,7 @@
         <v>Sample Motors Hyderabad</v>
       </c>
       <c r="D3" t="str">
-        <v>PV + EV</v>
+        <v>EV</v>
       </c>
       <c r="E3">
         <v>15</v>
@@ -981,7 +981,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1011,7 +1011,7 @@
         <v>PR-01</v>
       </c>
       <c r="B2" t="str">
-        <v>PV + EV</v>
+        <v>PV</v>
       </c>
       <c r="C2" t="str">
         <v>Parts Not Available</v>
@@ -1031,39 +1031,39 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>PR-02</v>
+        <v>PR-01-EV</v>
       </c>
       <c r="B3" t="str">
-        <v>PV + EV</v>
+        <v>EV</v>
       </c>
       <c r="C3" t="str">
-        <v>THD Resolution Pending</v>
+        <v>Parts Not Available</v>
       </c>
       <c r="D3" t="str">
-        <v>THD Number (Open/Closed)</v>
+        <v>Part Description (DPM Unissued)</v>
       </c>
       <c r="E3" t="str">
-        <v>NA</v>
+        <v>Order Number (SAP Order No)</v>
       </c>
       <c r="F3" t="str">
         <v>Y</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>PR-03</v>
+        <v>PR-02</v>
       </c>
       <c r="B4" t="str">
-        <v>PV + EV</v>
+        <v>PV</v>
       </c>
       <c r="C4" t="str">
-        <v>Waiting for customer approval</v>
+        <v>THD Resolution Pending</v>
       </c>
       <c r="D4" t="str">
-        <v>Customer Approval Doc / OTP</v>
+        <v>THD Number (Open/Closed)</v>
       </c>
       <c r="E4" t="str">
         <v>NA</v>
@@ -1072,21 +1072,21 @@
         <v>Y</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>PR-04</v>
+        <v>PR-02-EV</v>
       </c>
       <c r="B5" t="str">
-        <v>PV + EV</v>
+        <v>EV</v>
       </c>
       <c r="C5" t="str">
-        <v>Manpower absenteeism</v>
+        <v>THD Resolution Pending</v>
       </c>
       <c r="D5" t="str">
-        <v>Supervisor Override Code</v>
+        <v>THD Number (Open/Closed)</v>
       </c>
       <c r="E5" t="str">
         <v>NA</v>
@@ -1095,104 +1095,265 @@
         <v>Y</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PR-05</v>
+        <v>PR-03</v>
       </c>
       <c r="B6" t="str">
-        <v>EV</v>
+        <v>PV</v>
       </c>
       <c r="C6" t="str">
-        <v>HV Battery Support Awaited</v>
+        <v>Waiting for customer approval</v>
       </c>
       <c r="D6" t="str">
-        <v>Ticket No (Ticket Description)</v>
+        <v>Customer Approval Doc / OTP</v>
       </c>
       <c r="E6" t="str">
-        <v>Safety Officer Clearance</v>
+        <v>NA</v>
       </c>
       <c r="F6" t="str">
         <v>Y</v>
       </c>
       <c r="G6">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>PR-06</v>
+        <v>PR-03-EV</v>
       </c>
       <c r="B7" t="str">
-        <v>PV + EV</v>
+        <v>EV</v>
       </c>
       <c r="C7" t="str">
-        <v>Vendor Support Awaited</v>
+        <v>Waiting for customer approval</v>
       </c>
       <c r="D7" t="str">
-        <v>Vendor Name (BOSCH / Delphi)</v>
+        <v>Customer Approval Doc / OTP</v>
       </c>
       <c r="E7" t="str">
-        <v>Vendor Visit Date</v>
+        <v>NA</v>
       </c>
       <c r="F7" t="str">
         <v>Y</v>
       </c>
       <c r="G7">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>PR-07</v>
+        <v>PR-04</v>
       </c>
       <c r="B8" t="str">
-        <v>PV + EV</v>
+        <v>PV</v>
       </c>
       <c r="C8" t="str">
-        <v>Goodwill Approval Awaited</v>
+        <v>Manpower absenteeism</v>
       </c>
       <c r="D8" t="str">
-        <v>Goodwill Request ID (CRM)</v>
+        <v>Supervisor Override Code</v>
       </c>
       <c r="E8" t="str">
-        <v>DGM Endorsement ID</v>
+        <v>NA</v>
       </c>
       <c r="F8" t="str">
         <v>Y</v>
       </c>
       <c r="G8">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>PR-04-EV</v>
+      </c>
+      <c r="B9" t="str">
+        <v>EV</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Manpower absenteeism</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Supervisor Override Code</v>
+      </c>
+      <c r="E9" t="str">
+        <v>NA</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PR-05</v>
+      </c>
+      <c r="B10" t="str">
+        <v>EV</v>
+      </c>
+      <c r="C10" t="str">
+        <v>HV Battery Support Awaited</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Ticket No (Ticket Description)</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Safety Officer Clearance</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>PR-06</v>
+      </c>
+      <c r="B11" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Vendor Support Awaited</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Vendor Name (BOSCH / Delphi)</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Vendor Visit Date</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>PR-06-EV</v>
+      </c>
+      <c r="B12" t="str">
+        <v>EV</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Vendor Support Awaited</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Vendor Name (BOSCH / Delphi)</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Vendor Visit Date</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>PR-07</v>
+      </c>
+      <c r="B13" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Goodwill Approval Awaited</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Goodwill Request ID (CRM)</v>
+      </c>
+      <c r="E13" t="str">
+        <v>DGM Endorsement ID</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G13">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>PR-07-EV</v>
+      </c>
+      <c r="B14" t="str">
+        <v>EV</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Goodwill Approval Awaited</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Goodwill Request ID (CRM)</v>
+      </c>
+      <c r="E14" t="str">
+        <v>DGM Endorsement ID</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G14">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>PR-08</v>
       </c>
-      <c r="B9" t="str">
-        <v>PV + EV</v>
-      </c>
-      <c r="C9" t="str">
+      <c r="B15" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C15" t="str">
         <v>Extended Warranty Approval Awaited</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D15" t="str">
         <v>Request ID (Raised to TML)</v>
       </c>
-      <c r="E9" t="str">
+      <c r="E15" t="str">
         <v>Insurance Surveyor Ref</v>
       </c>
-      <c r="F9" t="str">
-        <v>Y</v>
-      </c>
-      <c r="G9">
+      <c r="F15" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G15">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>PR-08-EV</v>
+      </c>
+      <c r="B16" t="str">
+        <v>EV</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Extended Warranty Approval Awaited</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Request ID (Raised to TML)</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Insurance Surveyor Ref</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G16">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6616,7 +6777,7 @@
         <v>N</v>
       </c>
       <c r="F24" t="str">
-        <v>PV + EV, PV, EV, CV</v>
+        <v>PV, EV, CV</v>
       </c>
       <c r="G24" t="str">
         <v/>
@@ -8047,7 +8208,7 @@
         <v>N</v>
       </c>
       <c r="F51" t="str">
-        <v>PV + EV, PV, EV, CV</v>
+        <v>PV, EV, CV</v>
       </c>
       <c r="G51" t="str">
         <v/>
@@ -9001,7 +9162,7 @@
         <v>Y</v>
       </c>
       <c r="F69" t="str">
-        <v>PV + EV, PV, EV, CV</v>
+        <v>PV, EV, CV</v>
       </c>
       <c r="G69" t="str">
         <v/>
@@ -23487,7 +23648,7 @@
 
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I83"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -23607,19 +23768,19 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>COMMON_BU_SCOPE-01</v>
+        <v>THD_PROGRESS-01</v>
       </c>
       <c r="B5" t="str">
-        <v>COMMON_BU_SCOPE</v>
+        <v>THD_PROGRESS</v>
       </c>
       <c r="C5" t="str">
-        <v>COMMON</v>
+        <v>THD</v>
       </c>
       <c r="D5" t="str">
-        <v>Applicable BU</v>
+        <v>Progress</v>
       </c>
       <c r="E5" t="str">
-        <v>PV + EV</v>
+        <v>Under Diagnosis</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -23636,19 +23797,19 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>COMMON_BU_SCOPE-02</v>
+        <v>THD_PROGRESS-02</v>
       </c>
       <c r="B6" t="str">
-        <v>COMMON_BU_SCOPE</v>
+        <v>THD_PROGRESS</v>
       </c>
       <c r="C6" t="str">
-        <v>COMMON</v>
+        <v>THD</v>
       </c>
       <c r="D6" t="str">
-        <v>Applicable BU</v>
+        <v>Progress</v>
       </c>
       <c r="E6" t="str">
-        <v>PV</v>
+        <v>Work in process</v>
       </c>
       <c r="F6">
         <v>2</v>
@@ -23665,19 +23826,19 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>COMMON_BU_SCOPE-03</v>
+        <v>THD_PROGRESS-03</v>
       </c>
       <c r="B7" t="str">
-        <v>COMMON_BU_SCOPE</v>
+        <v>THD_PROGRESS</v>
       </c>
       <c r="C7" t="str">
-        <v>COMMON</v>
+        <v>THD</v>
       </c>
       <c r="D7" t="str">
-        <v>Applicable BU</v>
+        <v>Progress</v>
       </c>
       <c r="E7" t="str">
-        <v>EV</v>
+        <v>Pending for parts</v>
       </c>
       <c r="F7">
         <v>3</v>
@@ -23694,19 +23855,19 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>COMMON_BU_SCOPE-04</v>
+        <v>THD_PROGRESS-04</v>
       </c>
       <c r="B8" t="str">
-        <v>COMMON_BU_SCOPE</v>
+        <v>THD_PROGRESS</v>
       </c>
       <c r="C8" t="str">
-        <v>COMMON</v>
+        <v>THD</v>
       </c>
       <c r="D8" t="str">
-        <v>Applicable BU</v>
+        <v>Progress</v>
       </c>
       <c r="E8" t="str">
-        <v>CV</v>
+        <v>Pending for vendor support</v>
       </c>
       <c r="F8">
         <v>4</v>
@@ -23723,7 +23884,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>THD_PROGRESS-01</v>
+        <v>THD_PROGRESS-05</v>
       </c>
       <c r="B9" t="str">
         <v>THD_PROGRESS</v>
@@ -23735,10 +23896,10 @@
         <v>Progress</v>
       </c>
       <c r="E9" t="str">
-        <v>Under Diagnosis</v>
+        <v>Pending for commercial decision</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G9" t="str">
         <v/>
@@ -23752,7 +23913,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>THD_PROGRESS-02</v>
+        <v>THD_PROGRESS-06</v>
       </c>
       <c r="B10" t="str">
         <v>THD_PROGRESS</v>
@@ -23764,10 +23925,10 @@
         <v>Progress</v>
       </c>
       <c r="E10" t="str">
-        <v>Work in process</v>
+        <v>Pending for Vehicle availability</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G10" t="str">
         <v/>
@@ -23781,28 +23942,28 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>THD_PROGRESS-03</v>
+        <v>THD_PROGRESS_SUB_STATUS-01</v>
       </c>
       <c r="B11" t="str">
-        <v>THD_PROGRESS</v>
+        <v>THD_PROGRESS_SUB_STATUS</v>
       </c>
       <c r="C11" t="str">
         <v>THD</v>
       </c>
       <c r="D11" t="str">
-        <v>Progress</v>
+        <v>Progress Sub Status</v>
       </c>
       <c r="E11" t="str">
-        <v>Pending for parts</v>
+        <v>U/I DET</v>
       </c>
       <c r="F11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G11" t="str">
-        <v/>
+        <v>THD_PROGRESS</v>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>Under Diagnosis</v>
       </c>
       <c r="I11" t="str">
         <v>Active</v>
@@ -23810,28 +23971,28 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>THD_PROGRESS-04</v>
+        <v>THD_PROGRESS_SUB_STATUS-02</v>
       </c>
       <c r="B12" t="str">
-        <v>THD_PROGRESS</v>
+        <v>THD_PROGRESS_SUB_STATUS</v>
       </c>
       <c r="C12" t="str">
         <v>THD</v>
       </c>
       <c r="D12" t="str">
-        <v>Progress</v>
+        <v>Progress Sub Status</v>
       </c>
       <c r="E12" t="str">
-        <v>Pending for vendor support</v>
+        <v>U/I COC</v>
       </c>
       <c r="F12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G12" t="str">
-        <v/>
+        <v>THD_PROGRESS</v>
       </c>
       <c r="H12" t="str">
-        <v/>
+        <v>Under Diagnosis</v>
       </c>
       <c r="I12" t="str">
         <v>Active</v>
@@ -23839,28 +24000,28 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>THD_PROGRESS-05</v>
+        <v>THD_PROGRESS_SUB_STATUS-03</v>
       </c>
       <c r="B13" t="str">
-        <v>THD_PROGRESS</v>
+        <v>THD_PROGRESS_SUB_STATUS</v>
       </c>
       <c r="C13" t="str">
         <v>THD</v>
       </c>
       <c r="D13" t="str">
-        <v>Progress</v>
+        <v>Progress Sub Status</v>
       </c>
       <c r="E13" t="str">
-        <v>Pending for commercial decision</v>
+        <v>U/I Vendor</v>
       </c>
       <c r="F13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>THD_PROGRESS</v>
       </c>
       <c r="H13" t="str">
-        <v/>
+        <v>Under Diagnosis</v>
       </c>
       <c r="I13" t="str">
         <v>Active</v>
@@ -23868,28 +24029,28 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>THD_PROGRESS-06</v>
+        <v>THD_PROGRESS_SUB_STATUS-04</v>
       </c>
       <c r="B14" t="str">
-        <v>THD_PROGRESS</v>
+        <v>THD_PROGRESS_SUB_STATUS</v>
       </c>
       <c r="C14" t="str">
         <v>THD</v>
       </c>
       <c r="D14" t="str">
-        <v>Progress</v>
+        <v>Progress Sub Status</v>
       </c>
       <c r="E14" t="str">
-        <v>Pending for Vehicle availability</v>
+        <v>U/I Plant Team</v>
       </c>
       <c r="F14">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G14" t="str">
-        <v/>
+        <v>THD_PROGRESS</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>Under Diagnosis</v>
       </c>
       <c r="I14" t="str">
         <v>Active</v>
@@ -23897,7 +24058,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-01</v>
+        <v>THD_PROGRESS_SUB_STATUS-05</v>
       </c>
       <c r="B15" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -23909,16 +24070,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E15" t="str">
-        <v>U/I DET</v>
+        <v>WIP DET</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G15" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H15" t="str">
-        <v>Under Diagnosis</v>
+        <v>Work in process</v>
       </c>
       <c r="I15" t="str">
         <v>Active</v>
@@ -23926,7 +24087,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-02</v>
+        <v>THD_PROGRESS_SUB_STATUS-06</v>
       </c>
       <c r="B16" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -23938,16 +24099,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E16" t="str">
-        <v>U/I COC</v>
+        <v>WIP W/S Team</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G16" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H16" t="str">
-        <v>Under Diagnosis</v>
+        <v>Work in process</v>
       </c>
       <c r="I16" t="str">
         <v>Active</v>
@@ -23955,7 +24116,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-03</v>
+        <v>THD_PROGRESS_SUB_STATUS-07</v>
       </c>
       <c r="B17" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -23967,16 +24128,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E17" t="str">
-        <v>U/I Vendor</v>
+        <v>WIP Vendor</v>
       </c>
       <c r="F17">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G17" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H17" t="str">
-        <v>Under Diagnosis</v>
+        <v>Work in process</v>
       </c>
       <c r="I17" t="str">
         <v>Active</v>
@@ -23984,7 +24145,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-04</v>
+        <v>THD_PROGRESS_SUB_STATUS-08</v>
       </c>
       <c r="B18" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -23996,16 +24157,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E18" t="str">
-        <v>U/I Plant Team</v>
+        <v>Order status</v>
       </c>
       <c r="F18">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G18" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H18" t="str">
-        <v>Under Diagnosis</v>
+        <v>Pending for parts</v>
       </c>
       <c r="I18" t="str">
         <v>Active</v>
@@ -24013,7 +24174,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-05</v>
+        <v>THD_PROGRESS_SUB_STATUS-09</v>
       </c>
       <c r="B19" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24025,16 +24186,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E19" t="str">
-        <v>WIP DET</v>
+        <v>Part receipt status</v>
       </c>
       <c r="F19">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G19" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H19" t="str">
-        <v>Work in process</v>
+        <v>Pending for parts</v>
       </c>
       <c r="I19" t="str">
         <v>Active</v>
@@ -24042,7 +24203,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-06</v>
+        <v>THD_PROGRESS_SUB_STATUS-10</v>
       </c>
       <c r="B20" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24054,16 +24215,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E20" t="str">
-        <v>WIP W/S Team</v>
+        <v>Vendor details</v>
       </c>
       <c r="F20">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G20" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H20" t="str">
-        <v>Work in process</v>
+        <v>Pending for vendor support</v>
       </c>
       <c r="I20" t="str">
         <v>Active</v>
@@ -24071,7 +24232,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-07</v>
+        <v>THD_PROGRESS_SUB_STATUS-11</v>
       </c>
       <c r="B21" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24083,16 +24244,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E21" t="str">
-        <v>WIP Vendor</v>
+        <v>Request raised</v>
       </c>
       <c r="F21">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G21" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H21" t="str">
-        <v>Work in process</v>
+        <v>Pending for vendor support</v>
       </c>
       <c r="I21" t="str">
         <v>Active</v>
@@ -24100,7 +24261,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-08</v>
+        <v>THD_PROGRESS_SUB_STATUS-12</v>
       </c>
       <c r="B22" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24112,16 +24273,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E22" t="str">
-        <v>Order status</v>
+        <v>Status</v>
       </c>
       <c r="F22">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G22" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H22" t="str">
-        <v>Pending for parts</v>
+        <v>Pending for vendor support</v>
       </c>
       <c r="I22" t="str">
         <v>Active</v>
@@ -24129,7 +24290,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-09</v>
+        <v>THD_PROGRESS_SUB_STATUS-13</v>
       </c>
       <c r="B23" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24141,16 +24302,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E23" t="str">
-        <v>Part receipt status</v>
+        <v>Pending for approval</v>
       </c>
       <c r="F23">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G23" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H23" t="str">
-        <v>Pending for parts</v>
+        <v>Pending for commercial decision</v>
       </c>
       <c r="I23" t="str">
         <v>Active</v>
@@ -24158,7 +24319,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-10</v>
+        <v>THD_PROGRESS_SUB_STATUS-14</v>
       </c>
       <c r="B24" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24170,16 +24331,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E24" t="str">
-        <v>Vendor details</v>
+        <v>Approval received</v>
       </c>
       <c r="F24">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G24" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H24" t="str">
-        <v>Pending for vendor support</v>
+        <v>Pending for commercial decision</v>
       </c>
       <c r="I24" t="str">
         <v>Active</v>
@@ -24187,7 +24348,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-11</v>
+        <v>THD_PROGRESS_SUB_STATUS-15</v>
       </c>
       <c r="B25" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24199,16 +24360,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E25" t="str">
-        <v>Request raised</v>
+        <v>Expected date</v>
       </c>
       <c r="F25">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G25" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H25" t="str">
-        <v>Pending for vendor support</v>
+        <v>Pending for Vehicle availability</v>
       </c>
       <c r="I25" t="str">
         <v>Active</v>
@@ -24216,7 +24377,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-12</v>
+        <v>THD_PROGRESS_SUB_STATUS-16</v>
       </c>
       <c r="B26" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24228,16 +24389,16 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E26" t="str">
-        <v>Status</v>
+        <v>Status as on date</v>
       </c>
       <c r="F26">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G26" t="str">
         <v>THD_PROGRESS</v>
       </c>
       <c r="H26" t="str">
-        <v>Pending for vendor support</v>
+        <v>Pending for Vehicle availability</v>
       </c>
       <c r="I26" t="str">
         <v>Active</v>
@@ -24245,28 +24406,28 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-13</v>
+        <v>THD_COMPLAINT_TYPE-01</v>
       </c>
       <c r="B27" t="str">
-        <v>THD_PROGRESS_SUB_STATUS</v>
+        <v>THD_COMPLAINT_TYPE</v>
       </c>
       <c r="C27" t="str">
         <v>THD</v>
       </c>
       <c r="D27" t="str">
-        <v>Progress Sub Status</v>
+        <v>Type of Complaint</v>
       </c>
       <c r="E27" t="str">
-        <v>Pending for approval</v>
+        <v>Technical Query</v>
       </c>
       <c r="F27">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="G27" t="str">
-        <v>THD_PROGRESS</v>
+        <v/>
       </c>
       <c r="H27" t="str">
-        <v>Pending for commercial decision</v>
+        <v/>
       </c>
       <c r="I27" t="str">
         <v>Active</v>
@@ -24274,28 +24435,28 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-14</v>
+        <v>THD_COMPLAINT_TYPE-02</v>
       </c>
       <c r="B28" t="str">
-        <v>THD_PROGRESS_SUB_STATUS</v>
+        <v>THD_COMPLAINT_TYPE</v>
       </c>
       <c r="C28" t="str">
         <v>THD</v>
       </c>
       <c r="D28" t="str">
-        <v>Progress Sub Status</v>
+        <v>Type of Complaint</v>
       </c>
       <c r="E28" t="str">
-        <v>Approval received</v>
+        <v>Technical Support</v>
       </c>
       <c r="F28">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G28" t="str">
-        <v>THD_PROGRESS</v>
+        <v/>
       </c>
       <c r="H28" t="str">
-        <v>Pending for commercial decision</v>
+        <v/>
       </c>
       <c r="I28" t="str">
         <v>Active</v>
@@ -24303,28 +24464,28 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-15</v>
+        <v>THD_COMPLAINT_SHORT_DESC-01</v>
       </c>
       <c r="B29" t="str">
-        <v>THD_PROGRESS_SUB_STATUS</v>
+        <v>THD_COMPLAINT_SHORT_DESC</v>
       </c>
       <c r="C29" t="str">
         <v>THD</v>
       </c>
       <c r="D29" t="str">
-        <v>Progress Sub Status</v>
+        <v>Complaint Short Description</v>
       </c>
       <c r="E29" t="str">
-        <v>Expected date</v>
+        <v>Abnormal noise</v>
       </c>
       <c r="F29">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G29" t="str">
-        <v>THD_PROGRESS</v>
+        <v/>
       </c>
       <c r="H29" t="str">
-        <v>Pending for Vehicle availability</v>
+        <v/>
       </c>
       <c r="I29" t="str">
         <v>Active</v>
@@ -24332,28 +24493,28 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-16</v>
+        <v>THD_COMPLAINT_SHORT_DESC-02</v>
       </c>
       <c r="B30" t="str">
-        <v>THD_PROGRESS_SUB_STATUS</v>
+        <v>THD_COMPLAINT_SHORT_DESC</v>
       </c>
       <c r="C30" t="str">
         <v>THD</v>
       </c>
       <c r="D30" t="str">
-        <v>Progress Sub Status</v>
+        <v>Complaint Short Description</v>
       </c>
       <c r="E30" t="str">
-        <v>Status as on date</v>
+        <v>Warning lamps ON</v>
       </c>
       <c r="F30">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G30" t="str">
-        <v>THD_PROGRESS</v>
+        <v/>
       </c>
       <c r="H30" t="str">
-        <v>Pending for Vehicle availability</v>
+        <v/>
       </c>
       <c r="I30" t="str">
         <v>Active</v>
@@ -24361,22 +24522,22 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>THD_COMPLAINT_TYPE-01</v>
+        <v>THD_COMPLAINT_SHORT_DESC-03</v>
       </c>
       <c r="B31" t="str">
-        <v>THD_COMPLAINT_TYPE</v>
+        <v>THD_COMPLAINT_SHORT_DESC</v>
       </c>
       <c r="C31" t="str">
         <v>THD</v>
       </c>
       <c r="D31" t="str">
-        <v>Type of Complaint</v>
+        <v>Complaint Short Description</v>
       </c>
       <c r="E31" t="str">
-        <v>Technical Query</v>
+        <v>Oil leakage</v>
       </c>
       <c r="F31">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G31" t="str">
         <v/>
@@ -24390,22 +24551,22 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>THD_COMPLAINT_TYPE-02</v>
+        <v>THD_COMPLAINT_SHORT_DESC-04</v>
       </c>
       <c r="B32" t="str">
-        <v>THD_COMPLAINT_TYPE</v>
+        <v>THD_COMPLAINT_SHORT_DESC</v>
       </c>
       <c r="C32" t="str">
         <v>THD</v>
       </c>
       <c r="D32" t="str">
-        <v>Type of Complaint</v>
+        <v>Complaint Short Description</v>
       </c>
       <c r="E32" t="str">
-        <v>Technical Support</v>
+        <v>Coolant leakage</v>
       </c>
       <c r="F32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G32" t="str">
         <v/>
@@ -24419,7 +24580,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-01</v>
+        <v>THD_COMPLAINT_SHORT_DESC-05</v>
       </c>
       <c r="B33" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24431,10 +24592,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E33" t="str">
-        <v>Abnormal noise</v>
+        <v>Engine overheating</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G33" t="str">
         <v/>
@@ -24448,7 +24609,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-02</v>
+        <v>THD_COMPLAINT_SHORT_DESC-06</v>
       </c>
       <c r="B34" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24460,10 +24621,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E34" t="str">
-        <v>Warning lamps ON</v>
+        <v>Smell – burning, fuel, foul odor from outside, etc.</v>
       </c>
       <c r="F34">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G34" t="str">
         <v/>
@@ -24477,7 +24638,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-03</v>
+        <v>THD_COMPLAINT_SHORT_DESC-07</v>
       </c>
       <c r="B35" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24489,10 +24650,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E35" t="str">
-        <v>Oil leakage</v>
+        <v>Smoke issues</v>
       </c>
       <c r="F35">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G35" t="str">
         <v/>
@@ -24506,7 +24667,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-04</v>
+        <v>THD_COMPLAINT_SHORT_DESC-08</v>
       </c>
       <c r="B36" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24518,10 +24679,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E36" t="str">
-        <v>Coolant leakage</v>
+        <v>Oil-Coolant mix</v>
       </c>
       <c r="F36">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G36" t="str">
         <v/>
@@ -24535,7 +24696,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-05</v>
+        <v>THD_COMPLAINT_SHORT_DESC-09</v>
       </c>
       <c r="B37" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24547,10 +24708,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E37" t="str">
-        <v>Engine overheating</v>
+        <v>Gear shifting issues</v>
       </c>
       <c r="F37">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G37" t="str">
         <v/>
@@ -24564,7 +24725,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-06</v>
+        <v>THD_COMPLAINT_SHORT_DESC-10</v>
       </c>
       <c r="B38" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24576,10 +24737,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E38" t="str">
-        <v>Smell – burning, fuel, foul odor from outside, etc.</v>
+        <v>AC cooling issues</v>
       </c>
       <c r="F38">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G38" t="str">
         <v/>
@@ -24593,7 +24754,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-07</v>
+        <v>THD_COMPLAINT_SHORT_DESC-11</v>
       </c>
       <c r="B39" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24605,10 +24766,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E39" t="str">
-        <v>Smoke issues</v>
+        <v>Jerking / vibration / misfiring</v>
       </c>
       <c r="F39">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G39" t="str">
         <v/>
@@ -24622,7 +24783,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-08</v>
+        <v>THD_COMPLAINT_SHORT_DESC-12</v>
       </c>
       <c r="B40" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24634,10 +24795,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E40" t="str">
-        <v>Oil-Coolant mix</v>
+        <v>Steering hard</v>
       </c>
       <c r="F40">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G40" t="str">
         <v/>
@@ -24651,7 +24812,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-09</v>
+        <v>THD_COMPLAINT_SHORT_DESC-13</v>
       </c>
       <c r="B41" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24663,10 +24824,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E41" t="str">
-        <v>Gear shifting issues</v>
+        <v>Vehicle pulling</v>
       </c>
       <c r="F41">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G41" t="str">
         <v/>
@@ -24680,7 +24841,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-10</v>
+        <v>THD_COMPLAINT_SHORT_DESC-14</v>
       </c>
       <c r="B42" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24692,10 +24853,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E42" t="str">
-        <v>AC cooling issues</v>
+        <v>Starting problem</v>
       </c>
       <c r="F42">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G42" t="str">
         <v/>
@@ -24709,7 +24870,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-11</v>
+        <v>THD_COMPLAINT_SHORT_DESC-15</v>
       </c>
       <c r="B43" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24721,10 +24882,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E43" t="str">
-        <v>Jerking / vibration / misfiring</v>
+        <v>Tyre wear / cut</v>
       </c>
       <c r="F43">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G43" t="str">
         <v/>
@@ -24738,7 +24899,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-12</v>
+        <v>THD_COMPLAINT_SHORT_DESC-16</v>
       </c>
       <c r="B44" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24750,10 +24911,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E44" t="str">
-        <v>Steering hard</v>
+        <v>Damaged / broken / cracked / soiled</v>
       </c>
       <c r="F44">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G44" t="str">
         <v/>
@@ -24767,7 +24928,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-13</v>
+        <v>THD_COMPLAINT_SHORT_DESC-17</v>
       </c>
       <c r="B45" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24779,10 +24940,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E45" t="str">
-        <v>Vehicle pulling</v>
+        <v>Part missing / fallen-off</v>
       </c>
       <c r="F45">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G45" t="str">
         <v/>
@@ -24796,7 +24957,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-14</v>
+        <v>THD_COMPLAINT_SHORT_DESC-18</v>
       </c>
       <c r="B46" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24808,10 +24969,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E46" t="str">
-        <v>Starting problem</v>
+        <v>Uneven gaps / flushness issues</v>
       </c>
       <c r="F46">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G46" t="str">
         <v/>
@@ -24825,7 +24986,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-15</v>
+        <v>THD_COMPLAINT_SHORT_DESC-19</v>
       </c>
       <c r="B47" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24837,10 +24998,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E47" t="str">
-        <v>Tyre wear / cut</v>
+        <v>Paint / rust issues</v>
       </c>
       <c r="F47">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G47" t="str">
         <v/>
@@ -24854,7 +25015,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-16</v>
+        <v>THD_COMPLAINT_SHORT_DESC-20</v>
       </c>
       <c r="B48" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24866,10 +25027,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E48" t="str">
-        <v>Damaged / broken / cracked / soiled</v>
+        <v>Not working / functioning issues / system malfunction</v>
       </c>
       <c r="F48">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G48" t="str">
         <v/>
@@ -24883,7 +25044,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-17</v>
+        <v>THD_COMPLAINT_SHORT_DESC-21</v>
       </c>
       <c r="B49" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24895,10 +25056,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E49" t="str">
-        <v>Part missing / fallen-off</v>
+        <v>Crash / airbag related issues</v>
       </c>
       <c r="F49">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G49" t="str">
         <v/>
@@ -24912,7 +25073,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-18</v>
+        <v>THD_COMPLAINT_SHORT_DESC-22</v>
       </c>
       <c r="B50" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24924,10 +25085,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E50" t="str">
-        <v>Uneven gaps / flushness issues</v>
+        <v>Thermal issues</v>
       </c>
       <c r="F50">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G50" t="str">
         <v/>
@@ -24941,7 +25102,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-19</v>
+        <v>THD_COMPLAINT_SHORT_DESC-23</v>
       </c>
       <c r="B51" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24953,10 +25114,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E51" t="str">
-        <v>Paint / rust issues</v>
+        <v>Brake ineffective</v>
       </c>
       <c r="F51">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G51" t="str">
         <v/>
@@ -24970,7 +25131,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-20</v>
+        <v>THD_COMPLAINT_SHORT_DESC-24</v>
       </c>
       <c r="B52" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24982,10 +25143,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E52" t="str">
-        <v>Not working / functioning issues / system malfunction</v>
+        <v>Poor pick-up</v>
       </c>
       <c r="F52">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G52" t="str">
         <v/>
@@ -24999,7 +25160,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-21</v>
+        <v>THD_COMPLAINT_SHORT_DESC-25</v>
       </c>
       <c r="B53" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -25011,10 +25172,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E53" t="str">
-        <v>Crash / airbag related issues</v>
+        <v>Infotainment system issues</v>
       </c>
       <c r="F53">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G53" t="str">
         <v/>
@@ -25028,7 +25189,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-22</v>
+        <v>THD_COMPLAINT_SHORT_DESC-26</v>
       </c>
       <c r="B54" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -25040,10 +25201,10 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E54" t="str">
-        <v>Thermal issues</v>
+        <v>Water entry in cabin</v>
       </c>
       <c r="F54">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G54" t="str">
         <v/>
@@ -25057,22 +25218,22 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-23</v>
+        <v>THD_ACTION_TAKEN-01</v>
       </c>
       <c r="B55" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC</v>
+        <v>THD_ACTION_TAKEN</v>
       </c>
       <c r="C55" t="str">
         <v>THD</v>
       </c>
       <c r="D55" t="str">
-        <v>Complaint Short Description</v>
+        <v>Action Taken</v>
       </c>
       <c r="E55" t="str">
-        <v>Brake ineffective</v>
+        <v>Issue concluded and proceeded as per Field Investigation</v>
       </c>
       <c r="F55">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="G55" t="str">
         <v/>
@@ -25086,22 +25247,22 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-24</v>
+        <v>THD_ACTION_TAKEN-02</v>
       </c>
       <c r="B56" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC</v>
+        <v>THD_ACTION_TAKEN</v>
       </c>
       <c r="C56" t="str">
         <v>THD</v>
       </c>
       <c r="D56" t="str">
-        <v>Complaint Short Description</v>
+        <v>Action Taken</v>
       </c>
       <c r="E56" t="str">
-        <v>Poor pick-up</v>
+        <v>Suggested checks based on observations</v>
       </c>
       <c r="F56">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G56" t="str">
         <v/>
@@ -25115,22 +25276,22 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-25</v>
+        <v>THD_ACTION_TAKEN-03</v>
       </c>
       <c r="B57" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC</v>
+        <v>THD_ACTION_TAKEN</v>
       </c>
       <c r="C57" t="str">
         <v>THD</v>
       </c>
       <c r="D57" t="str">
-        <v>Complaint Short Description</v>
+        <v>Action Taken</v>
       </c>
       <c r="E57" t="str">
-        <v>Infotainment system issues</v>
+        <v>Known issue – suggested part replacement</v>
       </c>
       <c r="F57">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="G57" t="str">
         <v/>
@@ -25144,22 +25305,22 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-26</v>
+        <v>THD_ACTION_TAKEN-04</v>
       </c>
       <c r="B58" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC</v>
+        <v>THD_ACTION_TAKEN</v>
       </c>
       <c r="C58" t="str">
         <v>THD</v>
       </c>
       <c r="D58" t="str">
-        <v>Complaint Short Description</v>
+        <v>Action Taken</v>
       </c>
       <c r="E58" t="str">
-        <v>Water entry in cabin</v>
+        <v>Updated software / parameterization</v>
       </c>
       <c r="F58">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="G58" t="str">
         <v/>
@@ -25173,7 +25334,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>THD_ACTION_TAKEN-01</v>
+        <v>THD_ACTION_TAKEN-05</v>
       </c>
       <c r="B59" t="str">
         <v>THD_ACTION_TAKEN</v>
@@ -25185,10 +25346,10 @@
         <v>Action Taken</v>
       </c>
       <c r="E59" t="str">
-        <v>Issue concluded and proceeded as per Field Investigation</v>
+        <v>Suggested part replacement based on observation</v>
       </c>
       <c r="F59">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G59" t="str">
         <v/>
@@ -25202,7 +25363,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>THD_ACTION_TAKEN-02</v>
+        <v>THD_ACTION_TAKEN-06</v>
       </c>
       <c r="B60" t="str">
         <v>THD_ACTION_TAKEN</v>
@@ -25214,10 +25375,10 @@
         <v>Action Taken</v>
       </c>
       <c r="E60" t="str">
-        <v>Suggested checks based on observations</v>
+        <v>Vehicle ready for delivery</v>
       </c>
       <c r="F60">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G60" t="str">
         <v/>
@@ -25231,7 +25392,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>THD_ACTION_TAKEN-03</v>
+        <v>THD_ACTION_TAKEN-07</v>
       </c>
       <c r="B61" t="str">
         <v>THD_ACTION_TAKEN</v>
@@ -25243,10 +25404,10 @@
         <v>Action Taken</v>
       </c>
       <c r="E61" t="str">
-        <v>Known issue – suggested part replacement</v>
+        <v>Vehicle not available; is with Customer</v>
       </c>
       <c r="F61">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G61" t="str">
         <v/>
@@ -25260,22 +25421,22 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>THD_ACTION_TAKEN-04</v>
+        <v>THD_DELAY_REASON-01</v>
       </c>
       <c r="B62" t="str">
-        <v>THD_ACTION_TAKEN</v>
+        <v>THD_DELAY_REASON</v>
       </c>
       <c r="C62" t="str">
         <v>THD</v>
       </c>
       <c r="D62" t="str">
-        <v>Action Taken</v>
+        <v>Reason for Delay</v>
       </c>
       <c r="E62" t="str">
-        <v>Updated software / parameterization</v>
+        <v>Diagnosis and investigation</v>
       </c>
       <c r="F62">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G62" t="str">
         <v/>
@@ -25289,22 +25450,22 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>THD_ACTION_TAKEN-05</v>
+        <v>THD_DELAY_REASON-02</v>
       </c>
       <c r="B63" t="str">
-        <v>THD_ACTION_TAKEN</v>
+        <v>THD_DELAY_REASON</v>
       </c>
       <c r="C63" t="str">
         <v>THD</v>
       </c>
       <c r="D63" t="str">
-        <v>Action Taken</v>
+        <v>Reason for Delay</v>
       </c>
       <c r="E63" t="str">
-        <v>Suggested part replacement based on observation</v>
+        <v>Work content</v>
       </c>
       <c r="F63">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G63" t="str">
         <v/>
@@ -25318,22 +25479,22 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>THD_ACTION_TAKEN-06</v>
+        <v>THD_DELAY_REASON-03</v>
       </c>
       <c r="B64" t="str">
-        <v>THD_ACTION_TAKEN</v>
+        <v>THD_DELAY_REASON</v>
       </c>
       <c r="C64" t="str">
         <v>THD</v>
       </c>
       <c r="D64" t="str">
-        <v>Action Taken</v>
+        <v>Reason for Delay</v>
       </c>
       <c r="E64" t="str">
-        <v>Vehicle ready for delivery</v>
+        <v>Non-availability of spare parts</v>
       </c>
       <c r="F64">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G64" t="str">
         <v/>
@@ -25347,22 +25508,22 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>THD_ACTION_TAKEN-07</v>
+        <v>THD_DELAY_REASON-04</v>
       </c>
       <c r="B65" t="str">
-        <v>THD_ACTION_TAKEN</v>
+        <v>THD_DELAY_REASON</v>
       </c>
       <c r="C65" t="str">
         <v>THD</v>
       </c>
       <c r="D65" t="str">
-        <v>Action Taken</v>
+        <v>Reason for Delay</v>
       </c>
       <c r="E65" t="str">
-        <v>Vehicle not available; is with Customer</v>
+        <v>Non-availability of vehicle</v>
       </c>
       <c r="F65">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G65" t="str">
         <v/>
@@ -25376,7 +25537,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>THD_DELAY_REASON-01</v>
+        <v>THD_DELAY_REASON-05</v>
       </c>
       <c r="B66" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25388,10 +25549,10 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E66" t="str">
-        <v>Diagnosis and investigation</v>
+        <v>Dealer response</v>
       </c>
       <c r="F66">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G66" t="str">
         <v/>
@@ -25405,7 +25566,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>THD_DELAY_REASON-02</v>
+        <v>THD_DELAY_REASON-06</v>
       </c>
       <c r="B67" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25417,10 +25578,10 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E67" t="str">
-        <v>Work content</v>
+        <v>Plant / ERC / vendor intervention</v>
       </c>
       <c r="F67">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G67" t="str">
         <v/>
@@ -25434,7 +25595,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>THD_DELAY_REASON-03</v>
+        <v>THD_DELAY_REASON-07</v>
       </c>
       <c r="B68" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25446,10 +25607,10 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E68" t="str">
-        <v>Non-availability of spare parts</v>
+        <v>Software / server / TDS Tool issue</v>
       </c>
       <c r="F68">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G68" t="str">
         <v/>
@@ -25463,7 +25624,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>THD_DELAY_REASON-04</v>
+        <v>THD_DELAY_REASON-08</v>
       </c>
       <c r="B69" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25475,10 +25636,10 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E69" t="str">
-        <v>Non-availability of vehicle</v>
+        <v>Solution not available</v>
       </c>
       <c r="F69">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G69" t="str">
         <v/>
@@ -25492,7 +25653,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>THD_DELAY_REASON-05</v>
+        <v>THD_DELAY_REASON-09</v>
       </c>
       <c r="B70" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25504,10 +25665,10 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E70" t="str">
-        <v>Dealer response</v>
+        <v>Pending for Commercial Decision / Customer Approval</v>
       </c>
       <c r="F70">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G70" t="str">
         <v/>
@@ -25521,7 +25682,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>THD_DELAY_REASON-06</v>
+        <v>THD_DELAY_REASON-10</v>
       </c>
       <c r="B71" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25533,10 +25694,10 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E71" t="str">
-        <v>Plant / ERC / vendor intervention</v>
+        <v>Dealer not responding</v>
       </c>
       <c r="F71">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G71" t="str">
         <v/>
@@ -25550,22 +25711,22 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>THD_DELAY_REASON-07</v>
+        <v>THD_CLOSURE_ACTION-01</v>
       </c>
       <c r="B72" t="str">
-        <v>THD_DELAY_REASON</v>
+        <v>THD_CLOSURE_ACTION</v>
       </c>
       <c r="C72" t="str">
         <v>THD</v>
       </c>
       <c r="D72" t="str">
-        <v>Reason for Delay</v>
+        <v>Closure Action</v>
       </c>
       <c r="E72" t="str">
-        <v>Software / server / TDS Tool issue</v>
+        <v>Closed</v>
       </c>
       <c r="F72">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G72" t="str">
         <v/>
@@ -25579,22 +25740,22 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>THD_DELAY_REASON-08</v>
+        <v>THD_CLOSURE_ACTION-02</v>
       </c>
       <c r="B73" t="str">
-        <v>THD_DELAY_REASON</v>
+        <v>THD_CLOSURE_ACTION</v>
       </c>
       <c r="C73" t="str">
         <v>THD</v>
       </c>
       <c r="D73" t="str">
-        <v>Reason for Delay</v>
+        <v>Closure Action</v>
       </c>
       <c r="E73" t="str">
-        <v>Solution not available</v>
+        <v>Closed With Feedback</v>
       </c>
       <c r="F73">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G73" t="str">
         <v/>
@@ -25608,22 +25769,22 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>THD_DELAY_REASON-09</v>
+        <v>THD_CLOSURE_ACTION-03</v>
       </c>
       <c r="B74" t="str">
-        <v>THD_DELAY_REASON</v>
+        <v>THD_CLOSURE_ACTION</v>
       </c>
       <c r="C74" t="str">
         <v>THD</v>
       </c>
       <c r="D74" t="str">
-        <v>Reason for Delay</v>
+        <v>Closure Action</v>
       </c>
       <c r="E74" t="str">
-        <v>Pending for Commercial Decision / Customer Approval</v>
+        <v>Closed With Early Warning</v>
       </c>
       <c r="F74">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G74" t="str">
         <v/>
@@ -25637,22 +25798,22 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>THD_DELAY_REASON-10</v>
+        <v>THD_ATTACHMENT_TYPE-01</v>
       </c>
       <c r="B75" t="str">
-        <v>THD_DELAY_REASON</v>
+        <v>THD_ATTACHMENT_TYPE</v>
       </c>
       <c r="C75" t="str">
         <v>THD</v>
       </c>
       <c r="D75" t="str">
-        <v>Reason for Delay</v>
+        <v>Attachment Type</v>
       </c>
       <c r="E75" t="str">
-        <v>Dealer not responding</v>
+        <v>DIR Report</v>
       </c>
       <c r="F75">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G75" t="str">
         <v/>
@@ -25666,19 +25827,19 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>THD_CLOSURE_ACTION-01</v>
+        <v>CLAIM_BUDGET_PURPOSE-01</v>
       </c>
       <c r="B76" t="str">
-        <v>THD_CLOSURE_ACTION</v>
+        <v>CLAIM_BUDGET_PURPOSE</v>
       </c>
       <c r="C76" t="str">
-        <v>THD</v>
+        <v>CLAIM</v>
       </c>
       <c r="D76" t="str">
-        <v>Closure Action</v>
+        <v>Allocation Purpose</v>
       </c>
       <c r="E76" t="str">
-        <v>Closed</v>
+        <v>Approved Yearly Budget</v>
       </c>
       <c r="F76">
         <v>1</v>
@@ -25695,19 +25856,19 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>THD_CLOSURE_ACTION-02</v>
+        <v>CLAIM_BUDGET_PURPOSE-02</v>
       </c>
       <c r="B77" t="str">
-        <v>THD_CLOSURE_ACTION</v>
+        <v>CLAIM_BUDGET_PURPOSE</v>
       </c>
       <c r="C77" t="str">
-        <v>THD</v>
+        <v>CLAIM</v>
       </c>
       <c r="D77" t="str">
-        <v>Closure Action</v>
+        <v>Allocation Purpose</v>
       </c>
       <c r="E77" t="str">
-        <v>Closed With Feedback</v>
+        <v>Special Budget</v>
       </c>
       <c r="F77">
         <v>2</v>
@@ -25724,22 +25885,22 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>THD_CLOSURE_ACTION-03</v>
+        <v>CLAIM_SPECIAL_GOODWILL-01</v>
       </c>
       <c r="B78" t="str">
-        <v>THD_CLOSURE_ACTION</v>
+        <v>CLAIM_SPECIAL_GOODWILL</v>
       </c>
       <c r="C78" t="str">
-        <v>THD</v>
+        <v>CLAIM</v>
       </c>
       <c r="D78" t="str">
-        <v>Closure Action</v>
+        <v>Special Claim</v>
       </c>
       <c r="E78" t="str">
-        <v>Closed With Early Warning</v>
+        <v>IUPR</v>
       </c>
       <c r="F78">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G78" t="str">
         <v/>
@@ -25753,22 +25914,22 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>THD_ATTACHMENT_TYPE-01</v>
+        <v>CLAIM_SPECIAL_GOODWILL-02</v>
       </c>
       <c r="B79" t="str">
-        <v>THD_ATTACHMENT_TYPE</v>
+        <v>CLAIM_SPECIAL_GOODWILL</v>
       </c>
       <c r="C79" t="str">
-        <v>THD</v>
+        <v>CLAIM</v>
       </c>
       <c r="D79" t="str">
-        <v>Attachment Type</v>
+        <v>Special Claim</v>
       </c>
       <c r="E79" t="str">
-        <v>DIR Report</v>
+        <v>Thrive</v>
       </c>
       <c r="F79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G79" t="str">
         <v/>
@@ -25782,19 +25943,19 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>CLAIM_BUDGET_PURPOSE-01</v>
+        <v>CLAIM_ISSUE_DESCRIPTION-01</v>
       </c>
       <c r="B80" t="str">
-        <v>CLAIM_BUDGET_PURPOSE</v>
+        <v>CLAIM_ISSUE_DESCRIPTION</v>
       </c>
       <c r="C80" t="str">
         <v>CLAIM</v>
       </c>
       <c r="D80" t="str">
-        <v>Allocation Purpose</v>
+        <v>Issue Description</v>
       </c>
       <c r="E80" t="str">
-        <v>Approved Yearly Budget</v>
+        <v>Thermal Incident</v>
       </c>
       <c r="F80">
         <v>1</v>
@@ -25811,19 +25972,19 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>CLAIM_BUDGET_PURPOSE-02</v>
+        <v>CLAIM_ISSUE_DESCRIPTION-02</v>
       </c>
       <c r="B81" t="str">
-        <v>CLAIM_BUDGET_PURPOSE</v>
+        <v>CLAIM_ISSUE_DESCRIPTION</v>
       </c>
       <c r="C81" t="str">
         <v>CLAIM</v>
       </c>
       <c r="D81" t="str">
-        <v>Allocation Purpose</v>
+        <v>Issue Description</v>
       </c>
       <c r="E81" t="str">
-        <v>Special Budget</v>
+        <v>Engine Failure</v>
       </c>
       <c r="F81">
         <v>2</v>
@@ -25840,19 +26001,19 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>CLAIM_SPECIAL_GOODWILL-01</v>
+        <v>CLAIM_COMPLAINT_TYPE-01</v>
       </c>
       <c r="B82" t="str">
-        <v>CLAIM_SPECIAL_GOODWILL</v>
+        <v>CLAIM_COMPLAINT_TYPE</v>
       </c>
       <c r="C82" t="str">
         <v>CLAIM</v>
       </c>
       <c r="D82" t="str">
-        <v>Special Claim</v>
+        <v>Complaint Type</v>
       </c>
       <c r="E82" t="str">
-        <v>IUPR</v>
+        <v>Transmission</v>
       </c>
       <c r="F82">
         <v>1</v>
@@ -25869,19 +26030,19 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>CLAIM_SPECIAL_GOODWILL-02</v>
+        <v>CLAIM_COMPLAINT_TYPE-02</v>
       </c>
       <c r="B83" t="str">
-        <v>CLAIM_SPECIAL_GOODWILL</v>
+        <v>CLAIM_COMPLAINT_TYPE</v>
       </c>
       <c r="C83" t="str">
         <v>CLAIM</v>
       </c>
       <c r="D83" t="str">
-        <v>Special Claim</v>
+        <v>Complaint Type</v>
       </c>
       <c r="E83" t="str">
-        <v>Thrive</v>
+        <v>Clutch</v>
       </c>
       <c r="F83">
         <v>2</v>
@@ -25896,125 +26057,9 @@
         <v>Active</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" t="str">
-        <v>CLAIM_ISSUE_DESCRIPTION-01</v>
-      </c>
-      <c r="B84" t="str">
-        <v>CLAIM_ISSUE_DESCRIPTION</v>
-      </c>
-      <c r="C84" t="str">
-        <v>CLAIM</v>
-      </c>
-      <c r="D84" t="str">
-        <v>Issue Description</v>
-      </c>
-      <c r="E84" t="str">
-        <v>Thermal Incident</v>
-      </c>
-      <c r="F84">
-        <v>1</v>
-      </c>
-      <c r="G84" t="str">
-        <v/>
-      </c>
-      <c r="H84" t="str">
-        <v/>
-      </c>
-      <c r="I84" t="str">
-        <v>Active</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="str">
-        <v>CLAIM_ISSUE_DESCRIPTION-02</v>
-      </c>
-      <c r="B85" t="str">
-        <v>CLAIM_ISSUE_DESCRIPTION</v>
-      </c>
-      <c r="C85" t="str">
-        <v>CLAIM</v>
-      </c>
-      <c r="D85" t="str">
-        <v>Issue Description</v>
-      </c>
-      <c r="E85" t="str">
-        <v>Engine Failure</v>
-      </c>
-      <c r="F85">
-        <v>2</v>
-      </c>
-      <c r="G85" t="str">
-        <v/>
-      </c>
-      <c r="H85" t="str">
-        <v/>
-      </c>
-      <c r="I85" t="str">
-        <v>Active</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="str">
-        <v>CLAIM_COMPLAINT_TYPE-01</v>
-      </c>
-      <c r="B86" t="str">
-        <v>CLAIM_COMPLAINT_TYPE</v>
-      </c>
-      <c r="C86" t="str">
-        <v>CLAIM</v>
-      </c>
-      <c r="D86" t="str">
-        <v>Complaint Type</v>
-      </c>
-      <c r="E86" t="str">
-        <v>Transmission</v>
-      </c>
-      <c r="F86">
-        <v>1</v>
-      </c>
-      <c r="G86" t="str">
-        <v/>
-      </c>
-      <c r="H86" t="str">
-        <v/>
-      </c>
-      <c r="I86" t="str">
-        <v>Active</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="str">
-        <v>CLAIM_COMPLAINT_TYPE-02</v>
-      </c>
-      <c r="B87" t="str">
-        <v>CLAIM_COMPLAINT_TYPE</v>
-      </c>
-      <c r="C87" t="str">
-        <v>CLAIM</v>
-      </c>
-      <c r="D87" t="str">
-        <v>Complaint Type</v>
-      </c>
-      <c r="E87" t="str">
-        <v>Clutch</v>
-      </c>
-      <c r="F87">
-        <v>2</v>
-      </c>
-      <c r="G87" t="str">
-        <v/>
-      </c>
-      <c r="H87" t="str">
-        <v/>
-      </c>
-      <c r="I87" t="str">
-        <v>Active</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I87"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I83"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -26336,7 +26381,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -26398,7 +26443,7 @@
         <v>Steering shudder or brake pedal vibration on deceleration</v>
       </c>
       <c r="E3" t="str">
-        <v>PV + EV</v>
+        <v>PV</v>
       </c>
       <c r="F3" t="str">
         <v>High</v>
@@ -26409,16 +26454,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CC-03</v>
+        <v>CC-02-EV</v>
       </c>
       <c r="B4" t="str">
-        <v>BAT-SOC-03</v>
+        <v>BRK-VIB-02</v>
       </c>
       <c r="C4" t="str">
-        <v>Electrical &amp; Battery</v>
+        <v>Brakes &amp; Suspension</v>
       </c>
       <c r="D4" t="str">
-        <v>Sudden drop in EV Battery SOC / Limited Performance turtle lamp</v>
+        <v>Steering shudder or brake pedal vibration on deceleration</v>
       </c>
       <c r="E4" t="str">
         <v>EV</v>
@@ -26432,22 +26477,22 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CC-04</v>
+        <v>CC-03</v>
       </c>
       <c r="B5" t="str">
-        <v>AC-COOL-04</v>
+        <v>BAT-SOC-03</v>
       </c>
       <c r="C5" t="str">
-        <v>HVAC &amp; AC</v>
+        <v>Electrical &amp; Battery</v>
       </c>
       <c r="D5" t="str">
-        <v>Insufficient cooling during idle or city traffic</v>
+        <v>Sudden drop in EV Battery SOC / Limited Performance turtle lamp</v>
       </c>
       <c r="E5" t="str">
-        <v>PV + EV</v>
+        <v>EV</v>
       </c>
       <c r="F5" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
       <c r="G5" t="str">
         <v>Y</v>
@@ -26455,30 +26500,99 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>CC-04</v>
+      </c>
+      <c r="B6" t="str">
+        <v>AC-COOL-04</v>
+      </c>
+      <c r="C6" t="str">
+        <v>HVAC &amp; AC</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Insufficient cooling during idle or city traffic</v>
+      </c>
+      <c r="E6" t="str">
+        <v>PV</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>CC-04-EV</v>
+      </c>
+      <c r="B7" t="str">
+        <v>AC-COOL-04</v>
+      </c>
+      <c r="C7" t="str">
+        <v>HVAC &amp; AC</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Insufficient cooling during idle or city traffic</v>
+      </c>
+      <c r="E7" t="str">
+        <v>EV</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>CC-05</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B8" t="str">
         <v>INFO-SCR-05</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C8" t="str">
         <v>Infotainment &amp; Connected</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D8" t="str">
         <v>Harman touchscreen blanking / Apple CarPlay disconnects</v>
       </c>
-      <c r="E6" t="str">
-        <v>PV + EV</v>
-      </c>
-      <c r="F6" t="str">
+      <c r="E8" t="str">
+        <v>PV</v>
+      </c>
+      <c r="F8" t="str">
         <v>Low</v>
       </c>
-      <c r="G6" t="str">
+      <c r="G8" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>CC-05-EV</v>
+      </c>
+      <c r="B9" t="str">
+        <v>INFO-SCR-05</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Infotainment &amp; Connected</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Harman touchscreen blanking / Apple CarPlay disconnects</v>
+      </c>
+      <c r="E9" t="str">
+        <v>EV</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G9" t="str">
         <v>Y</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
List of Values screen (Siebel style); remove CV as a BU
- Common LOV Master opens in a List of Values screen: LOV Types on the left (find, module filter),
  values grid on the right (Order arrows, Display Value, Code (LIC), Parent Value, Active, Description),
  New Value / Add several (paste one per line) / Copy, Save with cell-level errors, Undo changes,
  New LOV Type with the Parameter proposed as <MODULE>_<FIELD>; Table / Excel view kept for import/export
- Common LOV values get a Code (LIC) and Description; duplicate codes refused
- CV is not a BU: COMMON_BU = PV, EV; BU types, filters, sample bays and examples updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DwiSAaMRyjNA589tWt8iz
</commit_message>
<xml_diff>
--- a/docs/templates/TML_Existing_Masters_Catalogue.xlsx
+++ b/docs/templates/TML_Existing_Masters_Catalogue.xlsx
@@ -5539,7 +5539,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q300"/>
+  <dimension ref="A1:Q302"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5611,7 +5611,7 @@
         <v>Y</v>
       </c>
       <c r="F2" t="str">
-        <v>PV, EV, CV</v>
+        <v>PV, EV</v>
       </c>
       <c r="G2" t="str">
         <v/>
@@ -6777,7 +6777,7 @@
         <v>N</v>
       </c>
       <c r="F24" t="str">
-        <v>PV, EV, CV</v>
+        <v>PV, EV</v>
       </c>
       <c r="G24" t="str">
         <v/>
@@ -8208,7 +8208,7 @@
         <v>N</v>
       </c>
       <c r="F51" t="str">
-        <v>PV, EV, CV</v>
+        <v>PV, EV</v>
       </c>
       <c r="G51" t="str">
         <v/>
@@ -9162,7 +9162,7 @@
         <v>Y</v>
       </c>
       <c r="F69" t="str">
-        <v>PV, EV, CV</v>
+        <v>PV, EV</v>
       </c>
       <c r="G69" t="str">
         <v/>
@@ -11812,7 +11812,7 @@
         <v>Y</v>
       </c>
       <c r="F119" t="str">
-        <v>PV, EV, CV</v>
+        <v>PV, EV</v>
       </c>
       <c r="G119" t="str">
         <v/>
@@ -12395,7 +12395,7 @@
         <v>Y</v>
       </c>
       <c r="F130" t="str">
-        <v>PV, EV, CV</v>
+        <v>PV, EV</v>
       </c>
       <c r="G130" t="str">
         <v/>
@@ -12978,7 +12978,7 @@
         <v>Y</v>
       </c>
       <c r="F141" t="str">
-        <v>PV, EV, CV</v>
+        <v>PV, EV</v>
       </c>
       <c r="G141" t="str">
         <v/>
@@ -16582,7 +16582,7 @@
         <v>Y</v>
       </c>
       <c r="F209" t="str">
-        <v>PV, EV, CV</v>
+        <v>PV, EV</v>
       </c>
       <c r="G209" t="str">
         <v/>
@@ -16847,7 +16847,7 @@
         <v>Y</v>
       </c>
       <c r="F214" t="str">
-        <v>PV, EV, CV</v>
+        <v>PV, EV</v>
       </c>
       <c r="G214" t="str">
         <v/>
@@ -19550,7 +19550,7 @@
         <v>Y</v>
       </c>
       <c r="F265" t="str">
-        <v>PV, EV, CV</v>
+        <v>PV, EV</v>
       </c>
       <c r="G265" t="str">
         <v/>
@@ -21025,7 +21025,7 @@
         <v>lovCode</v>
       </c>
       <c r="C293" t="str">
-        <v>Parameter (LOV Code)</v>
+        <v>LOV Type (Parameter)</v>
       </c>
       <c r="D293" t="str">
         <v>text</v>
@@ -21184,7 +21184,7 @@
         <v>value</v>
       </c>
       <c r="C296" t="str">
-        <v>Value</v>
+        <v>Display Value</v>
       </c>
       <c r="D296" t="str">
         <v>text</v>
@@ -21226,7 +21226,7 @@
         <v/>
       </c>
       <c r="Q296" t="str">
-        <v/>
+        <v>What users see in the dropdown.</v>
       </c>
     </row>
     <row r="297">
@@ -21234,25 +21234,25 @@
         <v>common_lov</v>
       </c>
       <c r="B297" t="str">
-        <v>order</v>
+        <v>lic</v>
       </c>
       <c r="C297" t="str">
-        <v>Order</v>
+        <v>Code (LIC)</v>
       </c>
       <c r="D297" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="E297" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F297" t="str">
         <v/>
       </c>
-      <c r="G297">
-        <v>1</v>
-      </c>
-      <c r="H297">
-        <v>999</v>
+      <c r="G297" t="str">
+        <v/>
+      </c>
+      <c r="H297" t="str">
+        <v/>
       </c>
       <c r="I297" t="str">
         <v/>
@@ -21261,10 +21261,10 @@
         <v/>
       </c>
       <c r="K297" t="str">
-        <v/>
+        <v>^[A-Z0-9][A-Z0-9_]*$</v>
       </c>
       <c r="L297" t="str">
-        <v/>
+        <v>Capitals, digits and _ only, e.g. WORK_IN_PROCESS.</v>
       </c>
       <c r="M297" t="str">
         <v>N</v>
@@ -21279,7 +21279,7 @@
         <v/>
       </c>
       <c r="Q297" t="str">
-        <v>Position in the dropdown.</v>
+        <v>Language-independent code kept in records; stays the same when the Display Value wording changes.</v>
       </c>
     </row>
     <row r="298">
@@ -21287,25 +21287,25 @@
         <v>common_lov</v>
       </c>
       <c r="B298" t="str">
-        <v>parentLovCode</v>
+        <v>order</v>
       </c>
       <c r="C298" t="str">
-        <v>Parent LOV Code</v>
+        <v>Order</v>
       </c>
       <c r="D298" t="str">
-        <v>text</v>
+        <v>number</v>
       </c>
       <c r="E298" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F298" t="str">
         <v/>
       </c>
-      <c r="G298" t="str">
-        <v/>
-      </c>
-      <c r="H298" t="str">
-        <v/>
+      <c r="G298">
+        <v>1</v>
+      </c>
+      <c r="H298">
+        <v>999</v>
       </c>
       <c r="I298" t="str">
         <v/>
@@ -21332,7 +21332,7 @@
         <v/>
       </c>
       <c r="Q298" t="str">
-        <v>Dependent dropdowns only: the list this value depends on.</v>
+        <v>Position in the dropdown.</v>
       </c>
     </row>
     <row r="299">
@@ -21340,10 +21340,10 @@
         <v>common_lov</v>
       </c>
       <c r="B299" t="str">
-        <v>parentValue</v>
+        <v>parentLovCode</v>
       </c>
       <c r="C299" t="str">
-        <v>Parent Value</v>
+        <v>Parent LOV Code</v>
       </c>
       <c r="D299" t="str">
         <v>text</v>
@@ -21385,7 +21385,7 @@
         <v/>
       </c>
       <c r="Q299" t="str">
-        <v>Dependent dropdowns only: the parent list value that shows this value.</v>
+        <v>Dependent dropdowns only: the list this value depends on.</v>
       </c>
     </row>
     <row r="300">
@@ -21393,57 +21393,163 @@
         <v>common_lov</v>
       </c>
       <c r="B300" t="str">
+        <v>parentValue</v>
+      </c>
+      <c r="C300" t="str">
+        <v>Parent Value</v>
+      </c>
+      <c r="D300" t="str">
+        <v>text</v>
+      </c>
+      <c r="E300" t="str">
+        <v>N</v>
+      </c>
+      <c r="F300" t="str">
+        <v/>
+      </c>
+      <c r="G300" t="str">
+        <v/>
+      </c>
+      <c r="H300" t="str">
+        <v/>
+      </c>
+      <c r="I300" t="str">
+        <v/>
+      </c>
+      <c r="J300" t="str">
+        <v/>
+      </c>
+      <c r="K300" t="str">
+        <v/>
+      </c>
+      <c r="L300" t="str">
+        <v/>
+      </c>
+      <c r="M300" t="str">
+        <v>N</v>
+      </c>
+      <c r="N300" t="str">
+        <v/>
+      </c>
+      <c r="O300" t="str">
+        <v/>
+      </c>
+      <c r="P300" t="str">
+        <v/>
+      </c>
+      <c r="Q300" t="str">
+        <v>Dependent dropdowns only: the parent list value that shows this value.</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>common_lov</v>
+      </c>
+      <c r="B301" t="str">
+        <v>description</v>
+      </c>
+      <c r="C301" t="str">
+        <v>Description</v>
+      </c>
+      <c r="D301" t="str">
+        <v>text</v>
+      </c>
+      <c r="E301" t="str">
+        <v>N</v>
+      </c>
+      <c r="F301" t="str">
+        <v/>
+      </c>
+      <c r="G301" t="str">
+        <v/>
+      </c>
+      <c r="H301" t="str">
+        <v/>
+      </c>
+      <c r="I301" t="str">
+        <v/>
+      </c>
+      <c r="J301" t="str">
+        <v/>
+      </c>
+      <c r="K301" t="str">
+        <v/>
+      </c>
+      <c r="L301" t="str">
+        <v/>
+      </c>
+      <c r="M301" t="str">
+        <v>N</v>
+      </c>
+      <c r="N301" t="str">
+        <v/>
+      </c>
+      <c r="O301" t="str">
+        <v/>
+      </c>
+      <c r="P301" t="str">
+        <v/>
+      </c>
+      <c r="Q301" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>common_lov</v>
+      </c>
+      <c r="B302" t="str">
         <v>status</v>
       </c>
-      <c r="C300" t="str">
+      <c r="C302" t="str">
         <v>Status</v>
       </c>
-      <c r="D300" t="str">
+      <c r="D302" t="str">
         <v>select</v>
       </c>
-      <c r="E300" t="str">
-        <v>Y</v>
-      </c>
-      <c r="F300" t="str">
+      <c r="E302" t="str">
+        <v>Y</v>
+      </c>
+      <c r="F302" t="str">
         <v>Active, Inactive</v>
       </c>
-      <c r="G300" t="str">
-        <v/>
-      </c>
-      <c r="H300" t="str">
-        <v/>
-      </c>
-      <c r="I300" t="str">
-        <v/>
-      </c>
-      <c r="J300" t="str">
-        <v/>
-      </c>
-      <c r="K300" t="str">
-        <v/>
-      </c>
-      <c r="L300" t="str">
-        <v/>
-      </c>
-      <c r="M300" t="str">
-        <v>N</v>
-      </c>
-      <c r="N300" t="str">
-        <v/>
-      </c>
-      <c r="O300" t="str">
-        <v/>
-      </c>
-      <c r="P300" t="str">
-        <v/>
-      </c>
-      <c r="Q300" t="str">
+      <c r="G302" t="str">
+        <v/>
+      </c>
+      <c r="H302" t="str">
+        <v/>
+      </c>
+      <c r="I302" t="str">
+        <v/>
+      </c>
+      <c r="J302" t="str">
+        <v/>
+      </c>
+      <c r="K302" t="str">
+        <v/>
+      </c>
+      <c r="L302" t="str">
+        <v/>
+      </c>
+      <c r="M302" t="str">
+        <v>N</v>
+      </c>
+      <c r="N302" t="str">
+        <v/>
+      </c>
+      <c r="O302" t="str">
+        <v/>
+      </c>
+      <c r="P302" t="str">
+        <v/>
+      </c>
+      <c r="Q302" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q300"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q302"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -23648,7 +23754,7 @@
 
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:K82"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -23667,15 +23773,21 @@
         <v>value</v>
       </c>
       <c r="F1" t="str">
+        <v>lic</v>
+      </c>
+      <c r="G1" t="str">
         <v>order</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>parentLovCode</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>parentValue</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
+        <v>description</v>
+      </c>
+      <c r="K1" t="str">
         <v>status</v>
       </c>
     </row>
@@ -23695,16 +23807,22 @@
       <c r="E2" t="str">
         <v>PV</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="str">
+        <v>PV</v>
+      </c>
+      <c r="G2">
         <v>1</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
         <v>Active</v>
       </c>
     </row>
@@ -23724,51 +23842,63 @@
       <c r="E3" t="str">
         <v>EV</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="str">
+        <v>EV</v>
+      </c>
+      <c r="G3">
         <v>2</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>COMMON_BU-03</v>
+        <v>THD_PROGRESS-01</v>
       </c>
       <c r="B4" t="str">
-        <v>COMMON_BU</v>
+        <v>THD_PROGRESS</v>
       </c>
       <c r="C4" t="str">
-        <v>COMMON</v>
+        <v>THD</v>
       </c>
       <c r="D4" t="str">
-        <v>BU</v>
+        <v>Progress</v>
       </c>
       <c r="E4" t="str">
-        <v>CV</v>
-      </c>
-      <c r="F4">
-        <v>3</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
+        <v>Under Diagnosis</v>
+      </c>
+      <c r="F4" t="str">
+        <v>UNDER_DIAGNOSIS</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
       </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>THD_PROGRESS-01</v>
+        <v>THD_PROGRESS-02</v>
       </c>
       <c r="B5" t="str">
         <v>THD_PROGRESS</v>
@@ -23780,24 +23910,30 @@
         <v>Progress</v>
       </c>
       <c r="E5" t="str">
-        <v>Under Diagnosis</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
+        <v>Work in process</v>
+      </c>
+      <c r="F5" t="str">
+        <v>WORK_IN_PROCESS</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
       </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>THD_PROGRESS-02</v>
+        <v>THD_PROGRESS-03</v>
       </c>
       <c r="B6" t="str">
         <v>THD_PROGRESS</v>
@@ -23809,24 +23945,30 @@
         <v>Progress</v>
       </c>
       <c r="E6" t="str">
-        <v>Work in process</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="G6" t="str">
-        <v/>
+        <v>Pending for parts</v>
+      </c>
+      <c r="F6" t="str">
+        <v>PENDING_FOR_PARTS</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
       </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>THD_PROGRESS-03</v>
+        <v>THD_PROGRESS-04</v>
       </c>
       <c r="B7" t="str">
         <v>THD_PROGRESS</v>
@@ -23838,24 +23980,30 @@
         <v>Progress</v>
       </c>
       <c r="E7" t="str">
-        <v>Pending for parts</v>
-      </c>
-      <c r="F7">
-        <v>3</v>
-      </c>
-      <c r="G7" t="str">
-        <v/>
+        <v>Pending for vendor support</v>
+      </c>
+      <c r="F7" t="str">
+        <v>PENDING_FOR_VENDOR_SUPPORT</v>
+      </c>
+      <c r="G7">
+        <v>4</v>
       </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>THD_PROGRESS-04</v>
+        <v>THD_PROGRESS-05</v>
       </c>
       <c r="B8" t="str">
         <v>THD_PROGRESS</v>
@@ -23867,24 +24015,30 @@
         <v>Progress</v>
       </c>
       <c r="E8" t="str">
-        <v>Pending for vendor support</v>
-      </c>
-      <c r="F8">
-        <v>4</v>
-      </c>
-      <c r="G8" t="str">
-        <v/>
+        <v>Pending for commercial decision</v>
+      </c>
+      <c r="F8" t="str">
+        <v>PENDING_FOR_COMMERCIAL_DECISION</v>
+      </c>
+      <c r="G8">
+        <v>5</v>
       </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>THD_PROGRESS-05</v>
+        <v>THD_PROGRESS-06</v>
       </c>
       <c r="B9" t="str">
         <v>THD_PROGRESS</v>
@@ -23896,53 +24050,65 @@
         <v>Progress</v>
       </c>
       <c r="E9" t="str">
-        <v>Pending for commercial decision</v>
-      </c>
-      <c r="F9">
-        <v>5</v>
-      </c>
-      <c r="G9" t="str">
-        <v/>
+        <v>Pending for Vehicle availability</v>
+      </c>
+      <c r="F9" t="str">
+        <v>PENDING_FOR_VEHICLE_AVAILABILITY</v>
+      </c>
+      <c r="G9">
+        <v>6</v>
       </c>
       <c r="H9" t="str">
         <v/>
       </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>THD_PROGRESS-06</v>
+        <v>THD_PROGRESS_SUB_STATUS-01</v>
       </c>
       <c r="B10" t="str">
-        <v>THD_PROGRESS</v>
+        <v>THD_PROGRESS_SUB_STATUS</v>
       </c>
       <c r="C10" t="str">
         <v>THD</v>
       </c>
       <c r="D10" t="str">
-        <v>Progress</v>
+        <v>Progress Sub Status</v>
       </c>
       <c r="E10" t="str">
-        <v>Pending for Vehicle availability</v>
-      </c>
-      <c r="F10">
-        <v>6</v>
-      </c>
-      <c r="G10" t="str">
-        <v/>
+        <v>U/I DET</v>
+      </c>
+      <c r="F10" t="str">
+        <v>U_I_DET</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>THD_PROGRESS</v>
       </c>
       <c r="I10" t="str">
+        <v>Under Diagnosis</v>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-01</v>
+        <v>THD_PROGRESS_SUB_STATUS-02</v>
       </c>
       <c r="B11" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -23954,24 +24120,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E11" t="str">
-        <v>U/I DET</v>
-      </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11" t="str">
+        <v>U/I COC</v>
+      </c>
+      <c r="F11" t="str">
+        <v>U_I_COC</v>
+      </c>
+      <c r="G11">
+        <v>2</v>
+      </c>
+      <c r="H11" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
         <v>Under Diagnosis</v>
       </c>
-      <c r="I11" t="str">
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-02</v>
+        <v>THD_PROGRESS_SUB_STATUS-03</v>
       </c>
       <c r="B12" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -23983,24 +24155,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E12" t="str">
-        <v>U/I COC</v>
-      </c>
-      <c r="F12">
-        <v>2</v>
-      </c>
-      <c r="G12" t="str">
+        <v>U/I Vendor</v>
+      </c>
+      <c r="F12" t="str">
+        <v>U_I_VENDOR</v>
+      </c>
+      <c r="G12">
+        <v>3</v>
+      </c>
+      <c r="H12" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H12" t="str">
+      <c r="I12" t="str">
         <v>Under Diagnosis</v>
       </c>
-      <c r="I12" t="str">
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-03</v>
+        <v>THD_PROGRESS_SUB_STATUS-04</v>
       </c>
       <c r="B13" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24012,24 +24190,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E13" t="str">
-        <v>U/I Vendor</v>
-      </c>
-      <c r="F13">
-        <v>3</v>
-      </c>
-      <c r="G13" t="str">
+        <v>U/I Plant Team</v>
+      </c>
+      <c r="F13" t="str">
+        <v>U_I_PLANT_TEAM</v>
+      </c>
+      <c r="G13">
+        <v>4</v>
+      </c>
+      <c r="H13" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H13" t="str">
+      <c r="I13" t="str">
         <v>Under Diagnosis</v>
       </c>
-      <c r="I13" t="str">
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-04</v>
+        <v>THD_PROGRESS_SUB_STATUS-05</v>
       </c>
       <c r="B14" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24041,24 +24225,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E14" t="str">
-        <v>U/I Plant Team</v>
-      </c>
-      <c r="F14">
-        <v>4</v>
-      </c>
-      <c r="G14" t="str">
+        <v>WIP DET</v>
+      </c>
+      <c r="F14" t="str">
+        <v>WIP_DET</v>
+      </c>
+      <c r="G14">
+        <v>5</v>
+      </c>
+      <c r="H14" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H14" t="str">
-        <v>Under Diagnosis</v>
-      </c>
       <c r="I14" t="str">
+        <v>Work in process</v>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-05</v>
+        <v>THD_PROGRESS_SUB_STATUS-06</v>
       </c>
       <c r="B15" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24070,24 +24260,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E15" t="str">
-        <v>WIP DET</v>
-      </c>
-      <c r="F15">
-        <v>5</v>
-      </c>
-      <c r="G15" t="str">
+        <v>WIP W/S Team</v>
+      </c>
+      <c r="F15" t="str">
+        <v>WIP_W_S_TEAM</v>
+      </c>
+      <c r="G15">
+        <v>6</v>
+      </c>
+      <c r="H15" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H15" t="str">
+      <c r="I15" t="str">
         <v>Work in process</v>
       </c>
-      <c r="I15" t="str">
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-06</v>
+        <v>THD_PROGRESS_SUB_STATUS-07</v>
       </c>
       <c r="B16" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24099,24 +24295,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E16" t="str">
-        <v>WIP W/S Team</v>
-      </c>
-      <c r="F16">
-        <v>6</v>
-      </c>
-      <c r="G16" t="str">
+        <v>WIP Vendor</v>
+      </c>
+      <c r="F16" t="str">
+        <v>WIP_VENDOR</v>
+      </c>
+      <c r="G16">
+        <v>7</v>
+      </c>
+      <c r="H16" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H16" t="str">
+      <c r="I16" t="str">
         <v>Work in process</v>
       </c>
-      <c r="I16" t="str">
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-07</v>
+        <v>THD_PROGRESS_SUB_STATUS-08</v>
       </c>
       <c r="B17" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24128,24 +24330,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E17" t="str">
-        <v>WIP Vendor</v>
-      </c>
-      <c r="F17">
-        <v>7</v>
-      </c>
-      <c r="G17" t="str">
+        <v>Order status</v>
+      </c>
+      <c r="F17" t="str">
+        <v>ORDER_STATUS</v>
+      </c>
+      <c r="G17">
+        <v>8</v>
+      </c>
+      <c r="H17" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H17" t="str">
-        <v>Work in process</v>
-      </c>
       <c r="I17" t="str">
+        <v>Pending for parts</v>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-08</v>
+        <v>THD_PROGRESS_SUB_STATUS-09</v>
       </c>
       <c r="B18" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24157,24 +24365,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E18" t="str">
-        <v>Order status</v>
-      </c>
-      <c r="F18">
-        <v>8</v>
-      </c>
-      <c r="G18" t="str">
+        <v>Part receipt status</v>
+      </c>
+      <c r="F18" t="str">
+        <v>PART_RECEIPT_STATUS</v>
+      </c>
+      <c r="G18">
+        <v>9</v>
+      </c>
+      <c r="H18" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H18" t="str">
+      <c r="I18" t="str">
         <v>Pending for parts</v>
       </c>
-      <c r="I18" t="str">
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-09</v>
+        <v>THD_PROGRESS_SUB_STATUS-10</v>
       </c>
       <c r="B19" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24186,24 +24400,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E19" t="str">
-        <v>Part receipt status</v>
-      </c>
-      <c r="F19">
-        <v>9</v>
-      </c>
-      <c r="G19" t="str">
+        <v>Vendor details</v>
+      </c>
+      <c r="F19" t="str">
+        <v>VENDOR_DETAILS</v>
+      </c>
+      <c r="G19">
+        <v>10</v>
+      </c>
+      <c r="H19" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H19" t="str">
-        <v>Pending for parts</v>
-      </c>
       <c r="I19" t="str">
+        <v>Pending for vendor support</v>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-10</v>
+        <v>THD_PROGRESS_SUB_STATUS-11</v>
       </c>
       <c r="B20" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24215,24 +24435,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E20" t="str">
-        <v>Vendor details</v>
-      </c>
-      <c r="F20">
-        <v>10</v>
-      </c>
-      <c r="G20" t="str">
+        <v>Request raised</v>
+      </c>
+      <c r="F20" t="str">
+        <v>REQUEST_RAISED</v>
+      </c>
+      <c r="G20">
+        <v>11</v>
+      </c>
+      <c r="H20" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H20" t="str">
+      <c r="I20" t="str">
         <v>Pending for vendor support</v>
       </c>
-      <c r="I20" t="str">
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-11</v>
+        <v>THD_PROGRESS_SUB_STATUS-12</v>
       </c>
       <c r="B21" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24244,24 +24470,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E21" t="str">
-        <v>Request raised</v>
-      </c>
-      <c r="F21">
-        <v>11</v>
-      </c>
-      <c r="G21" t="str">
+        <v>Status</v>
+      </c>
+      <c r="F21" t="str">
+        <v>STATUS</v>
+      </c>
+      <c r="G21">
+        <v>12</v>
+      </c>
+      <c r="H21" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H21" t="str">
+      <c r="I21" t="str">
         <v>Pending for vendor support</v>
       </c>
-      <c r="I21" t="str">
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-12</v>
+        <v>THD_PROGRESS_SUB_STATUS-13</v>
       </c>
       <c r="B22" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24273,24 +24505,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E22" t="str">
-        <v>Status</v>
-      </c>
-      <c r="F22">
-        <v>12</v>
-      </c>
-      <c r="G22" t="str">
+        <v>Pending for approval</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PENDING_FOR_APPROVAL</v>
+      </c>
+      <c r="G22">
+        <v>13</v>
+      </c>
+      <c r="H22" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H22" t="str">
-        <v>Pending for vendor support</v>
-      </c>
       <c r="I22" t="str">
+        <v>Pending for commercial decision</v>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-13</v>
+        <v>THD_PROGRESS_SUB_STATUS-14</v>
       </c>
       <c r="B23" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24302,24 +24540,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E23" t="str">
-        <v>Pending for approval</v>
-      </c>
-      <c r="F23">
-        <v>13</v>
-      </c>
-      <c r="G23" t="str">
+        <v>Approval received</v>
+      </c>
+      <c r="F23" t="str">
+        <v>APPROVAL_RECEIVED</v>
+      </c>
+      <c r="G23">
+        <v>14</v>
+      </c>
+      <c r="H23" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H23" t="str">
+      <c r="I23" t="str">
         <v>Pending for commercial decision</v>
       </c>
-      <c r="I23" t="str">
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-14</v>
+        <v>THD_PROGRESS_SUB_STATUS-15</v>
       </c>
       <c r="B24" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24331,24 +24575,30 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E24" t="str">
-        <v>Approval received</v>
-      </c>
-      <c r="F24">
-        <v>14</v>
-      </c>
-      <c r="G24" t="str">
+        <v>Expected date</v>
+      </c>
+      <c r="F24" t="str">
+        <v>EXPECTED_DATE</v>
+      </c>
+      <c r="G24">
+        <v>15</v>
+      </c>
+      <c r="H24" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H24" t="str">
-        <v>Pending for commercial decision</v>
-      </c>
       <c r="I24" t="str">
+        <v>Pending for Vehicle availability</v>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-15</v>
+        <v>THD_PROGRESS_SUB_STATUS-16</v>
       </c>
       <c r="B25" t="str">
         <v>THD_PROGRESS_SUB_STATUS</v>
@@ -24360,53 +24610,65 @@
         <v>Progress Sub Status</v>
       </c>
       <c r="E25" t="str">
-        <v>Expected date</v>
-      </c>
-      <c r="F25">
-        <v>15</v>
-      </c>
-      <c r="G25" t="str">
+        <v>Status as on date</v>
+      </c>
+      <c r="F25" t="str">
+        <v>STATUS_AS_ON_DATE</v>
+      </c>
+      <c r="G25">
+        <v>16</v>
+      </c>
+      <c r="H25" t="str">
         <v>THD_PROGRESS</v>
       </c>
-      <c r="H25" t="str">
+      <c r="I25" t="str">
         <v>Pending for Vehicle availability</v>
       </c>
-      <c r="I25" t="str">
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>THD_PROGRESS_SUB_STATUS-16</v>
+        <v>THD_COMPLAINT_TYPE-01</v>
       </c>
       <c r="B26" t="str">
-        <v>THD_PROGRESS_SUB_STATUS</v>
+        <v>THD_COMPLAINT_TYPE</v>
       </c>
       <c r="C26" t="str">
         <v>THD</v>
       </c>
       <c r="D26" t="str">
-        <v>Progress Sub Status</v>
+        <v>Type of Complaint</v>
       </c>
       <c r="E26" t="str">
-        <v>Status as on date</v>
-      </c>
-      <c r="F26">
-        <v>16</v>
-      </c>
-      <c r="G26" t="str">
-        <v>THD_PROGRESS</v>
+        <v>Technical Query</v>
+      </c>
+      <c r="F26" t="str">
+        <v>TECHNICAL_QUERY</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
       </c>
       <c r="H26" t="str">
-        <v>Pending for Vehicle availability</v>
+        <v/>
       </c>
       <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>THD_COMPLAINT_TYPE-01</v>
+        <v>THD_COMPLAINT_TYPE-02</v>
       </c>
       <c r="B27" t="str">
         <v>THD_COMPLAINT_TYPE</v>
@@ -24418,53 +24680,65 @@
         <v>Type of Complaint</v>
       </c>
       <c r="E27" t="str">
-        <v>Technical Query</v>
-      </c>
-      <c r="F27">
-        <v>1</v>
-      </c>
-      <c r="G27" t="str">
-        <v/>
+        <v>Technical Support</v>
+      </c>
+      <c r="F27" t="str">
+        <v>TECHNICAL_SUPPORT</v>
+      </c>
+      <c r="G27">
+        <v>2</v>
       </c>
       <c r="H27" t="str">
         <v/>
       </c>
       <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>THD_COMPLAINT_TYPE-02</v>
+        <v>THD_COMPLAINT_SHORT_DESC-01</v>
       </c>
       <c r="B28" t="str">
-        <v>THD_COMPLAINT_TYPE</v>
+        <v>THD_COMPLAINT_SHORT_DESC</v>
       </c>
       <c r="C28" t="str">
         <v>THD</v>
       </c>
       <c r="D28" t="str">
-        <v>Type of Complaint</v>
+        <v>Complaint Short Description</v>
       </c>
       <c r="E28" t="str">
-        <v>Technical Support</v>
-      </c>
-      <c r="F28">
-        <v>2</v>
-      </c>
-      <c r="G28" t="str">
-        <v/>
+        <v>Abnormal noise</v>
+      </c>
+      <c r="F28" t="str">
+        <v>ABNORMAL_NOISE</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
       </c>
       <c r="H28" t="str">
         <v/>
       </c>
       <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-01</v>
+        <v>THD_COMPLAINT_SHORT_DESC-02</v>
       </c>
       <c r="B29" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24476,24 +24750,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E29" t="str">
-        <v>Abnormal noise</v>
-      </c>
-      <c r="F29">
-        <v>1</v>
-      </c>
-      <c r="G29" t="str">
-        <v/>
+        <v>Warning lamps ON</v>
+      </c>
+      <c r="F29" t="str">
+        <v>WARNING_LAMPS_ON</v>
+      </c>
+      <c r="G29">
+        <v>2</v>
       </c>
       <c r="H29" t="str">
         <v/>
       </c>
       <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-02</v>
+        <v>THD_COMPLAINT_SHORT_DESC-03</v>
       </c>
       <c r="B30" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24505,24 +24785,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E30" t="str">
-        <v>Warning lamps ON</v>
-      </c>
-      <c r="F30">
-        <v>2</v>
-      </c>
-      <c r="G30" t="str">
-        <v/>
+        <v>Oil leakage</v>
+      </c>
+      <c r="F30" t="str">
+        <v>OIL_LEAKAGE</v>
+      </c>
+      <c r="G30">
+        <v>3</v>
       </c>
       <c r="H30" t="str">
         <v/>
       </c>
       <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-03</v>
+        <v>THD_COMPLAINT_SHORT_DESC-04</v>
       </c>
       <c r="B31" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24534,24 +24820,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E31" t="str">
-        <v>Oil leakage</v>
-      </c>
-      <c r="F31">
-        <v>3</v>
-      </c>
-      <c r="G31" t="str">
-        <v/>
+        <v>Coolant leakage</v>
+      </c>
+      <c r="F31" t="str">
+        <v>COOLANT_LEAKAGE</v>
+      </c>
+      <c r="G31">
+        <v>4</v>
       </c>
       <c r="H31" t="str">
         <v/>
       </c>
       <c r="I31" t="str">
+        <v/>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-04</v>
+        <v>THD_COMPLAINT_SHORT_DESC-05</v>
       </c>
       <c r="B32" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24563,24 +24855,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E32" t="str">
-        <v>Coolant leakage</v>
-      </c>
-      <c r="F32">
-        <v>4</v>
-      </c>
-      <c r="G32" t="str">
-        <v/>
+        <v>Engine overheating</v>
+      </c>
+      <c r="F32" t="str">
+        <v>ENGINE_OVERHEATING</v>
+      </c>
+      <c r="G32">
+        <v>5</v>
       </c>
       <c r="H32" t="str">
         <v/>
       </c>
       <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-05</v>
+        <v>THD_COMPLAINT_SHORT_DESC-06</v>
       </c>
       <c r="B33" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24592,24 +24890,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E33" t="str">
-        <v>Engine overheating</v>
-      </c>
-      <c r="F33">
-        <v>5</v>
-      </c>
-      <c r="G33" t="str">
-        <v/>
+        <v>Smell – burning, fuel, foul odor from outside, etc.</v>
+      </c>
+      <c r="F33" t="str">
+        <v>SMELL_BURNING_FUEL_FOUL_ODOR_FROM_OUTSID</v>
+      </c>
+      <c r="G33">
+        <v>6</v>
       </c>
       <c r="H33" t="str">
         <v/>
       </c>
       <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-06</v>
+        <v>THD_COMPLAINT_SHORT_DESC-07</v>
       </c>
       <c r="B34" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24621,24 +24925,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E34" t="str">
-        <v>Smell – burning, fuel, foul odor from outside, etc.</v>
-      </c>
-      <c r="F34">
-        <v>6</v>
-      </c>
-      <c r="G34" t="str">
-        <v/>
+        <v>Smoke issues</v>
+      </c>
+      <c r="F34" t="str">
+        <v>SMOKE_ISSUES</v>
+      </c>
+      <c r="G34">
+        <v>7</v>
       </c>
       <c r="H34" t="str">
         <v/>
       </c>
       <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-07</v>
+        <v>THD_COMPLAINT_SHORT_DESC-08</v>
       </c>
       <c r="B35" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24650,24 +24960,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E35" t="str">
-        <v>Smoke issues</v>
-      </c>
-      <c r="F35">
-        <v>7</v>
-      </c>
-      <c r="G35" t="str">
-        <v/>
+        <v>Oil-Coolant mix</v>
+      </c>
+      <c r="F35" t="str">
+        <v>OIL_COOLANT_MIX</v>
+      </c>
+      <c r="G35">
+        <v>8</v>
       </c>
       <c r="H35" t="str">
         <v/>
       </c>
       <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-08</v>
+        <v>THD_COMPLAINT_SHORT_DESC-09</v>
       </c>
       <c r="B36" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24679,24 +24995,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E36" t="str">
-        <v>Oil-Coolant mix</v>
-      </c>
-      <c r="F36">
-        <v>8</v>
-      </c>
-      <c r="G36" t="str">
-        <v/>
+        <v>Gear shifting issues</v>
+      </c>
+      <c r="F36" t="str">
+        <v>GEAR_SHIFTING_ISSUES</v>
+      </c>
+      <c r="G36">
+        <v>9</v>
       </c>
       <c r="H36" t="str">
         <v/>
       </c>
       <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-09</v>
+        <v>THD_COMPLAINT_SHORT_DESC-10</v>
       </c>
       <c r="B37" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24708,24 +25030,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E37" t="str">
-        <v>Gear shifting issues</v>
-      </c>
-      <c r="F37">
-        <v>9</v>
-      </c>
-      <c r="G37" t="str">
-        <v/>
+        <v>AC cooling issues</v>
+      </c>
+      <c r="F37" t="str">
+        <v>AC_COOLING_ISSUES</v>
+      </c>
+      <c r="G37">
+        <v>10</v>
       </c>
       <c r="H37" t="str">
         <v/>
       </c>
       <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-10</v>
+        <v>THD_COMPLAINT_SHORT_DESC-11</v>
       </c>
       <c r="B38" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24737,24 +25065,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E38" t="str">
-        <v>AC cooling issues</v>
-      </c>
-      <c r="F38">
-        <v>10</v>
-      </c>
-      <c r="G38" t="str">
-        <v/>
+        <v>Jerking / vibration / misfiring</v>
+      </c>
+      <c r="F38" t="str">
+        <v>JERKING_VIBRATION_MISFIRING</v>
+      </c>
+      <c r="G38">
+        <v>11</v>
       </c>
       <c r="H38" t="str">
         <v/>
       </c>
       <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-11</v>
+        <v>THD_COMPLAINT_SHORT_DESC-12</v>
       </c>
       <c r="B39" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24766,24 +25100,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E39" t="str">
-        <v>Jerking / vibration / misfiring</v>
-      </c>
-      <c r="F39">
-        <v>11</v>
-      </c>
-      <c r="G39" t="str">
-        <v/>
+        <v>Steering hard</v>
+      </c>
+      <c r="F39" t="str">
+        <v>STEERING_HARD</v>
+      </c>
+      <c r="G39">
+        <v>12</v>
       </c>
       <c r="H39" t="str">
         <v/>
       </c>
       <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-12</v>
+        <v>THD_COMPLAINT_SHORT_DESC-13</v>
       </c>
       <c r="B40" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24795,24 +25135,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E40" t="str">
-        <v>Steering hard</v>
-      </c>
-      <c r="F40">
-        <v>12</v>
-      </c>
-      <c r="G40" t="str">
-        <v/>
+        <v>Vehicle pulling</v>
+      </c>
+      <c r="F40" t="str">
+        <v>VEHICLE_PULLING</v>
+      </c>
+      <c r="G40">
+        <v>13</v>
       </c>
       <c r="H40" t="str">
         <v/>
       </c>
       <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+      <c r="K40" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-13</v>
+        <v>THD_COMPLAINT_SHORT_DESC-14</v>
       </c>
       <c r="B41" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24824,24 +25170,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E41" t="str">
-        <v>Vehicle pulling</v>
-      </c>
-      <c r="F41">
-        <v>13</v>
-      </c>
-      <c r="G41" t="str">
-        <v/>
+        <v>Starting problem</v>
+      </c>
+      <c r="F41" t="str">
+        <v>STARTING_PROBLEM</v>
+      </c>
+      <c r="G41">
+        <v>14</v>
       </c>
       <c r="H41" t="str">
         <v/>
       </c>
       <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
+      <c r="K41" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-14</v>
+        <v>THD_COMPLAINT_SHORT_DESC-15</v>
       </c>
       <c r="B42" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24853,24 +25205,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E42" t="str">
-        <v>Starting problem</v>
-      </c>
-      <c r="F42">
-        <v>14</v>
-      </c>
-      <c r="G42" t="str">
-        <v/>
+        <v>Tyre wear / cut</v>
+      </c>
+      <c r="F42" t="str">
+        <v>TYRE_WEAR_CUT</v>
+      </c>
+      <c r="G42">
+        <v>15</v>
       </c>
       <c r="H42" t="str">
         <v/>
       </c>
       <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-15</v>
+        <v>THD_COMPLAINT_SHORT_DESC-16</v>
       </c>
       <c r="B43" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24882,24 +25240,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E43" t="str">
-        <v>Tyre wear / cut</v>
-      </c>
-      <c r="F43">
-        <v>15</v>
-      </c>
-      <c r="G43" t="str">
-        <v/>
+        <v>Damaged / broken / cracked / soiled</v>
+      </c>
+      <c r="F43" t="str">
+        <v>DAMAGED_BROKEN_CRACKED_SOILED</v>
+      </c>
+      <c r="G43">
+        <v>16</v>
       </c>
       <c r="H43" t="str">
         <v/>
       </c>
       <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-16</v>
+        <v>THD_COMPLAINT_SHORT_DESC-17</v>
       </c>
       <c r="B44" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24911,24 +25275,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E44" t="str">
-        <v>Damaged / broken / cracked / soiled</v>
-      </c>
-      <c r="F44">
-        <v>16</v>
-      </c>
-      <c r="G44" t="str">
-        <v/>
+        <v>Part missing / fallen-off</v>
+      </c>
+      <c r="F44" t="str">
+        <v>PART_MISSING_FALLEN_OFF</v>
+      </c>
+      <c r="G44">
+        <v>17</v>
       </c>
       <c r="H44" t="str">
         <v/>
       </c>
       <c r="I44" t="str">
+        <v/>
+      </c>
+      <c r="J44" t="str">
+        <v/>
+      </c>
+      <c r="K44" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-17</v>
+        <v>THD_COMPLAINT_SHORT_DESC-18</v>
       </c>
       <c r="B45" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24940,24 +25310,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E45" t="str">
-        <v>Part missing / fallen-off</v>
-      </c>
-      <c r="F45">
-        <v>17</v>
-      </c>
-      <c r="G45" t="str">
-        <v/>
+        <v>Uneven gaps / flushness issues</v>
+      </c>
+      <c r="F45" t="str">
+        <v>UNEVEN_GAPS_FLUSHNESS_ISSUES</v>
+      </c>
+      <c r="G45">
+        <v>18</v>
       </c>
       <c r="H45" t="str">
         <v/>
       </c>
       <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
+      <c r="K45" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-18</v>
+        <v>THD_COMPLAINT_SHORT_DESC-19</v>
       </c>
       <c r="B46" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24969,24 +25345,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E46" t="str">
-        <v>Uneven gaps / flushness issues</v>
-      </c>
-      <c r="F46">
-        <v>18</v>
-      </c>
-      <c r="G46" t="str">
-        <v/>
+        <v>Paint / rust issues</v>
+      </c>
+      <c r="F46" t="str">
+        <v>PAINT_RUST_ISSUES</v>
+      </c>
+      <c r="G46">
+        <v>19</v>
       </c>
       <c r="H46" t="str">
         <v/>
       </c>
       <c r="I46" t="str">
+        <v/>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+      <c r="K46" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-19</v>
+        <v>THD_COMPLAINT_SHORT_DESC-20</v>
       </c>
       <c r="B47" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -24998,24 +25380,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E47" t="str">
-        <v>Paint / rust issues</v>
-      </c>
-      <c r="F47">
-        <v>19</v>
-      </c>
-      <c r="G47" t="str">
-        <v/>
+        <v>Not working / functioning issues / system malfunction</v>
+      </c>
+      <c r="F47" t="str">
+        <v>NOT_WORKING_FUNCTIONING_ISSUES_SYSTEM_MA</v>
+      </c>
+      <c r="G47">
+        <v>20</v>
       </c>
       <c r="H47" t="str">
         <v/>
       </c>
       <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+      <c r="K47" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-20</v>
+        <v>THD_COMPLAINT_SHORT_DESC-21</v>
       </c>
       <c r="B48" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -25027,24 +25415,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E48" t="str">
-        <v>Not working / functioning issues / system malfunction</v>
-      </c>
-      <c r="F48">
-        <v>20</v>
-      </c>
-      <c r="G48" t="str">
-        <v/>
+        <v>Crash / airbag related issues</v>
+      </c>
+      <c r="F48" t="str">
+        <v>CRASH_AIRBAG_RELATED_ISSUES</v>
+      </c>
+      <c r="G48">
+        <v>21</v>
       </c>
       <c r="H48" t="str">
         <v/>
       </c>
       <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
+      <c r="K48" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-21</v>
+        <v>THD_COMPLAINT_SHORT_DESC-22</v>
       </c>
       <c r="B49" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -25056,24 +25450,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E49" t="str">
-        <v>Crash / airbag related issues</v>
-      </c>
-      <c r="F49">
-        <v>21</v>
-      </c>
-      <c r="G49" t="str">
-        <v/>
+        <v>Thermal issues</v>
+      </c>
+      <c r="F49" t="str">
+        <v>THERMAL_ISSUES</v>
+      </c>
+      <c r="G49">
+        <v>22</v>
       </c>
       <c r="H49" t="str">
         <v/>
       </c>
       <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+      <c r="K49" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-22</v>
+        <v>THD_COMPLAINT_SHORT_DESC-23</v>
       </c>
       <c r="B50" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -25085,24 +25485,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E50" t="str">
-        <v>Thermal issues</v>
-      </c>
-      <c r="F50">
-        <v>22</v>
-      </c>
-      <c r="G50" t="str">
-        <v/>
+        <v>Brake ineffective</v>
+      </c>
+      <c r="F50" t="str">
+        <v>BRAKE_INEFFECTIVE</v>
+      </c>
+      <c r="G50">
+        <v>23</v>
       </c>
       <c r="H50" t="str">
         <v/>
       </c>
       <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+      <c r="K50" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-23</v>
+        <v>THD_COMPLAINT_SHORT_DESC-24</v>
       </c>
       <c r="B51" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -25114,24 +25520,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E51" t="str">
-        <v>Brake ineffective</v>
-      </c>
-      <c r="F51">
-        <v>23</v>
-      </c>
-      <c r="G51" t="str">
-        <v/>
+        <v>Poor pick-up</v>
+      </c>
+      <c r="F51" t="str">
+        <v>POOR_PICK_UP</v>
+      </c>
+      <c r="G51">
+        <v>24</v>
       </c>
       <c r="H51" t="str">
         <v/>
       </c>
       <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+      <c r="K51" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-24</v>
+        <v>THD_COMPLAINT_SHORT_DESC-25</v>
       </c>
       <c r="B52" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -25143,24 +25555,30 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E52" t="str">
-        <v>Poor pick-up</v>
-      </c>
-      <c r="F52">
-        <v>24</v>
-      </c>
-      <c r="G52" t="str">
-        <v/>
+        <v>Infotainment system issues</v>
+      </c>
+      <c r="F52" t="str">
+        <v>INFOTAINMENT_SYSTEM_ISSUES</v>
+      </c>
+      <c r="G52">
+        <v>25</v>
       </c>
       <c r="H52" t="str">
         <v/>
       </c>
       <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+      <c r="K52" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-25</v>
+        <v>THD_COMPLAINT_SHORT_DESC-26</v>
       </c>
       <c r="B53" t="str">
         <v>THD_COMPLAINT_SHORT_DESC</v>
@@ -25172,53 +25590,65 @@
         <v>Complaint Short Description</v>
       </c>
       <c r="E53" t="str">
-        <v>Infotainment system issues</v>
-      </c>
-      <c r="F53">
-        <v>25</v>
-      </c>
-      <c r="G53" t="str">
-        <v/>
+        <v>Water entry in cabin</v>
+      </c>
+      <c r="F53" t="str">
+        <v>WATER_ENTRY_IN_CABIN</v>
+      </c>
+      <c r="G53">
+        <v>26</v>
       </c>
       <c r="H53" t="str">
         <v/>
       </c>
       <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+      <c r="K53" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC-26</v>
+        <v>THD_ACTION_TAKEN-01</v>
       </c>
       <c r="B54" t="str">
-        <v>THD_COMPLAINT_SHORT_DESC</v>
+        <v>THD_ACTION_TAKEN</v>
       </c>
       <c r="C54" t="str">
         <v>THD</v>
       </c>
       <c r="D54" t="str">
-        <v>Complaint Short Description</v>
+        <v>Action Taken</v>
       </c>
       <c r="E54" t="str">
-        <v>Water entry in cabin</v>
-      </c>
-      <c r="F54">
-        <v>26</v>
-      </c>
-      <c r="G54" t="str">
-        <v/>
+        <v>Issue concluded and proceeded as per Field Investigation</v>
+      </c>
+      <c r="F54" t="str">
+        <v>ISSUE_CONCLUDED_AND_PROCEEDED_AS_PER_FIE</v>
+      </c>
+      <c r="G54">
+        <v>1</v>
       </c>
       <c r="H54" t="str">
         <v/>
       </c>
       <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+      <c r="K54" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>THD_ACTION_TAKEN-01</v>
+        <v>THD_ACTION_TAKEN-02</v>
       </c>
       <c r="B55" t="str">
         <v>THD_ACTION_TAKEN</v>
@@ -25230,24 +25660,30 @@
         <v>Action Taken</v>
       </c>
       <c r="E55" t="str">
-        <v>Issue concluded and proceeded as per Field Investigation</v>
-      </c>
-      <c r="F55">
-        <v>1</v>
-      </c>
-      <c r="G55" t="str">
-        <v/>
+        <v>Suggested checks based on observations</v>
+      </c>
+      <c r="F55" t="str">
+        <v>SUGGESTED_CHECKS_BASED_ON_OBSERVATIONS</v>
+      </c>
+      <c r="G55">
+        <v>2</v>
       </c>
       <c r="H55" t="str">
         <v/>
       </c>
       <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+      <c r="K55" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>THD_ACTION_TAKEN-02</v>
+        <v>THD_ACTION_TAKEN-03</v>
       </c>
       <c r="B56" t="str">
         <v>THD_ACTION_TAKEN</v>
@@ -25259,24 +25695,30 @@
         <v>Action Taken</v>
       </c>
       <c r="E56" t="str">
-        <v>Suggested checks based on observations</v>
-      </c>
-      <c r="F56">
-        <v>2</v>
-      </c>
-      <c r="G56" t="str">
-        <v/>
+        <v>Known issue – suggested part replacement</v>
+      </c>
+      <c r="F56" t="str">
+        <v>KNOWN_ISSUE_SUGGESTED_PART_REPLACEMENT</v>
+      </c>
+      <c r="G56">
+        <v>3</v>
       </c>
       <c r="H56" t="str">
         <v/>
       </c>
       <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+      <c r="K56" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>THD_ACTION_TAKEN-03</v>
+        <v>THD_ACTION_TAKEN-04</v>
       </c>
       <c r="B57" t="str">
         <v>THD_ACTION_TAKEN</v>
@@ -25288,24 +25730,30 @@
         <v>Action Taken</v>
       </c>
       <c r="E57" t="str">
-        <v>Known issue – suggested part replacement</v>
-      </c>
-      <c r="F57">
-        <v>3</v>
-      </c>
-      <c r="G57" t="str">
-        <v/>
+        <v>Updated software / parameterization</v>
+      </c>
+      <c r="F57" t="str">
+        <v>UPDATED_SOFTWARE_PARAMETERIZATION</v>
+      </c>
+      <c r="G57">
+        <v>4</v>
       </c>
       <c r="H57" t="str">
         <v/>
       </c>
       <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+      <c r="K57" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>THD_ACTION_TAKEN-04</v>
+        <v>THD_ACTION_TAKEN-05</v>
       </c>
       <c r="B58" t="str">
         <v>THD_ACTION_TAKEN</v>
@@ -25317,24 +25765,30 @@
         <v>Action Taken</v>
       </c>
       <c r="E58" t="str">
-        <v>Updated software / parameterization</v>
-      </c>
-      <c r="F58">
-        <v>4</v>
-      </c>
-      <c r="G58" t="str">
-        <v/>
+        <v>Suggested part replacement based on observation</v>
+      </c>
+      <c r="F58" t="str">
+        <v>SUGGESTED_PART_REPLACEMENT_BASED_ON_OBSE</v>
+      </c>
+      <c r="G58">
+        <v>5</v>
       </c>
       <c r="H58" t="str">
         <v/>
       </c>
       <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
+      <c r="K58" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>THD_ACTION_TAKEN-05</v>
+        <v>THD_ACTION_TAKEN-06</v>
       </c>
       <c r="B59" t="str">
         <v>THD_ACTION_TAKEN</v>
@@ -25346,24 +25800,30 @@
         <v>Action Taken</v>
       </c>
       <c r="E59" t="str">
-        <v>Suggested part replacement based on observation</v>
-      </c>
-      <c r="F59">
-        <v>5</v>
-      </c>
-      <c r="G59" t="str">
-        <v/>
+        <v>Vehicle ready for delivery</v>
+      </c>
+      <c r="F59" t="str">
+        <v>VEHICLE_READY_FOR_DELIVERY</v>
+      </c>
+      <c r="G59">
+        <v>6</v>
       </c>
       <c r="H59" t="str">
         <v/>
       </c>
       <c r="I59" t="str">
+        <v/>
+      </c>
+      <c r="J59" t="str">
+        <v/>
+      </c>
+      <c r="K59" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>THD_ACTION_TAKEN-06</v>
+        <v>THD_ACTION_TAKEN-07</v>
       </c>
       <c r="B60" t="str">
         <v>THD_ACTION_TAKEN</v>
@@ -25375,53 +25835,65 @@
         <v>Action Taken</v>
       </c>
       <c r="E60" t="str">
-        <v>Vehicle ready for delivery</v>
-      </c>
-      <c r="F60">
-        <v>6</v>
-      </c>
-      <c r="G60" t="str">
-        <v/>
+        <v>Vehicle not available; is with Customer</v>
+      </c>
+      <c r="F60" t="str">
+        <v>VEHICLE_NOT_AVAILABLE_IS_WITH_CUSTOMER</v>
+      </c>
+      <c r="G60">
+        <v>7</v>
       </c>
       <c r="H60" t="str">
         <v/>
       </c>
       <c r="I60" t="str">
+        <v/>
+      </c>
+      <c r="J60" t="str">
+        <v/>
+      </c>
+      <c r="K60" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>THD_ACTION_TAKEN-07</v>
+        <v>THD_DELAY_REASON-01</v>
       </c>
       <c r="B61" t="str">
-        <v>THD_ACTION_TAKEN</v>
+        <v>THD_DELAY_REASON</v>
       </c>
       <c r="C61" t="str">
         <v>THD</v>
       </c>
       <c r="D61" t="str">
-        <v>Action Taken</v>
+        <v>Reason for Delay</v>
       </c>
       <c r="E61" t="str">
-        <v>Vehicle not available; is with Customer</v>
-      </c>
-      <c r="F61">
-        <v>7</v>
-      </c>
-      <c r="G61" t="str">
-        <v/>
+        <v>Diagnosis and investigation</v>
+      </c>
+      <c r="F61" t="str">
+        <v>DIAGNOSIS_AND_INVESTIGATION</v>
+      </c>
+      <c r="G61">
+        <v>1</v>
       </c>
       <c r="H61" t="str">
         <v/>
       </c>
       <c r="I61" t="str">
+        <v/>
+      </c>
+      <c r="J61" t="str">
+        <v/>
+      </c>
+      <c r="K61" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>THD_DELAY_REASON-01</v>
+        <v>THD_DELAY_REASON-02</v>
       </c>
       <c r="B62" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25433,24 +25905,30 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E62" t="str">
-        <v>Diagnosis and investigation</v>
-      </c>
-      <c r="F62">
-        <v>1</v>
-      </c>
-      <c r="G62" t="str">
-        <v/>
+        <v>Work content</v>
+      </c>
+      <c r="F62" t="str">
+        <v>WORK_CONTENT</v>
+      </c>
+      <c r="G62">
+        <v>2</v>
       </c>
       <c r="H62" t="str">
         <v/>
       </c>
       <c r="I62" t="str">
+        <v/>
+      </c>
+      <c r="J62" t="str">
+        <v/>
+      </c>
+      <c r="K62" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>THD_DELAY_REASON-02</v>
+        <v>THD_DELAY_REASON-03</v>
       </c>
       <c r="B63" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25462,24 +25940,30 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E63" t="str">
-        <v>Work content</v>
-      </c>
-      <c r="F63">
-        <v>2</v>
-      </c>
-      <c r="G63" t="str">
-        <v/>
+        <v>Non-availability of spare parts</v>
+      </c>
+      <c r="F63" t="str">
+        <v>NON_AVAILABILITY_OF_SPARE_PARTS</v>
+      </c>
+      <c r="G63">
+        <v>3</v>
       </c>
       <c r="H63" t="str">
         <v/>
       </c>
       <c r="I63" t="str">
+        <v/>
+      </c>
+      <c r="J63" t="str">
+        <v/>
+      </c>
+      <c r="K63" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>THD_DELAY_REASON-03</v>
+        <v>THD_DELAY_REASON-04</v>
       </c>
       <c r="B64" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25491,24 +25975,30 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E64" t="str">
-        <v>Non-availability of spare parts</v>
-      </c>
-      <c r="F64">
-        <v>3</v>
-      </c>
-      <c r="G64" t="str">
-        <v/>
+        <v>Non-availability of vehicle</v>
+      </c>
+      <c r="F64" t="str">
+        <v>NON_AVAILABILITY_OF_VEHICLE</v>
+      </c>
+      <c r="G64">
+        <v>4</v>
       </c>
       <c r="H64" t="str">
         <v/>
       </c>
       <c r="I64" t="str">
+        <v/>
+      </c>
+      <c r="J64" t="str">
+        <v/>
+      </c>
+      <c r="K64" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>THD_DELAY_REASON-04</v>
+        <v>THD_DELAY_REASON-05</v>
       </c>
       <c r="B65" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25520,24 +26010,30 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E65" t="str">
-        <v>Non-availability of vehicle</v>
-      </c>
-      <c r="F65">
-        <v>4</v>
-      </c>
-      <c r="G65" t="str">
-        <v/>
+        <v>Dealer response</v>
+      </c>
+      <c r="F65" t="str">
+        <v>DEALER_RESPONSE</v>
+      </c>
+      <c r="G65">
+        <v>5</v>
       </c>
       <c r="H65" t="str">
         <v/>
       </c>
       <c r="I65" t="str">
+        <v/>
+      </c>
+      <c r="J65" t="str">
+        <v/>
+      </c>
+      <c r="K65" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>THD_DELAY_REASON-05</v>
+        <v>THD_DELAY_REASON-06</v>
       </c>
       <c r="B66" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25549,24 +26045,30 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E66" t="str">
-        <v>Dealer response</v>
-      </c>
-      <c r="F66">
-        <v>5</v>
-      </c>
-      <c r="G66" t="str">
-        <v/>
+        <v>Plant / ERC / vendor intervention</v>
+      </c>
+      <c r="F66" t="str">
+        <v>PLANT_ERC_VENDOR_INTERVENTION</v>
+      </c>
+      <c r="G66">
+        <v>6</v>
       </c>
       <c r="H66" t="str">
         <v/>
       </c>
       <c r="I66" t="str">
+        <v/>
+      </c>
+      <c r="J66" t="str">
+        <v/>
+      </c>
+      <c r="K66" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>THD_DELAY_REASON-06</v>
+        <v>THD_DELAY_REASON-07</v>
       </c>
       <c r="B67" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25578,24 +26080,30 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E67" t="str">
-        <v>Plant / ERC / vendor intervention</v>
-      </c>
-      <c r="F67">
-        <v>6</v>
-      </c>
-      <c r="G67" t="str">
-        <v/>
+        <v>Software / server / TDS Tool issue</v>
+      </c>
+      <c r="F67" t="str">
+        <v>SOFTWARE_SERVER_TDS_TOOL_ISSUE</v>
+      </c>
+      <c r="G67">
+        <v>7</v>
       </c>
       <c r="H67" t="str">
         <v/>
       </c>
       <c r="I67" t="str">
+        <v/>
+      </c>
+      <c r="J67" t="str">
+        <v/>
+      </c>
+      <c r="K67" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>THD_DELAY_REASON-07</v>
+        <v>THD_DELAY_REASON-08</v>
       </c>
       <c r="B68" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25607,24 +26115,30 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E68" t="str">
-        <v>Software / server / TDS Tool issue</v>
-      </c>
-      <c r="F68">
-        <v>7</v>
-      </c>
-      <c r="G68" t="str">
-        <v/>
+        <v>Solution not available</v>
+      </c>
+      <c r="F68" t="str">
+        <v>SOLUTION_NOT_AVAILABLE</v>
+      </c>
+      <c r="G68">
+        <v>8</v>
       </c>
       <c r="H68" t="str">
         <v/>
       </c>
       <c r="I68" t="str">
+        <v/>
+      </c>
+      <c r="J68" t="str">
+        <v/>
+      </c>
+      <c r="K68" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>THD_DELAY_REASON-08</v>
+        <v>THD_DELAY_REASON-09</v>
       </c>
       <c r="B69" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25636,24 +26150,30 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E69" t="str">
-        <v>Solution not available</v>
-      </c>
-      <c r="F69">
-        <v>8</v>
-      </c>
-      <c r="G69" t="str">
-        <v/>
+        <v>Pending for Commercial Decision / Customer Approval</v>
+      </c>
+      <c r="F69" t="str">
+        <v>PENDING_FOR_COMMERCIAL_DECISION_CUSTOMER</v>
+      </c>
+      <c r="G69">
+        <v>9</v>
       </c>
       <c r="H69" t="str">
         <v/>
       </c>
       <c r="I69" t="str">
+        <v/>
+      </c>
+      <c r="J69" t="str">
+        <v/>
+      </c>
+      <c r="K69" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>THD_DELAY_REASON-09</v>
+        <v>THD_DELAY_REASON-10</v>
       </c>
       <c r="B70" t="str">
         <v>THD_DELAY_REASON</v>
@@ -25665,53 +26185,65 @@
         <v>Reason for Delay</v>
       </c>
       <c r="E70" t="str">
-        <v>Pending for Commercial Decision / Customer Approval</v>
-      </c>
-      <c r="F70">
-        <v>9</v>
-      </c>
-      <c r="G70" t="str">
-        <v/>
+        <v>Dealer not responding</v>
+      </c>
+      <c r="F70" t="str">
+        <v>DEALER_NOT_RESPONDING</v>
+      </c>
+      <c r="G70">
+        <v>10</v>
       </c>
       <c r="H70" t="str">
         <v/>
       </c>
       <c r="I70" t="str">
+        <v/>
+      </c>
+      <c r="J70" t="str">
+        <v/>
+      </c>
+      <c r="K70" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>THD_DELAY_REASON-10</v>
+        <v>THD_CLOSURE_ACTION-01</v>
       </c>
       <c r="B71" t="str">
-        <v>THD_DELAY_REASON</v>
+        <v>THD_CLOSURE_ACTION</v>
       </c>
       <c r="C71" t="str">
         <v>THD</v>
       </c>
       <c r="D71" t="str">
-        <v>Reason for Delay</v>
+        <v>Closure Action</v>
       </c>
       <c r="E71" t="str">
-        <v>Dealer not responding</v>
-      </c>
-      <c r="F71">
-        <v>10</v>
-      </c>
-      <c r="G71" t="str">
-        <v/>
+        <v>Closed</v>
+      </c>
+      <c r="F71" t="str">
+        <v>CLOSED</v>
+      </c>
+      <c r="G71">
+        <v>1</v>
       </c>
       <c r="H71" t="str">
         <v/>
       </c>
       <c r="I71" t="str">
+        <v/>
+      </c>
+      <c r="J71" t="str">
+        <v/>
+      </c>
+      <c r="K71" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>THD_CLOSURE_ACTION-01</v>
+        <v>THD_CLOSURE_ACTION-02</v>
       </c>
       <c r="B72" t="str">
         <v>THD_CLOSURE_ACTION</v>
@@ -25723,24 +26255,30 @@
         <v>Closure Action</v>
       </c>
       <c r="E72" t="str">
-        <v>Closed</v>
-      </c>
-      <c r="F72">
-        <v>1</v>
-      </c>
-      <c r="G72" t="str">
-        <v/>
+        <v>Closed With Feedback</v>
+      </c>
+      <c r="F72" t="str">
+        <v>CLOSED_WITH_FEEDBACK</v>
+      </c>
+      <c r="G72">
+        <v>2</v>
       </c>
       <c r="H72" t="str">
         <v/>
       </c>
       <c r="I72" t="str">
+        <v/>
+      </c>
+      <c r="J72" t="str">
+        <v/>
+      </c>
+      <c r="K72" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>THD_CLOSURE_ACTION-02</v>
+        <v>THD_CLOSURE_ACTION-03</v>
       </c>
       <c r="B73" t="str">
         <v>THD_CLOSURE_ACTION</v>
@@ -25752,82 +26290,100 @@
         <v>Closure Action</v>
       </c>
       <c r="E73" t="str">
-        <v>Closed With Feedback</v>
-      </c>
-      <c r="F73">
-        <v>2</v>
-      </c>
-      <c r="G73" t="str">
-        <v/>
+        <v>Closed With Early Warning</v>
+      </c>
+      <c r="F73" t="str">
+        <v>CLOSED_WITH_EARLY_WARNING</v>
+      </c>
+      <c r="G73">
+        <v>3</v>
       </c>
       <c r="H73" t="str">
         <v/>
       </c>
       <c r="I73" t="str">
+        <v/>
+      </c>
+      <c r="J73" t="str">
+        <v/>
+      </c>
+      <c r="K73" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>THD_CLOSURE_ACTION-03</v>
+        <v>THD_ATTACHMENT_TYPE-01</v>
       </c>
       <c r="B74" t="str">
-        <v>THD_CLOSURE_ACTION</v>
+        <v>THD_ATTACHMENT_TYPE</v>
       </c>
       <c r="C74" t="str">
         <v>THD</v>
       </c>
       <c r="D74" t="str">
-        <v>Closure Action</v>
+        <v>Attachment Type</v>
       </c>
       <c r="E74" t="str">
-        <v>Closed With Early Warning</v>
-      </c>
-      <c r="F74">
-        <v>3</v>
-      </c>
-      <c r="G74" t="str">
-        <v/>
+        <v>DIR Report</v>
+      </c>
+      <c r="F74" t="str">
+        <v>DIR_REPORT</v>
+      </c>
+      <c r="G74">
+        <v>1</v>
       </c>
       <c r="H74" t="str">
         <v/>
       </c>
       <c r="I74" t="str">
+        <v/>
+      </c>
+      <c r="J74" t="str">
+        <v/>
+      </c>
+      <c r="K74" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>THD_ATTACHMENT_TYPE-01</v>
+        <v>CLAIM_BUDGET_PURPOSE-01</v>
       </c>
       <c r="B75" t="str">
-        <v>THD_ATTACHMENT_TYPE</v>
+        <v>CLAIM_BUDGET_PURPOSE</v>
       </c>
       <c r="C75" t="str">
-        <v>THD</v>
+        <v>CLAIM</v>
       </c>
       <c r="D75" t="str">
-        <v>Attachment Type</v>
+        <v>Allocation Purpose</v>
       </c>
       <c r="E75" t="str">
-        <v>DIR Report</v>
-      </c>
-      <c r="F75">
+        <v>Approved Yearly Budget</v>
+      </c>
+      <c r="F75" t="str">
+        <v>APPROVED_YEARLY_BUDGET</v>
+      </c>
+      <c r="G75">
         <v>1</v>
       </c>
-      <c r="G75" t="str">
-        <v/>
-      </c>
       <c r="H75" t="str">
         <v/>
       </c>
       <c r="I75" t="str">
+        <v/>
+      </c>
+      <c r="J75" t="str">
+        <v/>
+      </c>
+      <c r="K75" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>CLAIM_BUDGET_PURPOSE-01</v>
+        <v>CLAIM_BUDGET_PURPOSE-02</v>
       </c>
       <c r="B76" t="str">
         <v>CLAIM_BUDGET_PURPOSE</v>
@@ -25839,53 +26395,65 @@
         <v>Allocation Purpose</v>
       </c>
       <c r="E76" t="str">
-        <v>Approved Yearly Budget</v>
-      </c>
-      <c r="F76">
-        <v>1</v>
-      </c>
-      <c r="G76" t="str">
-        <v/>
+        <v>Special Budget</v>
+      </c>
+      <c r="F76" t="str">
+        <v>SPECIAL_BUDGET</v>
+      </c>
+      <c r="G76">
+        <v>2</v>
       </c>
       <c r="H76" t="str">
         <v/>
       </c>
       <c r="I76" t="str">
+        <v/>
+      </c>
+      <c r="J76" t="str">
+        <v/>
+      </c>
+      <c r="K76" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>CLAIM_BUDGET_PURPOSE-02</v>
+        <v>CLAIM_SPECIAL_GOODWILL-01</v>
       </c>
       <c r="B77" t="str">
-        <v>CLAIM_BUDGET_PURPOSE</v>
+        <v>CLAIM_SPECIAL_GOODWILL</v>
       </c>
       <c r="C77" t="str">
         <v>CLAIM</v>
       </c>
       <c r="D77" t="str">
-        <v>Allocation Purpose</v>
+        <v>Special Claim</v>
       </c>
       <c r="E77" t="str">
-        <v>Special Budget</v>
-      </c>
-      <c r="F77">
-        <v>2</v>
-      </c>
-      <c r="G77" t="str">
-        <v/>
+        <v>IUPR</v>
+      </c>
+      <c r="F77" t="str">
+        <v>IUPR</v>
+      </c>
+      <c r="G77">
+        <v>1</v>
       </c>
       <c r="H77" t="str">
         <v/>
       </c>
       <c r="I77" t="str">
+        <v/>
+      </c>
+      <c r="J77" t="str">
+        <v/>
+      </c>
+      <c r="K77" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>CLAIM_SPECIAL_GOODWILL-01</v>
+        <v>CLAIM_SPECIAL_GOODWILL-02</v>
       </c>
       <c r="B78" t="str">
         <v>CLAIM_SPECIAL_GOODWILL</v>
@@ -25897,53 +26465,65 @@
         <v>Special Claim</v>
       </c>
       <c r="E78" t="str">
-        <v>IUPR</v>
-      </c>
-      <c r="F78">
-        <v>1</v>
-      </c>
-      <c r="G78" t="str">
-        <v/>
+        <v>Thrive</v>
+      </c>
+      <c r="F78" t="str">
+        <v>THRIVE</v>
+      </c>
+      <c r="G78">
+        <v>2</v>
       </c>
       <c r="H78" t="str">
         <v/>
       </c>
       <c r="I78" t="str">
+        <v/>
+      </c>
+      <c r="J78" t="str">
+        <v/>
+      </c>
+      <c r="K78" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>CLAIM_SPECIAL_GOODWILL-02</v>
+        <v>CLAIM_ISSUE_DESCRIPTION-01</v>
       </c>
       <c r="B79" t="str">
-        <v>CLAIM_SPECIAL_GOODWILL</v>
+        <v>CLAIM_ISSUE_DESCRIPTION</v>
       </c>
       <c r="C79" t="str">
         <v>CLAIM</v>
       </c>
       <c r="D79" t="str">
-        <v>Special Claim</v>
+        <v>Issue Description</v>
       </c>
       <c r="E79" t="str">
-        <v>Thrive</v>
-      </c>
-      <c r="F79">
-        <v>2</v>
-      </c>
-      <c r="G79" t="str">
-        <v/>
+        <v>Thermal Incident</v>
+      </c>
+      <c r="F79" t="str">
+        <v>THERMAL_INCIDENT</v>
+      </c>
+      <c r="G79">
+        <v>1</v>
       </c>
       <c r="H79" t="str">
         <v/>
       </c>
       <c r="I79" t="str">
+        <v/>
+      </c>
+      <c r="J79" t="str">
+        <v/>
+      </c>
+      <c r="K79" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>CLAIM_ISSUE_DESCRIPTION-01</v>
+        <v>CLAIM_ISSUE_DESCRIPTION-02</v>
       </c>
       <c r="B80" t="str">
         <v>CLAIM_ISSUE_DESCRIPTION</v>
@@ -25955,53 +26535,65 @@
         <v>Issue Description</v>
       </c>
       <c r="E80" t="str">
-        <v>Thermal Incident</v>
-      </c>
-      <c r="F80">
-        <v>1</v>
-      </c>
-      <c r="G80" t="str">
-        <v/>
+        <v>Engine Failure</v>
+      </c>
+      <c r="F80" t="str">
+        <v>ENGINE_FAILURE</v>
+      </c>
+      <c r="G80">
+        <v>2</v>
       </c>
       <c r="H80" t="str">
         <v/>
       </c>
       <c r="I80" t="str">
+        <v/>
+      </c>
+      <c r="J80" t="str">
+        <v/>
+      </c>
+      <c r="K80" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>CLAIM_ISSUE_DESCRIPTION-02</v>
+        <v>CLAIM_COMPLAINT_TYPE-01</v>
       </c>
       <c r="B81" t="str">
-        <v>CLAIM_ISSUE_DESCRIPTION</v>
+        <v>CLAIM_COMPLAINT_TYPE</v>
       </c>
       <c r="C81" t="str">
         <v>CLAIM</v>
       </c>
       <c r="D81" t="str">
-        <v>Issue Description</v>
+        <v>Complaint Type</v>
       </c>
       <c r="E81" t="str">
-        <v>Engine Failure</v>
-      </c>
-      <c r="F81">
-        <v>2</v>
-      </c>
-      <c r="G81" t="str">
-        <v/>
+        <v>Transmission</v>
+      </c>
+      <c r="F81" t="str">
+        <v>TRANSMISSION</v>
+      </c>
+      <c r="G81">
+        <v>1</v>
       </c>
       <c r="H81" t="str">
         <v/>
       </c>
       <c r="I81" t="str">
+        <v/>
+      </c>
+      <c r="J81" t="str">
+        <v/>
+      </c>
+      <c r="K81" t="str">
         <v>Active</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>CLAIM_COMPLAINT_TYPE-01</v>
+        <v>CLAIM_COMPLAINT_TYPE-02</v>
       </c>
       <c r="B82" t="str">
         <v>CLAIM_COMPLAINT_TYPE</v>
@@ -26013,53 +26605,30 @@
         <v>Complaint Type</v>
       </c>
       <c r="E82" t="str">
-        <v>Transmission</v>
-      </c>
-      <c r="F82">
-        <v>1</v>
-      </c>
-      <c r="G82" t="str">
-        <v/>
+        <v>Clutch</v>
+      </c>
+      <c r="F82" t="str">
+        <v>CLUTCH</v>
+      </c>
+      <c r="G82">
+        <v>2</v>
       </c>
       <c r="H82" t="str">
         <v/>
       </c>
       <c r="I82" t="str">
-        <v>Active</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="str">
-        <v>CLAIM_COMPLAINT_TYPE-02</v>
-      </c>
-      <c r="B83" t="str">
-        <v>CLAIM_COMPLAINT_TYPE</v>
-      </c>
-      <c r="C83" t="str">
-        <v>CLAIM</v>
-      </c>
-      <c r="D83" t="str">
-        <v>Complaint Type</v>
-      </c>
-      <c r="E83" t="str">
-        <v>Clutch</v>
-      </c>
-      <c r="F83">
-        <v>2</v>
-      </c>
-      <c r="G83" t="str">
-        <v/>
-      </c>
-      <c r="H83" t="str">
-        <v/>
-      </c>
-      <c r="I83" t="str">
+        <v/>
+      </c>
+      <c r="J82" t="str">
+        <v/>
+      </c>
+      <c r="K82" t="str">
         <v>Active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I83"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K82"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rules tab: no-code business rules for every master
- 7 rule types (Required when, No duplicates, From <= To, Allowed values depend on another field,
  Must exist in another master, Number between, Format); error or warning; on/off; own message
- Rules stored with the master; checked on record save, new rows / Ctrl+B copies, the List of Values
  screen, Upload a Master and BA workbook import (rows from the file)
- Rules tab shows each rule in plain words and which saved rows do not follow it
- BA workbook: optional Rules sheet (import, export, template examples)
- Backend design: master_rule table (+ version bump trigger) with schema tests
- Pure evaluator src/utils/masterRules.ts with unit tests; E2E for the tab, uploads and LOV

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DwiSAaMRyjNA589tWt8iz
</commit_message>
<xml_diff>
--- a/docs/templates/TML_Existing_Masters_Catalogue.xlsx
+++ b/docs/templates/TML_Existing_Masters_Catalogue.xlsx
@@ -6,52 +6,53 @@
     <sheet name="README" sheetId="1" r:id="rId1"/>
     <sheet name="Masters" sheetId="2" r:id="rId2"/>
     <sheet name="Fields" sheetId="3" r:id="rId3"/>
-    <sheet name="ppl_master" sheetId="4" r:id="rId4"/>
-    <sheet name="model_checklists" sheetId="5" r:id="rId5"/>
-    <sheet name="complaint_codes" sheetId="6" r:id="rId6"/>
-    <sheet name="job_codes" sheetId="7" r:id="rId7"/>
-    <sheet name="complaint_job_linkage" sheetId="8" r:id="rId8"/>
-    <sheet name="ev_safety_protocols" sheetId="9" r:id="rId9"/>
-    <sheet name="dtc_telematics_alerts" sheetId="10" r:id="rId10"/>
-    <sheet name="bay_division_summary" sheetId="11" r:id="rId11"/>
-    <sheet name="bay_technician" sheetId="12" r:id="rId12"/>
-    <sheet name="pause_reasons" sheetId="13" r:id="rId13"/>
-    <sheet name="revisit_reasons" sheetId="14" r:id="rId14"/>
-    <sheet name="appointment_cancellation_lov" sheetId="15" r:id="rId15"/>
-    <sheet name="eqc_inspection_checklist" sheetId="16" r:id="rId16"/>
-    <sheet name="torque_verification_standards" sheetId="17" r:id="rId17"/>
-    <sheet name="eqc_gc_mandate" sheetId="18" r:id="rId18"/>
-    <sheet name="eqc_gc_steps" sheetId="19" r:id="rId19"/>
-    <sheet name="eqc_ptd_risk" sheetId="20" r:id="rId20"/>
-    <sheet name="eqc_did_thresholds" sheetId="21" r:id="rId21"/>
-    <sheet name="eqc_general_checklist" sheetId="22" r:id="rId22"/>
-    <sheet name="eqc_schedule_checklist" sheetId="23" r:id="rId23"/>
-    <sheet name="bs_inventory_sections" sheetId="24" r:id="rId24"/>
-    <sheet name="bs_inventory_checkpoints" sheetId="25" r:id="rId25"/>
-    <sheet name="bs_insurance_documents" sheetId="26" r:id="rId26"/>
-    <sheet name="bodyshop_process_stages" sheetId="27" r:id="rId27"/>
-    <sheet name="paint_booth_schedule" sheetId="28" r:id="rId28"/>
-    <sheet name="amc_pricing" sheetId="29" r:id="rId29"/>
-    <sheet name="warranty_defect_codes" sheetId="30" r:id="rId30"/>
-    <sheet name="goodwill_approval_limits" sheetId="31" r:id="rId31"/>
-    <sheet name="claim_goodwill_category" sheetId="32" r:id="rId32"/>
-    <sheet name="claim_warranty_approval_matrix" sheetId="33" r:id="rId33"/>
-    <sheet name="claim_service_guideline" sheetId="34" r:id="rId34"/>
-    <sheet name="claim_shq_users" sheetId="35" r:id="rId35"/>
-    <sheet name="spd_issuance_priority" sheetId="36" r:id="rId36"/>
-    <sheet name="parts_delay_reasons" sheetId="37" r:id="rId37"/>
-    <sheet name="thd_escalation_categories" sheetId="38" r:id="rId38"/>
-    <sheet name="tib_bulletin_codes" sheetId="39" r:id="rId39"/>
-    <sheet name="thd_auto_trigger_rules" sheetId="40" r:id="rId40"/>
-    <sheet name="thd_critical_complaints" sheetId="41" r:id="rId41"/>
-    <sheet name="thd_kms_range" sheetId="42" r:id="rId42"/>
-    <sheet name="thd_vehicle_age" sheetId="43" r:id="rId43"/>
-    <sheet name="thd_users" sheetId="44" r:id="rId44"/>
-    <sheet name="driver_transit_roster" sheetId="45" r:id="rId45"/>
-    <sheet name="lounge_reception_checklist" sheetId="46" r:id="rId46"/>
-    <sheet name="gate_security_checklist" sheetId="47" r:id="rId47"/>
-    <sheet name="gate_denial_reasons" sheetId="48" r:id="rId48"/>
-    <sheet name="common_lov" sheetId="49" r:id="rId49"/>
+    <sheet name="Rules" sheetId="4" r:id="rId4"/>
+    <sheet name="ppl_master" sheetId="5" r:id="rId5"/>
+    <sheet name="model_checklists" sheetId="6" r:id="rId6"/>
+    <sheet name="complaint_codes" sheetId="7" r:id="rId7"/>
+    <sheet name="job_codes" sheetId="8" r:id="rId8"/>
+    <sheet name="complaint_job_linkage" sheetId="9" r:id="rId9"/>
+    <sheet name="ev_safety_protocols" sheetId="10" r:id="rId10"/>
+    <sheet name="dtc_telematics_alerts" sheetId="11" r:id="rId11"/>
+    <sheet name="bay_division_summary" sheetId="12" r:id="rId12"/>
+    <sheet name="bay_technician" sheetId="13" r:id="rId13"/>
+    <sheet name="pause_reasons" sheetId="14" r:id="rId14"/>
+    <sheet name="revisit_reasons" sheetId="15" r:id="rId15"/>
+    <sheet name="appointment_cancellation_lov" sheetId="16" r:id="rId16"/>
+    <sheet name="eqc_inspection_checklist" sheetId="17" r:id="rId17"/>
+    <sheet name="torque_verification_standards" sheetId="18" r:id="rId18"/>
+    <sheet name="eqc_gc_mandate" sheetId="19" r:id="rId19"/>
+    <sheet name="eqc_gc_steps" sheetId="20" r:id="rId20"/>
+    <sheet name="eqc_ptd_risk" sheetId="21" r:id="rId21"/>
+    <sheet name="eqc_did_thresholds" sheetId="22" r:id="rId22"/>
+    <sheet name="eqc_general_checklist" sheetId="23" r:id="rId23"/>
+    <sheet name="eqc_schedule_checklist" sheetId="24" r:id="rId24"/>
+    <sheet name="bs_inventory_sections" sheetId="25" r:id="rId25"/>
+    <sheet name="bs_inventory_checkpoints" sheetId="26" r:id="rId26"/>
+    <sheet name="bs_insurance_documents" sheetId="27" r:id="rId27"/>
+    <sheet name="bodyshop_process_stages" sheetId="28" r:id="rId28"/>
+    <sheet name="paint_booth_schedule" sheetId="29" r:id="rId29"/>
+    <sheet name="amc_pricing" sheetId="30" r:id="rId30"/>
+    <sheet name="warranty_defect_codes" sheetId="31" r:id="rId31"/>
+    <sheet name="goodwill_approval_limits" sheetId="32" r:id="rId32"/>
+    <sheet name="claim_goodwill_category" sheetId="33" r:id="rId33"/>
+    <sheet name="claim_warranty_approval_matrix" sheetId="34" r:id="rId34"/>
+    <sheet name="claim_service_guideline" sheetId="35" r:id="rId35"/>
+    <sheet name="claim_shq_users" sheetId="36" r:id="rId36"/>
+    <sheet name="spd_issuance_priority" sheetId="37" r:id="rId37"/>
+    <sheet name="parts_delay_reasons" sheetId="38" r:id="rId38"/>
+    <sheet name="thd_escalation_categories" sheetId="39" r:id="rId39"/>
+    <sheet name="tib_bulletin_codes" sheetId="40" r:id="rId40"/>
+    <sheet name="thd_auto_trigger_rules" sheetId="41" r:id="rId41"/>
+    <sheet name="thd_critical_complaints" sheetId="42" r:id="rId42"/>
+    <sheet name="thd_kms_range" sheetId="43" r:id="rId43"/>
+    <sheet name="thd_vehicle_age" sheetId="44" r:id="rId44"/>
+    <sheet name="thd_users" sheetId="45" r:id="rId45"/>
+    <sheet name="driver_transit_roster" sheetId="46" r:id="rId46"/>
+    <sheet name="lounge_reception_checklist" sheetId="47" r:id="rId47"/>
+    <sheet name="gate_security_checklist" sheetId="48" r:id="rId48"/>
+    <sheet name="gate_denial_reasons" sheetId="49" r:id="rId49"/>
+    <sheet name="common_lov" sheetId="50" r:id="rId50"/>
   </sheets>
 </workbook>
 </file>
@@ -445,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -579,47 +580,117 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>RECORDS — one sheet per master, named exactly as its Master ID</v>
+        <v>SHEET "Rules" (optional) — business rules, one row per rule; checked on every save and upload, no coding</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  Row 1 = column headers: "id" plus each Field Key (the Field Label also works).</v>
+        <v xml:space="preserve">  Rule Type      required_if | unique | not_greater | allowed_if | exists_in | range | pattern</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  "id" is optional; blank ids are generated. Booleans: Y/N. Dates: YYYY-MM-DD.</v>
+        <v xml:space="preserve">    required_if  A field must be filled when another field has a certain value. e.g. Plant Name is required when Role is Plant.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v xml:space="preserve">  For an existing record, blank cells are left unchanged — you only need id + the columns you are filling in.</v>
+        <v xml:space="preserve">    unique       No two active rows may have the same values in these fields. e.g. PPL + Complaint Code must be unique.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v/>
+        <v xml:space="preserve">    not_greater  One number or date must not be greater than another. e.g. From Km must not be greater than To Km.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Adding things you missed later: add the new master/field/rows to a workbook and import it again with</v>
+        <v xml:space="preserve">    allowed_if   While a condition holds, a field may only take some values. e.g. When BU is EV, Powertrain may only be EV.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>"Update existing masters" selected. Existing fields are never changed or removed by an import;</v>
+        <v xml:space="preserve">    exists_in    The value must be an active value of a field in another master. e.g. Dealer Code must exist in the Dealer Registry.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
+        <v xml:space="preserve">    range        A number must be within a minimum and / or maximum. e.g. Warranty Months between 0 and 120.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v xml:space="preserve">    pattern      A text must follow a fixed pattern. e.g. Dealer Code: 3 capitals, a hyphen and 3 digits.</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v xml:space="preserve">  Field / When Field / Other Field   field key or label; Fields (No duplicates) and value lists are comma separated</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v xml:space="preserve">  When Values    condition values (blank = "is filled"); Allowed Values: values allowed while the condition holds</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v xml:space="preserve">  Min / Max      for "range"; Format: a pattern for "pattern"; Other Master / Other Master Field: for "exists_in"</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v xml:space="preserve">  Severity       error (row refused) or warning (saved, user warned); Message: optional own wording; Enabled: Y / N</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>RECORDS — one sheet per master, named exactly as its Master ID</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v xml:space="preserve">  Row 1 = column headers: "id" plus each Field Key (the Field Label also works).</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v xml:space="preserve">  "id" is optional; blank ids are generated. Booleans: Y/N. Dates: YYYY-MM-DD.</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v xml:space="preserve">  For an existing record, blank cells are left unchanged — you only need id + the columns you are filling in.</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Adding things you missed later: add the new master/field/rows to a workbook and import it again with</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>"Update existing masters" selected. Existing fields are never changed or removed by an import;</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
         <v>records are matched by id (existing ids are updated, new ids are added).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A48"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -633,16 +704,16 @@
         <v>id</v>
       </c>
       <c r="B1" t="str">
-        <v>dtcCode</v>
+        <v>protocolCode</v>
       </c>
       <c r="C1" t="str">
-        <v>description</v>
+        <v>safetyGate</v>
       </c>
       <c r="D1" t="str">
-        <v>alertSeverity</v>
+        <v>requiredPpe</v>
       </c>
       <c r="E1" t="str">
-        <v>autoBookAppointment</v>
+        <v>digitalMultimeterCheck</v>
       </c>
       <c r="F1" t="str">
         <v>active</v>
@@ -650,16 +721,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>DTC-01</v>
+        <v>EV-01</v>
       </c>
       <c r="B2" t="str">
-        <v>P0A80-00</v>
+        <v>EV-ISO-01</v>
       </c>
       <c r="C2" t="str">
-        <v>HV Battery Pack Cell Imbalance &gt; 150mV across modules</v>
+        <v>Manual Service Disconnect (MSD) orange plug removal &amp; lock-out tag-out (LOTO)</v>
       </c>
       <c r="D2" t="str">
-        <v>Critical Emergency (Red Lamp)</v>
+        <v>Class 0 1000V Insulated Gloves + Face Shield</v>
       </c>
       <c r="E2" t="str">
         <v>Y</v>
@@ -670,16 +741,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>DTC-02</v>
+        <v>EV-02</v>
       </c>
       <c r="B3" t="str">
-        <v>P1A02-14</v>
+        <v>EV-ISO-02</v>
       </c>
       <c r="C3" t="str">
-        <v>Electric Motor Inverter Coolant Flow Below Threshold</v>
+        <v>12V Auxiliary battery terminal disconnection to disable HV contactor control</v>
       </c>
       <c r="D3" t="str">
-        <v>Warning Advisory (Amber Lamp)</v>
+        <v>Class 0 1000V Insulated Gloves + Face Shield</v>
       </c>
       <c r="E3" t="str">
         <v>Y</v>
@@ -690,19 +761,19 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>DTC-03</v>
+        <v>EV-03</v>
       </c>
       <c r="B4" t="str">
-        <v>B1245-01</v>
+        <v>EV-ISO-03</v>
       </c>
       <c r="C4" t="str">
-        <v>Smart Key Fob Battery Low (30-day forecast)</v>
+        <v>Capacitor discharge wait cycle (10 mins) and inverter busbar residual test</v>
       </c>
       <c r="D4" t="str">
-        <v>Informational Routine (Blue)</v>
+        <v>Rubber Insulated Floor Matting 17kV</v>
       </c>
       <c r="E4" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F4" t="str">
         <v>Y</v>
@@ -717,6 +788,97 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>dtcCode</v>
+      </c>
+      <c r="C1" t="str">
+        <v>description</v>
+      </c>
+      <c r="D1" t="str">
+        <v>alertSeverity</v>
+      </c>
+      <c r="E1" t="str">
+        <v>autoBookAppointment</v>
+      </c>
+      <c r="F1" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>DTC-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>P0A80-00</v>
+      </c>
+      <c r="C2" t="str">
+        <v>HV Battery Pack Cell Imbalance &gt; 150mV across modules</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Critical Emergency (Red Lamp)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>DTC-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>P1A02-14</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Electric Motor Inverter Coolant Flow Below Threshold</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Warning Advisory (Amber Lamp)</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>DTC-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>B1245-01</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Smart Key Fob Battery Low (30-day forecast)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Informational Routine (Blue)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>N</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L3"/>
   <sheetData>
     <row r="1">
@@ -840,7 +1002,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J4"/>
   <sheetData>
@@ -979,7 +1141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G16"/>
   <sheetData>
@@ -1354,117 +1516,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>reasonCode</v>
-      </c>
-      <c r="C1" t="str">
-        <v>reasonName</v>
-      </c>
-      <c r="D1" t="str">
-        <v>department</v>
-      </c>
-      <c r="E1" t="str">
-        <v>escalateToDGM</v>
-      </c>
-      <c r="F1" t="str">
-        <v>active</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>RR-01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>REV-TECH-01</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Incomplete torque or loose fastener during initial repair</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Workmanship / Technician</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Y</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>RR-02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>REV-PART-02</v>
-      </c>
-      <c r="C3" t="str">
-        <v>New spare part premature failure within warranty</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Parts Quality / Defective Spare</v>
-      </c>
-      <c r="E3" t="str">
-        <v>N</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>RR-03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>REV-DIAG-03</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Incorrect fault diagnosis (Replaced wrong component)</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Diagnosis Error</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Y</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>RR-04</v>
-      </c>
-      <c r="B5" t="str">
-        <v>REV-CUST-04</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Operating nuance / normal NVH characteristic explained</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Customer Education</v>
-      </c>
-      <c r="E5" t="str">
-        <v>N</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1484,10 +1535,10 @@
         <v>reasonName</v>
       </c>
       <c r="D1" t="str">
-        <v>category</v>
+        <v>department</v>
       </c>
       <c r="E1" t="str">
-        <v>allowAutoReschedule</v>
+        <v>escalateToDGM</v>
       </c>
       <c r="F1" t="str">
         <v>active</v>
@@ -1495,16 +1546,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AC-01</v>
+        <v>RR-01</v>
       </c>
       <c r="B2" t="str">
-        <v>CANC-CUST-OUT</v>
+        <v>REV-TECH-01</v>
       </c>
       <c r="C2" t="str">
-        <v>Customer out of town / traveling</v>
+        <v>Incomplete torque or loose fastener during initial repair</v>
       </c>
       <c r="D2" t="str">
-        <v>Customer Request</v>
+        <v>Workmanship / Technician</v>
       </c>
       <c r="E2" t="str">
         <v>Y</v>
@@ -1515,16 +1566,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>AC-02</v>
+        <v>RR-02</v>
       </c>
       <c r="B3" t="str">
-        <v>CANC-PRICE-HIGH</v>
+        <v>REV-PART-02</v>
       </c>
       <c r="C3" t="str">
-        <v>Service estimate higher than expected (Cost objection)</v>
+        <v>New spare part premature failure within warranty</v>
       </c>
       <c r="D3" t="str">
-        <v>Customer Request</v>
+        <v>Parts Quality / Defective Spare</v>
       </c>
       <c r="E3" t="str">
         <v>N</v>
@@ -1535,16 +1586,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>AC-03</v>
+        <v>RR-03</v>
       </c>
       <c r="B4" t="str">
-        <v>CANC-BAY-CAP</v>
+        <v>REV-DIAG-03</v>
       </c>
       <c r="C4" t="str">
-        <v>Specialized EV / Alignment bay overbooked</v>
+        <v>Incorrect fault diagnosis (Replaced wrong component)</v>
       </c>
       <c r="D4" t="str">
-        <v>Dealership Capacity Constrained</v>
+        <v>Diagnosis Error</v>
       </c>
       <c r="E4" t="str">
         <v>Y</v>
@@ -1555,19 +1606,19 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>AC-04</v>
+        <v>RR-04</v>
       </c>
       <c r="B5" t="str">
-        <v>CANC-PART-BO</v>
+        <v>REV-CUST-04</v>
       </c>
       <c r="C5" t="str">
-        <v>Critical spare part on transit backorder</v>
+        <v>Operating nuance / normal NVH characteristic explained</v>
       </c>
       <c r="D5" t="str">
-        <v>Parts Shortage</v>
+        <v>Customer Education</v>
       </c>
       <c r="E5" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F5" t="str">
         <v>Y</v>
@@ -1589,16 +1640,16 @@
         <v>id</v>
       </c>
       <c r="B1" t="str">
-        <v>checkCode</v>
+        <v>reasonCode</v>
       </c>
       <c r="C1" t="str">
-        <v>stageName</v>
+        <v>reasonName</v>
       </c>
       <c r="D1" t="str">
-        <v>description</v>
+        <v>category</v>
       </c>
       <c r="E1" t="str">
-        <v>mandatoryPass</v>
+        <v>allowAutoReschedule</v>
       </c>
       <c r="F1" t="str">
         <v>active</v>
@@ -1606,16 +1657,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EQC-01</v>
+        <v>AC-01</v>
       </c>
       <c r="B2" t="str">
-        <v>EQC-OBD-01</v>
+        <v>CANC-CUST-OUT</v>
       </c>
       <c r="C2" t="str">
-        <v>Diagnostic Scan &amp; OBD-II</v>
+        <v>Customer out of town / traveling</v>
       </c>
       <c r="D2" t="str">
-        <v>Complete ECU fault code clear verification (Zero active DTCs)</v>
+        <v>Customer Request</v>
       </c>
       <c r="E2" t="str">
         <v>Y</v>
@@ -1626,19 +1677,19 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EQC-02</v>
+        <v>AC-02</v>
       </c>
       <c r="B3" t="str">
-        <v>EQC-TORQ-02</v>
+        <v>CANC-PRICE-HIGH</v>
       </c>
       <c r="C3" t="str">
-        <v>Underbody &amp; Suspension</v>
+        <v>Service estimate higher than expected (Cost objection)</v>
       </c>
       <c r="D3" t="str">
-        <v>Four-wheel lug nuts torque verification with calibrated digital wrench</v>
+        <v>Customer Request</v>
       </c>
       <c r="E3" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="F3" t="str">
         <v>Y</v>
@@ -1646,16 +1697,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EQC-03</v>
+        <v>AC-03</v>
       </c>
       <c r="B4" t="str">
-        <v>EQC-ROAD-03</v>
+        <v>CANC-BAY-CAP</v>
       </c>
       <c r="C4" t="str">
-        <v>Road Test Evaluation</v>
+        <v>Specialized EV / Alignment bay overbooked</v>
       </c>
       <c r="D4" t="str">
-        <v>5 km dynamic road test: straight line tracking and ABS bite test</v>
+        <v>Dealership Capacity Constrained</v>
       </c>
       <c r="E4" t="str">
         <v>Y</v>
@@ -1666,19 +1717,19 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>EQC-04</v>
+        <v>AC-04</v>
       </c>
       <c r="B5" t="str">
-        <v>EQC-WASH-04</v>
+        <v>CANC-PART-BO</v>
       </c>
       <c r="C5" t="str">
-        <v>Washing &amp; Interior Cleanliness</v>
+        <v>Critical spare part on transit backorder</v>
       </c>
       <c r="D5" t="str">
-        <v>Zero water seepage, spotless dashboard, paper floor mats installed</v>
+        <v>Parts Shortage</v>
       </c>
       <c r="E5" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="F5" t="str">
         <v>Y</v>
@@ -1693,6 +1744,117 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>checkCode</v>
+      </c>
+      <c r="C1" t="str">
+        <v>stageName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>description</v>
+      </c>
+      <c r="E1" t="str">
+        <v>mandatoryPass</v>
+      </c>
+      <c r="F1" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>EQC-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>EQC-OBD-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Diagnostic Scan &amp; OBD-II</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Complete ECU fault code clear verification (Zero active DTCs)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>EQC-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>EQC-TORQ-02</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Underbody &amp; Suspension</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Four-wheel lug nuts torque verification with calibrated digital wrench</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>EQC-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>EQC-ROAD-03</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Road Test Evaluation</v>
+      </c>
+      <c r="D4" t="str">
+        <v>5 km dynamic road test: straight line tracking and ABS bite test</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>EQC-04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>EQC-WASH-04</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Washing &amp; Interior Cleanliness</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Zero water seepage, spotless dashboard, paper floor mats installed</v>
+      </c>
+      <c r="E5" t="str">
+        <v>N</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
@@ -1794,7 +1956,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H7"/>
   <sheetData>
@@ -1983,277 +2145,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H10"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>ppl</v>
-      </c>
-      <c r="C1" t="str">
-        <v>complaintCode</v>
-      </c>
-      <c r="D1" t="str">
-        <v>stepNo</v>
-      </c>
-      <c r="E1" t="str">
-        <v>gcStep</v>
-      </c>
-      <c r="F1" t="str">
-        <v>gcImage1</v>
-      </c>
-      <c r="G1" t="str">
-        <v>gcImage2</v>
-      </c>
-      <c r="H1" t="str">
-        <v>active</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>GCS-01</v>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v>BRK-VIB-02</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Measure front disc run-out with dial gauge (limit 0.05 mm)</v>
-      </c>
-      <c r="F2" t="str">
-        <v>gc/brk-disc-runout.jpg</v>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>GCS-02</v>
-      </c>
-      <c r="B3" t="str">
-        <v/>
-      </c>
-      <c r="C3" t="str">
-        <v>BRK-VIB-02</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Check caliper guide pins for free movement and grease</v>
-      </c>
-      <c r="F3" t="str">
-        <v>gc/brk-guide-pins.jpg</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>GCS-03</v>
-      </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <v>BRK-VIB-02</v>
-      </c>
-      <c r="D4">
-        <v>3</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Inspect wheel balancing and tyre wear pattern</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>GCS-04</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Nexon EV</v>
-      </c>
-      <c r="C5" t="str">
-        <v>BAT-SOC-03</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Read HV battery SOC and cell voltage spread via VCI</v>
-      </c>
-      <c r="F5" t="str">
-        <v>gc/ev-vci-soc.jpg</v>
-      </c>
-      <c r="G5" t="str">
-        <v>gc/ev-cell-spread.jpg</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>GCS-05</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Nexon EV</v>
-      </c>
-      <c r="C6" t="str">
-        <v>BAT-SOC-03</v>
-      </c>
-      <c r="D6">
-        <v>2</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Check BMS DTC history and last OTA version</v>
-      </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-      <c r="H6" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>GCS-06</v>
-      </c>
-      <c r="B7" t="str">
-        <v/>
-      </c>
-      <c r="C7" t="str">
-        <v>BAT-SOC-03</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Check 12V auxiliary battery voltage and terminals</v>
-      </c>
-      <c r="F7" t="str">
-        <v>gc/12v-terminals.jpg</v>
-      </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>GCS-07</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Altroz</v>
-      </c>
-      <c r="C8" t="str">
-        <v>ENG-NOIS-01</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Cold start: listen at timing belt tensioner with stethoscope</v>
-      </c>
-      <c r="F8" t="str">
-        <v>gc/eng-tensioner.jpg</v>
-      </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
-      <c r="H8" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>GCS-08</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Altroz</v>
-      </c>
-      <c r="C9" t="str">
-        <v>ENG-NOIS-01</v>
-      </c>
-      <c r="D9">
-        <v>2</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Check engine mount bushes for cracks</v>
-      </c>
-      <c r="F9" t="str">
-        <v/>
-      </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
-      <c r="H9" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>GCS-09</v>
-      </c>
-      <c r="B10" t="str">
-        <v/>
-      </c>
-      <c r="C10" t="str">
-        <v>AC-COOL-04</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Measure vent outlet temperature at idle (target ≤ 8 °C)</v>
-      </c>
-      <c r="F10" t="str">
-        <v>gc/ac-vent-temp.jpg</v>
-      </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
-      <c r="H10" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3352,6 +3243,277 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ppl</v>
+      </c>
+      <c r="C1" t="str">
+        <v>complaintCode</v>
+      </c>
+      <c r="D1" t="str">
+        <v>stepNo</v>
+      </c>
+      <c r="E1" t="str">
+        <v>gcStep</v>
+      </c>
+      <c r="F1" t="str">
+        <v>gcImage1</v>
+      </c>
+      <c r="G1" t="str">
+        <v>gcImage2</v>
+      </c>
+      <c r="H1" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>GCS-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>BRK-VIB-02</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Measure front disc run-out with dial gauge (limit 0.05 mm)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>gc/brk-disc-runout.jpg</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>GCS-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>BRK-VIB-02</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Check caliper guide pins for free movement and grease</v>
+      </c>
+      <c r="F3" t="str">
+        <v>gc/brk-guide-pins.jpg</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>GCS-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v>BRK-VIB-02</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Inspect wheel balancing and tyre wear pattern</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>GCS-04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Nexon EV</v>
+      </c>
+      <c r="C5" t="str">
+        <v>BAT-SOC-03</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Read HV battery SOC and cell voltage spread via VCI</v>
+      </c>
+      <c r="F5" t="str">
+        <v>gc/ev-vci-soc.jpg</v>
+      </c>
+      <c r="G5" t="str">
+        <v>gc/ev-cell-spread.jpg</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>GCS-05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Nexon EV</v>
+      </c>
+      <c r="C6" t="str">
+        <v>BAT-SOC-03</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Check BMS DTC history and last OTA version</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>GCS-06</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v>BAT-SOC-03</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Check 12V auxiliary battery voltage and terminals</v>
+      </c>
+      <c r="F7" t="str">
+        <v>gc/12v-terminals.jpg</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>GCS-07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Altroz</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ENG-NOIS-01</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Cold start: listen at timing belt tensioner with stethoscope</v>
+      </c>
+      <c r="F8" t="str">
+        <v>gc/eng-tensioner.jpg</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>GCS-08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Altroz</v>
+      </c>
+      <c r="C9" t="str">
+        <v>ENG-NOIS-01</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Check engine mount bushes for cracks</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>GCS-09</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v>AC-COOL-04</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Measure vent outlet temperature at idle (target ≤ 8 °C)</v>
+      </c>
+      <c r="F10" t="str">
+        <v>gc/ac-vent-temp.jpg</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
@@ -3412,7 +3574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F7"/>
   <sheetData>
@@ -3559,321 +3721,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L8"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>bu</v>
-      </c>
-      <c r="C1" t="str">
-        <v>checklistType</v>
-      </c>
-      <c r="D1" t="str">
-        <v>checklistItem</v>
-      </c>
-      <c r="E1" t="str">
-        <v>rangeStartKm</v>
-      </c>
-      <c r="F1" t="str">
-        <v>rangeEndKm</v>
-      </c>
-      <c r="G1" t="str">
-        <v>ppl</v>
-      </c>
-      <c r="H1" t="str">
-        <v>active</v>
-      </c>
-      <c r="I1" t="str">
-        <v>notOkPhoto</v>
-      </c>
-      <c r="J1" t="str">
-        <v>notOkAudio</v>
-      </c>
-      <c r="K1" t="str">
-        <v>notOkVideo</v>
-      </c>
-      <c r="L1" t="str">
-        <v>notOkText</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>GCL-01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>PV</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Pre-Delivery Inspection</v>
-      </c>
-      <c r="D2" t="str">
-        <v>All warning lamps OFF after engine start</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v>Y</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Y</v>
-      </c>
-      <c r="J2" t="str">
-        <v>N</v>
-      </c>
-      <c r="K2" t="str">
-        <v>N</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>GCL-02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>PV</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Road Test</v>
-      </c>
-      <c r="D3" t="str">
-        <v>No pull to either side under braking</v>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Y</v>
-      </c>
-      <c r="I3" t="str">
-        <v>N</v>
-      </c>
-      <c r="J3" t="str">
-        <v>N</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Y</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>GCL-03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>PV</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Underbody</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Clutch plate wear within limit</v>
-      </c>
-      <c r="E4">
-        <v>40000</v>
-      </c>
-      <c r="F4">
-        <v>80000</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>Y</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Y</v>
-      </c>
-      <c r="J4" t="str">
-        <v>N</v>
-      </c>
-      <c r="K4" t="str">
-        <v>N</v>
-      </c>
-      <c r="L4" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>GCL-04</v>
-      </c>
-      <c r="B5" t="str">
-        <v>PV</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Road Test</v>
-      </c>
-      <c r="D5" t="str">
-        <v>DCA gear shift smooth, no judder at 1st–2nd</v>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v>Altroz</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Y</v>
-      </c>
-      <c r="I5" t="str">
-        <v>N</v>
-      </c>
-      <c r="J5" t="str">
-        <v>Y</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Y</v>
-      </c>
-      <c r="L5" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>GCL-05</v>
-      </c>
-      <c r="B6" t="str">
-        <v>EV</v>
-      </c>
-      <c r="C6" t="str">
-        <v>EV Safety</v>
-      </c>
-      <c r="D6" t="str">
-        <v>HV connector seals and orange cable insulation intact</v>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-      <c r="H6" t="str">
-        <v>Y</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Y</v>
-      </c>
-      <c r="J6" t="str">
-        <v>N</v>
-      </c>
-      <c r="K6" t="str">
-        <v>N</v>
-      </c>
-      <c r="L6" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>GCL-06</v>
-      </c>
-      <c r="B7" t="str">
-        <v>EV</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Pre-Delivery Inspection</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Regen braking levels switch correctly</v>
-      </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
-      <c r="G7" t="str">
-        <v>Nexon EV</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Y</v>
-      </c>
-      <c r="I7" t="str">
-        <v>N</v>
-      </c>
-      <c r="J7" t="str">
-        <v>N</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Y</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>GCL-07</v>
-      </c>
-      <c r="B8" t="str">
-        <v>PV</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Interior &amp; Cleanliness</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Paper floor mats and seat covers removed</v>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
-        <v/>
-      </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
-      <c r="H8" t="str">
-        <v>N</v>
-      </c>
-      <c r="I8" t="str">
-        <v>N</v>
-      </c>
-      <c r="J8" t="str">
-        <v>N</v>
-      </c>
-      <c r="K8" t="str">
-        <v>N</v>
-      </c>
-      <c r="L8" t="str">
-        <v>N</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3890,174 +3737,174 @@
         <v>bu</v>
       </c>
       <c r="C1" t="str">
-        <v>section</v>
+        <v>checklistType</v>
       </c>
       <c r="D1" t="str">
-        <v>subSection</v>
+        <v>checklistItem</v>
       </c>
       <c r="E1" t="str">
+        <v>rangeStartKm</v>
+      </c>
+      <c r="F1" t="str">
+        <v>rangeEndKm</v>
+      </c>
+      <c r="G1" t="str">
         <v>ppl</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>active</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>notOkPhoto</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>notOkAudio</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>notOkVideo</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>notOkText</v>
-      </c>
-      <c r="K1" t="str">
-        <v>rangeStartKm</v>
-      </c>
-      <c r="L1" t="str">
-        <v>rangeEndKm</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SCL-01</v>
+        <v>GCL-01</v>
       </c>
       <c r="B2" t="str">
         <v>PV</v>
       </c>
       <c r="C2" t="str">
-        <v>Engine Compartment</v>
+        <v>Pre-Delivery Inspection</v>
       </c>
       <c r="D2" t="str">
-        <v>Engine oil level and leakage</v>
+        <v>All warning lamps OFF after engine start</v>
       </c>
       <c r="E2" t="str">
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I2" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="J2" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>N</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>Y</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SCL-02</v>
+        <v>GCL-02</v>
       </c>
       <c r="B3" t="str">
         <v>PV</v>
       </c>
       <c r="C3" t="str">
-        <v>Engine Compartment</v>
+        <v>Road Test</v>
       </c>
       <c r="D3" t="str">
-        <v>Drive belt condition</v>
+        <v>No pull to either side under braking</v>
       </c>
       <c r="E3" t="str">
         <v/>
       </c>
       <c r="F3" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="G3" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I3" t="str">
         <v>N</v>
       </c>
       <c r="J3" t="str">
-        <v>Y</v>
-      </c>
-      <c r="K3">
-        <v>20000</v>
+        <v>N</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Y</v>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>Y</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SCL-03</v>
+        <v>GCL-03</v>
       </c>
       <c r="B4" t="str">
         <v>PV</v>
       </c>
       <c r="C4" t="str">
-        <v>Brakes</v>
+        <v>Underbody</v>
       </c>
       <c r="D4" t="str">
-        <v>Front pad thickness ≥ 3 mm</v>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v>Y</v>
+        <v>Clutch plate wear within limit</v>
+      </c>
+      <c r="E4">
+        <v>40000</v>
+      </c>
+      <c r="F4">
+        <v>80000</v>
       </c>
       <c r="G4" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I4" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="J4" t="str">
-        <v>Y</v>
-      </c>
-      <c r="K4">
-        <v>10000</v>
+        <v>N</v>
+      </c>
+      <c r="K4" t="str">
+        <v>N</v>
       </c>
       <c r="L4" t="str">
-        <v/>
+        <v>Y</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SCL-04</v>
+        <v>GCL-04</v>
       </c>
       <c r="B5" t="str">
         <v>PV</v>
       </c>
       <c r="C5" t="str">
-        <v>Underbody</v>
+        <v>Road Test</v>
       </c>
       <c r="D5" t="str">
-        <v>Turbo intercooler hoses</v>
+        <v>DCA gear shift smooth, no judder at 1st–2nd</v>
       </c>
       <c r="E5" t="str">
-        <v>Harrier</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="G5" t="str">
-        <v>Y</v>
+        <v>Altroz</v>
       </c>
       <c r="H5" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I5" t="str">
         <v>N</v>
@@ -4066,124 +3913,124 @@
         <v>Y</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>Y</v>
       </c>
       <c r="L5" t="str">
-        <v/>
+        <v>Y</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SCL-05</v>
+        <v>GCL-05</v>
       </c>
       <c r="B6" t="str">
         <v>EV</v>
       </c>
       <c r="C6" t="str">
-        <v>HV System</v>
+        <v>EV Safety</v>
       </c>
       <c r="D6" t="str">
-        <v>Battery pack mounting bolts torque</v>
+        <v>HV connector seals and orange cable insulation intact</v>
       </c>
       <c r="E6" t="str">
         <v/>
       </c>
       <c r="F6" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="G6" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="H6" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I6" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="J6" t="str">
-        <v>Y</v>
-      </c>
-      <c r="K6">
-        <v>15000</v>
+        <v>N</v>
+      </c>
+      <c r="K6" t="str">
+        <v>N</v>
       </c>
       <c r="L6" t="str">
-        <v/>
+        <v>Y</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SCL-06</v>
+        <v>GCL-06</v>
       </c>
       <c r="B7" t="str">
         <v>EV</v>
       </c>
       <c r="C7" t="str">
-        <v>HV System</v>
+        <v>Pre-Delivery Inspection</v>
       </c>
       <c r="D7" t="str">
-        <v>Coolant level in battery thermal loop</v>
+        <v>Regen braking levels switch correctly</v>
       </c>
       <c r="E7" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="G7" t="str">
-        <v>Y</v>
+        <v>Nexon EV</v>
       </c>
       <c r="H7" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I7" t="str">
         <v>N</v>
       </c>
       <c r="J7" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="K7" t="str">
-        <v/>
+        <v>Y</v>
       </c>
       <c r="L7" t="str">
-        <v/>
+        <v>Y</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>SCL-07</v>
+        <v>GCL-07</v>
       </c>
       <c r="B8" t="str">
         <v>PV</v>
       </c>
       <c r="C8" t="str">
-        <v>Electricals</v>
+        <v>Interior &amp; Cleanliness</v>
       </c>
       <c r="D8" t="str">
-        <v>Headlamp aim and fog lamps</v>
+        <v>Paper floor mats and seat covers removed</v>
       </c>
       <c r="E8" t="str">
         <v/>
       </c>
       <c r="F8" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="G8" t="str">
-        <v>N</v>
+        <v/>
       </c>
       <c r="H8" t="str">
         <v>N</v>
       </c>
       <c r="I8" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="J8" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="K8" t="str">
-        <v/>
-      </c>
-      <c r="L8">
-        <v>30000</v>
+        <v>N</v>
+      </c>
+      <c r="L8" t="str">
+        <v>N</v>
       </c>
     </row>
   </sheetData>
@@ -4195,6 +4042,321 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L8"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>bu</v>
+      </c>
+      <c r="C1" t="str">
+        <v>section</v>
+      </c>
+      <c r="D1" t="str">
+        <v>subSection</v>
+      </c>
+      <c r="E1" t="str">
+        <v>ppl</v>
+      </c>
+      <c r="F1" t="str">
+        <v>active</v>
+      </c>
+      <c r="G1" t="str">
+        <v>notOkPhoto</v>
+      </c>
+      <c r="H1" t="str">
+        <v>notOkAudio</v>
+      </c>
+      <c r="I1" t="str">
+        <v>notOkVideo</v>
+      </c>
+      <c r="J1" t="str">
+        <v>notOkText</v>
+      </c>
+      <c r="K1" t="str">
+        <v>rangeStartKm</v>
+      </c>
+      <c r="L1" t="str">
+        <v>rangeEndKm</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>SCL-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Engine Compartment</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Engine oil level and leakage</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H2" t="str">
+        <v>N</v>
+      </c>
+      <c r="I2" t="str">
+        <v>N</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SCL-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Engine Compartment</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Drive belt condition</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H3" t="str">
+        <v>N</v>
+      </c>
+      <c r="I3" t="str">
+        <v>N</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="K3">
+        <v>20000</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>SCL-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Brakes</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Front pad thickness ≥ 3 mm</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H4" t="str">
+        <v>N</v>
+      </c>
+      <c r="I4" t="str">
+        <v>N</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="K4">
+        <v>10000</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>SCL-04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Underbody</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Turbo intercooler hoses</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Harrier</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H5" t="str">
+        <v>N</v>
+      </c>
+      <c r="I5" t="str">
+        <v>N</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Y</v>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>SCL-05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>EV</v>
+      </c>
+      <c r="C6" t="str">
+        <v>HV System</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Battery pack mounting bolts torque</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H6" t="str">
+        <v>N</v>
+      </c>
+      <c r="I6" t="str">
+        <v>N</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Y</v>
+      </c>
+      <c r="K6">
+        <v>15000</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>SCL-06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>EV</v>
+      </c>
+      <c r="C7" t="str">
+        <v>HV System</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Coolant level in battery thermal loop</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H7" t="str">
+        <v>N</v>
+      </c>
+      <c r="I7" t="str">
+        <v>N</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Y</v>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>SCL-07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Electricals</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Headlamp aim and fog lamps</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G8" t="str">
+        <v>N</v>
+      </c>
+      <c r="H8" t="str">
+        <v>N</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Y</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Y</v>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8">
+        <v>30000</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G15"/>
   <sheetData>
     <row r="1">
@@ -4549,7 +4711,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P12"/>
   <sheetData>
@@ -5160,7 +5322,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G3"/>
   <sheetData>
@@ -5240,7 +5402,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
   <sheetData>
@@ -5351,7 +5513,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
   <sheetData>
@@ -5418,121 +5580,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>amcCode</v>
-      </c>
-      <c r="C1" t="str">
-        <v>planName</v>
-      </c>
-      <c r="D1" t="str">
-        <v>pplName</v>
-      </c>
-      <c r="E1" t="str">
-        <v>tenureYears</v>
-      </c>
-      <c r="F1" t="str">
-        <v>maxKms</v>
-      </c>
-      <c r="G1" t="str">
-        <v>priceInr</v>
-      </c>
-      <c r="H1" t="str">
-        <v>active</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>AMC-01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>TML-VC-SILVER-02</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Value Care Silver (Scheduled Lube &amp; Filters)</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Nexon</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>30000</v>
-      </c>
-      <c r="G2">
-        <v>12500</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>AMC-02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>TML-VC-GOLD-03</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Value Care Gold (Wear &amp; Tear + Scheduled)</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Harrier / Safari</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>45000</v>
-      </c>
-      <c r="G3">
-        <v>34000</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>AMC-03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>TML-EV-PROMISE-05</v>
-      </c>
-      <c r="C4" t="str">
-        <v>EV Battery &amp; Motor Health Guard AMC</v>
-      </c>
-      <c r="D4" t="str">
-        <v>EV Fleet</v>
-      </c>
-      <c r="E4">
-        <v>5</v>
-      </c>
-      <c r="F4">
-        <v>100000</v>
-      </c>
-      <c r="G4">
-        <v>28500</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -21556,6 +21603,121 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>amcCode</v>
+      </c>
+      <c r="C1" t="str">
+        <v>planName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>pplName</v>
+      </c>
+      <c r="E1" t="str">
+        <v>tenureYears</v>
+      </c>
+      <c r="F1" t="str">
+        <v>maxKms</v>
+      </c>
+      <c r="G1" t="str">
+        <v>priceInr</v>
+      </c>
+      <c r="H1" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>AMC-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>TML-VC-SILVER-02</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Value Care Silver (Scheduled Lube &amp; Filters)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Nexon</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>30000</v>
+      </c>
+      <c r="G2">
+        <v>12500</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>AMC-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>TML-VC-GOLD-03</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Value Care Gold (Wear &amp; Tear + Scheduled)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Harrier / Safari</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>45000</v>
+      </c>
+      <c r="G3">
+        <v>34000</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>AMC-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>TML-EV-PROMISE-05</v>
+      </c>
+      <c r="C4" t="str">
+        <v>EV Battery &amp; Motor Health Guard AMC</v>
+      </c>
+      <c r="D4" t="str">
+        <v>EV Fleet</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>100000</v>
+      </c>
+      <c r="G4">
+        <v>28500</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
@@ -21645,7 +21807,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
   <sheetData>
@@ -21756,7 +21918,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
   <sheetData>
@@ -21818,7 +21980,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J4"/>
   <sheetData>
@@ -21957,7 +22119,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G1"/>
   <sheetData>
@@ -21991,7 +22153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -22036,7 +22198,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
   <sheetData>
@@ -22147,7 +22309,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
   <sheetData>
@@ -22238,7 +22400,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
   <sheetData>
@@ -22349,7 +22511,68 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Master ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Rule Type</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Fields (No duplicates)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>When Field</v>
+      </c>
+      <c r="F1" t="str">
+        <v>When Values</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Other Field</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Allowed Values</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Min</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Max</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Format</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Other Master</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Other Master Field</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Severity</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Message</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
   <sheetData>
@@ -22440,192 +22663,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>bu</v>
-      </c>
-      <c r="C1" t="str">
-        <v>pplCode</v>
-      </c>
-      <c r="D1" t="str">
-        <v>pplName</v>
-      </c>
-      <c r="E1" t="str">
-        <v>plName</v>
-      </c>
-      <c r="F1" t="str">
-        <v>fuelType</v>
-      </c>
-      <c r="G1" t="str">
-        <v>active</v>
-      </c>
-      <c r="H1" t="str">
-        <v>extended_warranty_tier</v>
-      </c>
-      <c r="I1" t="str">
-        <v>telematics_ota_status</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>PPL-01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>EV</v>
-      </c>
-      <c r="C2" t="str">
-        <v>PPL-NEXON-EV</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Nexon</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Nexon EV Long Range (45 kWh)</v>
-      </c>
-      <c r="F2" t="str">
-        <v>EV</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Y</v>
-      </c>
-      <c r="H2" t="str">
-        <v>PLATINUM</v>
-      </c>
-      <c r="I2" t="str">
-        <v>OTA_ACTIVE</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>PPL-02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>PV</v>
-      </c>
-      <c r="C3" t="str">
-        <v>PPL-NEXON-ICE</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Nexon</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Nexon Fearless+ DCA Petrol</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Petrol</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Y</v>
-      </c>
-      <c r="H3" t="str">
-        <v>GOLD</v>
-      </c>
-      <c r="I3" t="str">
-        <v>OTA_ACTIVE</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>PPL-03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>PV</v>
-      </c>
-      <c r="C4" t="str">
-        <v>PPL-ALTROZ</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Altroz</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Altroz XZ i-CNG Twin Cylinder</v>
-      </c>
-      <c r="F4" t="str">
-        <v>CNG</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Y</v>
-      </c>
-      <c r="H4" t="str">
-        <v>GOLD</v>
-      </c>
-      <c r="I4" t="str">
-        <v>NON_CONNECTED</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>PPL-04</v>
-      </c>
-      <c r="B5" t="str">
-        <v>PV</v>
-      </c>
-      <c r="C5" t="str">
-        <v>PPL-HARRIER</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Harrier</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Harrier Fearless Dark 2.0L Diesel AT</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Diesel</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Y</v>
-      </c>
-      <c r="H5" t="str">
-        <v>PLATINUM</v>
-      </c>
-      <c r="I5" t="str">
-        <v>ECU_FLASH_REQ</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>PPL-05</v>
-      </c>
-      <c r="B6" t="str">
-        <v>EV</v>
-      </c>
-      <c r="C6" t="str">
-        <v>PPL-CURVV-EV</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Curvv</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Curvv EV 55 kWh Hyperion</v>
-      </c>
-      <c r="F6" t="str">
-        <v>EV</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Y</v>
-      </c>
-      <c r="H6" t="str">
-        <v>PLATINUM</v>
-      </c>
-      <c r="I6" t="str">
-        <v>OTA_ACTIVE</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L9"/>
   <sheetData>
@@ -22978,7 +23016,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H2"/>
   <sheetData>
@@ -23037,68 +23075,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>label</v>
-      </c>
-      <c r="C1" t="str">
-        <v>fromKm</v>
-      </c>
-      <c r="D1" t="str">
-        <v>toKm</v>
-      </c>
-      <c r="E1" t="str">
-        <v>status</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>KMR-01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>0 - 1,000</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>1000</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Active</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>KMR-02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>1,001 - 10,000</v>
-      </c>
-      <c r="C3">
-        <v>1001</v>
-      </c>
-      <c r="D3">
-        <v>10000</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Active</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -23115,10 +23091,10 @@
         <v>label</v>
       </c>
       <c r="C1" t="str">
-        <v>fromYears</v>
+        <v>fromKm</v>
       </c>
       <c r="D1" t="str">
-        <v>toYears</v>
+        <v>toKm</v>
       </c>
       <c r="E1" t="str">
         <v>status</v>
@@ -23126,16 +23102,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AGE-01</v>
+        <v>KMR-01</v>
       </c>
       <c r="B2" t="str">
-        <v>0 - 1</v>
+        <v>0 - 1,000</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="E2" t="str">
         <v>Active</v>
@@ -23143,16 +23119,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>AGE-02</v>
+        <v>KMR-02</v>
       </c>
       <c r="B3" t="str">
-        <v>0 - 5</v>
+        <v>1,001 - 10,000</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>1001</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>10000</v>
       </c>
       <c r="E3" t="str">
         <v>Active</v>
@@ -23167,6 +23143,68 @@
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>label</v>
+      </c>
+      <c r="C1" t="str">
+        <v>fromYears</v>
+      </c>
+      <c r="D1" t="str">
+        <v>toYears</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>AGE-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>0 - 1</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>AGE-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>0 - 5</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J6"/>
   <sheetData>
     <row r="1">
@@ -23368,7 +23406,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
   <sheetData>
@@ -23471,7 +23509,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
   <sheetData>
@@ -23562,7 +23600,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
   <sheetData>
@@ -23673,7 +23711,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
   <sheetData>
@@ -23752,7 +23790,192 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>bu</v>
+      </c>
+      <c r="C1" t="str">
+        <v>pplCode</v>
+      </c>
+      <c r="D1" t="str">
+        <v>pplName</v>
+      </c>
+      <c r="E1" t="str">
+        <v>plName</v>
+      </c>
+      <c r="F1" t="str">
+        <v>fuelType</v>
+      </c>
+      <c r="G1" t="str">
+        <v>active</v>
+      </c>
+      <c r="H1" t="str">
+        <v>extended_warranty_tier</v>
+      </c>
+      <c r="I1" t="str">
+        <v>telematics_ota_status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>PPL-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>EV</v>
+      </c>
+      <c r="C2" t="str">
+        <v>PPL-NEXON-EV</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Nexon</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Nexon EV Long Range (45 kWh)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>EV</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H2" t="str">
+        <v>PLATINUM</v>
+      </c>
+      <c r="I2" t="str">
+        <v>OTA_ACTIVE</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>PPL-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C3" t="str">
+        <v>PPL-NEXON-ICE</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Nexon</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Nexon Fearless+ DCA Petrol</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Petrol</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H3" t="str">
+        <v>GOLD</v>
+      </c>
+      <c r="I3" t="str">
+        <v>OTA_ACTIVE</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>PPL-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C4" t="str">
+        <v>PPL-ALTROZ</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Altroz</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Altroz XZ i-CNG Twin Cylinder</v>
+      </c>
+      <c r="F4" t="str">
+        <v>CNG</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H4" t="str">
+        <v>GOLD</v>
+      </c>
+      <c r="I4" t="str">
+        <v>NON_CONNECTED</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PPL-04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>PV</v>
+      </c>
+      <c r="C5" t="str">
+        <v>PPL-HARRIER</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Harrier</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Harrier Fearless Dark 2.0L Diesel AT</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Diesel</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H5" t="str">
+        <v>PLATINUM</v>
+      </c>
+      <c r="I5" t="str">
+        <v>ECU_FLASH_REQ</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>PPL-05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>EV</v>
+      </c>
+      <c r="C6" t="str">
+        <v>PPL-CURVV-EV</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Curvv</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Curvv EV 55 kWh Hyperion</v>
+      </c>
+      <c r="F6" t="str">
+        <v>EV</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Y</v>
+      </c>
+      <c r="H6" t="str">
+        <v>PLATINUM</v>
+      </c>
+      <c r="I6" t="str">
+        <v>OTA_ACTIVE</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K82"/>
   <sheetData>
@@ -26633,7 +26856,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L8"/>
   <sheetData>
@@ -26948,7 +27171,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G9"/>
   <sheetData>
@@ -27166,7 +27389,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G5"/>
   <sheetData>
@@ -27292,7 +27515,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
   <sheetData>
@@ -27393,95 +27616,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>protocolCode</v>
-      </c>
-      <c r="C1" t="str">
-        <v>safetyGate</v>
-      </c>
-      <c r="D1" t="str">
-        <v>requiredPpe</v>
-      </c>
-      <c r="E1" t="str">
-        <v>digitalMultimeterCheck</v>
-      </c>
-      <c r="F1" t="str">
-        <v>active</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>EV-01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>EV-ISO-01</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Manual Service Disconnect (MSD) orange plug removal &amp; lock-out tag-out (LOTO)</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Class 0 1000V Insulated Gloves + Face Shield</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Y</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>EV-02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>EV-ISO-02</v>
-      </c>
-      <c r="C3" t="str">
-        <v>12V Auxiliary battery terminal disconnection to disable HV contactor control</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Class 0 1000V Insulated Gloves + Face Shield</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Y</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>EV-03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>EV-ISO-03</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Capacitor discharge wait cycle (10 mins) and inverter busbar residual test</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Rubber Insulated Floor Matting 17kV</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Y</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>